<commit_message>
Complete V2.1 P5 data layer: hash duplicate history
</commit_message>
<xml_diff>
--- a/output/result.xlsx
+++ b/output/result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,16 @@
           <t>status</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>document_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -466,29 +476,35 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 | TechNews 科技新報</t>
+          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://finance.technews.tw/2026/05/01/semiconductor-inflation-trend-takes-shape-wafer-foundries-ic-design-price-hikes/</t>
+          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Fri, 01 May 2026 07:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 | TechNews 科技新報 搜尋： 登入 註冊 登出 VIP會員 Menu Skip to content 會員專區 訂閱專區 技術分析 焦點新聞評析 拓墣觀點 TechNews Smart AI 活動專區 常見問題 半導體 晶圓 晶片 IC 設計 封裝測試 處理器 GPU 記憶體 零組件 光電科技 面板 電池 3C周邊 AI 人工智慧 Claude Apple Intelligence DeepSeek Gemini Copilot ChatGPT Perplexity Grok 財經 財報 證券 房地產 Fintech 加密貨幣 金融政策 國際貿易 國際金融 支付方案 尖端科技 奈米 衛星通訊 汽車科技 航太科技 機器人 軍事科技 材料 無人機 環境科學 醫療科技 生物科技 科技生活 科技教育 能源科技 太陽能 風力 核能 電力儲存 企業永續 科技人才 系列專題 Token 戰爭：AI 推論時代的結構性大洗牌 光速革命 2026：矽光子與 CPO 領航 AI 下半場 AI 全方位解析：看懂任務分類、硬體門檻與你的產業卡位戰 能源即算力！2026 資料中心電源保衛戰 川普重返白宮一年，全球科技規則如何改變？ AI 晶片封裝技術革命 晶片戰場的隱形冠軍：先進封裝需求背後，一場決定全球 AI 命脈的設備軍備競賽 財報快訊 企業部落格 市場動態 關於我們 內容合作單位 菁英人才招募中 廣告合作 TN Smart 半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 作者 中央社 | 發布日期 2026 年 05 月 01 日 9:59 | 分類 IC 設計 , 半導體 , 晶圓 | edit Loading... Now Translating . . . 半導體通膨趨勢成形，因應成本高漲，包括晶圓代工及 IC 設計廠紛紛調漲價格，對於智慧手機等消費產品市場影響逐步顯現，智慧手機等今年出貨量恐面臨衰退壓力。 半導體廠法人說明會陸續登場，成本壓力及產品價格策略成為法人關注的焦點。晶圓代工廠除將持續投入技術開發及擴充產能，中東緊張局勢也造成能源和物流等成本升高。 晶圓代工廠 力積電 已搶先於今年1月調漲驅動IC及感測器代工價格，3月調漲功率元件代工價格， 世界 先進跟進於4月調漲代工價格， 聯電 也於4月通知客戶，將於下半年調整價格。 不僅晶圓代工價格調漲，後段封測價格也傳出漲價消息，IC設計廠紛紛決定調漲產品售價，減緩成本升高的影響， 盛群 3月已通知客戶， 聯發科 透露將藉由嚴謹的定價策略，目標將全年毛利率維持在44.5%至47.5%區間。 觀察目前整體市況依然呈現不同調的態勢，AI相關市場需求持續強勁，消費電子市場需求相對疲弱，IC設計廠不打算全面調漲產品價格。 雅特力-KY認為，近期微控制器（MCU）市場掀起一波漲價潮，並不是終端市場強勁需求所帶動，而是AI需求強勁占用產能，以及原材料漲價所致，雅特力-KY僅會適度漲價，力求毛利率持穩。 盛群認為，目前經濟情勢並未變好，需求僅穩定，因應晶圓代工與封測漲價10%至15%，盛群將僅調漲低毛利產品售價，期能讓毛利回歸合理。 繼記憶體價格飆漲後，晶圓代工和IC設計紛紛調漲價格，半導體通膨趨勢成形，使得智慧手機等消費產品市場，面臨成本升高的壓力進一步加劇。廠商除將資源集中於高階產品因應，需求也開始趨緩，聯發科預估，今年手機出貨量恐減少15%。漲價對市場需求的影響，未來是否進一步擴大，備受市場關注。 （作者：張建中；首圖來源：shutterstock） 文章看完覺得有幫助，何不給我們一個鼓勵 請我們喝杯咖啡 想請我們喝幾杯咖啡？ 每杯咖啡 65 元 x 1 x 3 x 5 x 您的咖啡贊助將是讓我們持續走下去的動力 總金額共新臺幣 0 元 《關於請喝咖啡的 Q &amp; A》 留給我們的話 取消 確認 從這裡可透過《Google 新聞》追蹤 TechNews 科技新知，時時更新 科技新報粉絲團 加入好友 訂閱免費電子報 關鍵字: 半導體通路 , 晶圓代工 , 智慧手機 , 漲價 Post navigation ← 抓無人機不靠雷達，波蘭測試「聲學感測器」揪出隱形威脅 當「好公司」成為一種人設？拆解 B 型企業的道德溢價與認證背後的機制失靈 → 我們偵測 到您有啟用 AD Block 請您暫停使用AD Block，以支持我們持續能提供更多新聞資訊與優質的閱讀環境。 新報特企 焦點動態 系列專題 AI 推論的 Token 戰爭 小龍蝦點燃「算力即營收」新紀元！Vera Rubin 引爆台美供應鏈一次看 代理 AI 重塑晶片架構！「成本才是王道」，ASIC、CPU 與記憶體牆成新戰場 從 SaaS 到 TaaS：AI 時代為何你不是付月費，而是 Token？ VIP 全預觀 本田續約廣汽十年：從技術輸出到技術汲取的合資 2.0 模式 從馬路到水路，小米申請新能源車水下推進器專利 FEV 與微軟部署車端小語言模型，確保離線語音服務與高效運用記憶體 全球儲能產業發展趨勢：政策、法規與標準化 1.6T 世代：通訊關鍵元件洗牌與台灣廠商切入路徑 本週熱門 數學界天翻地覆，代數幾何 87 年懸案「雅可比猜想」遭 Claude 證偽 焦慮、肥胖、不婚不生，研究：人類演化無法適應現代社會 全球水域含氧量迅速流失，科學家警告「水體脫氧」恐不可逆 根本沒有 100%「美國製造」路由器，廠商群起申請豁免使 FCC 禁令漸鬆 海洋蠕蟲超硬顎部揭密，科學家首度定義全新「生體金屬」 一天喝五杯咖啡也無妨？研究揭開咖啡的護肝潛力 喝咖啡能護心？美國心臟協會揭每日黃金杯數，警告避開三大飲用地雷 是太空垃圾也是天然實驗場！SpaceX 火箭殘骸 8/5 將墜入月球表面 財訊快報 宜特6月營收月增10.5% 漢唐6月營收87.43 億元 台灣大6月營收月增5.4% 科嘉-KY6月營收月減17.3% 康控-KY6月營收月減4.3% 漢磊6月營收6.20 億元 嘉晶6月營收月增3.3% 中華電6月營收月增9.3% 中環6月營收6.39 億元 台積電6月營收月增6.2% 更多&gt;&gt; 編輯精選 [ 專欄 ] 美國與中國分居最大出口市場與進口來源國下的台灣貿易結構 [ 專欄 ] 記憶體價格上漲，難成為美國政府鬆綁中國管制的理由 [ 專題 ] 小龍蝦點燃「算力即營收」新紀元！Vera Rubin 引爆台美供應鏈一次看 [ 專題 ] 代理 AI 重塑晶片架構！「成本才是王道」，ASIC、CPU 與記憶體牆成新戰場 [ 專題 ] 從 SaaS 到 TaaS：AI 時代為何你不是付月費，而是 Token？ [ 專欄 ] 「中小微企業多元振興發展計畫」落實，對提高台灣經濟韌性有重大幫助 [ 專訪 ] AI 資料傳輸量暴增！WD 談「兩大儲存挑戰」：關鍵在分層式架構 [ 專欄 ] 鼓勵「不勞而獲」降稅政策只會擴大台灣社會失衡 FB 粉絲團 我的最愛 趕快加入最愛頁面 Facebook 成為我們的小粉絲 RSS 即時更新新知 相關連結 Facebook 功能 文章 RSS 訂閱 迴響 RSS 訂閱 © 2013-2026 TechNews Inc. All rights reserved. | 關於我們 | 使用條款 | 隱私權政策 | 著作權與授權轉載 登入裝置已達上限 親愛的會員, 您的帳戶已經在其他裝置進行登入，於是系統將自動把您的帳戶登出本裝置。 若需要繼續瀏覽網站，請 重新登入 網站 若非您本人的操作，為保障您的帳戶安全，請您儘快至會員中心 修改密碼 × 請您暫停使用AD Block，以支持我們持續能提供更多新聞資訊與優質的閱讀環境。</t>
-        </is>
-      </c>
+          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>科技產業資訊室</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Success</t>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Download failed</t>
         </is>
       </c>
     </row>
@@ -500,25 +516,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-	NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development | 中央社訊息平台
-</t>
+          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 - TechNews 科技新報</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.cna.com.tw/postwrite/eng/432806</t>
+          <t>https://finance.technews.tw/2026/05/01/semiconductor-inflation-trend-takes-shape-wafer-foundries-ic-design-price-hikes/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 07:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>Fri, 01 May 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TechNews 科技新報</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development | 中央社訊息平台 財經訊息平台 知訊台 好生活 影像空間 客戶頻道 中文稿 英文稿 電信 簡介 投稿 投稿 中文稿 英文稿 電信 簡介 平台簡介 服務辦法 投稿流程 收款方式 供稿啓事 新聞稿寫作原則 其他服務 財經訊息平台 知訊台 歡迎公司行號投遞新聞訊息！詳洽業務行銷中心 人工服務時間為週一至週六9:30-12:00、14:00-18:30 如有週日發稿需求請於週六18:00前完成刊登程序。 了解更多 訊息來源：國立陽明交通大學 轉載網址 更多訊息 Matsu’s “Blue Tears” Inspire NYCU Breakthrough in Next-Generation Luminescent Materials NYCU Partners with Kneron to Advance Edge AI Education and Real-World Deployment NYCU and Changhua County Launch Smart Agriculture App to Help Farmers Monitor Crops with AI NYCU Team Wins Taiwan Title at Red Bull Basement, Heads to Silicon Valley for Global Finals NYCU Study Finds Belly Fat May Signal Hidden Heart Failure Risk—Even at Normal Weight 首頁 英文稿 NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development 發稿時間：2026/05/07 14:14:32 (中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide. The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management. The program is designed for working professionals, engineers, and learners seeking to deepen their expertise or enter the rapidly evolving semiconductor field. Courses will be delivered online in a modular, stackable format, allowing learners to tailor their studies to their professional goals and industry needs. The Semiconductor Academy is a flexible, industry-aligned portfolio of Purdue University micro-credentials developed in collaboration with faculty from NYCU in Taiwan to help upskill the global semiconductor workforce. As one of Taiwan’s leading universities in electrical engineering, computer science, photonics, AI, and semiconductor research, NYCU has long played a central role in nurturing talent for Taiwan’s semiconductor industry and the Hsinchu Science Park ecosystem. Through the Semiconductor Academy, NYCU faculty will contribute academic expertise and real-world industry perspectives drawn from Taiwan’s globally influential semiconductor ecosystem, offering international learners a unique window into the technologies and manufacturing practices shaping the future of chips and AI computing. “Semiconductor innovation requires a deep understanding of the entire technology stack,” said Mark Lundstrom, Don and Carol Scifres Distinguished Professor of Electrical and Computer Engineering at Purdue University. “By bringing together the strengths of both Purdue and NYCU, the Semiconductor Academy provides learners with a rigorous, globally informed perspective on the technologies shaping the future of the industry.” The collaboration also reflects NYCU’s broader internationalization strategy and its commitment to strengthening global partnerships in semiconductors, AI, and emerging technologies. Covering topics from chip design and semiconductor materials to packaging and supply chain management, the Semiconductor Academy’s two-hour modular courses allow learners to build industry-relevant skills at their own pace. According to Purdue, the Semiconductor Academy is part of a broader expansion of semiconductor professional education aimed at addressing rising workforce demands across the global chip industry. Each course in the academy will feature approximately 2 hours of focused learning content and be accessible through flexible online formats. The academy will also be featured on SEMI University (SEMI U), a global digital learning platform serving semiconductor professionals and organizations worldwide. Topics planned for the initial course offerings include: 。Chip Design for AI 。Packaging, Reliability and Characterization 。IC Design, EDA and Analog 。Semiconductor Materials and Devices 。Supply Chain Management and Leadership in the Semiconductor Industry Additional semiconductor professional education courses developed by Purdue are expected to launch in summer 2026, including transistor fundamentals, nanolithography, RF design, and data analysis for semiconductor applications. The launch ceremony for the Semiconductor Academy was held via livestream between Purdue and NYCU, underscoring the growing importance of international collaboration in building the future semiconductor workforce. 文章附檔 For more NYCU News, please visit the official NYCU website. 訊息平台 平台簡介 | 服務辦法 | 投稿流程 | 收款方式 | 供稿啟事 | 新聞稿寫作原則 | 其他服務 關於中央社 公司簡介 | 企業識別 | 公開資訊 | 設置條例摘要 | 隱私權聲明 | 聯絡我們 友善連結 曾虛白新聞獎基金會 | 公職人員及關係人補助交易身分關係公開及查詢平臺 中央社網站 中央通訊社 | Focus Taiwan | フォーカス台湾 | Fokus Taiwan 關注更多 iOS app 下載 | Android app 下載 | Focus Taiwan APP | 全球中央雜誌 | 文化+ | 淨零碳排 | 新聞學院 | 中央社電子報 產品與服務 產品總覽 | 客戶頻道 | 影像空間 | 訊息平台 | 財經訊息平台 | 知訊台 本平台資料均由投稿單位輸入後對外公布，資料如有錯誤、遺漏或虛偽不實，均由投稿單位負責 copyright © 2021 中央通訊社版權所有</t>
+          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 | TechNews 科技新報 搜尋： 登入 註冊 登出 VIP會員 Menu Skip to content 會員專區 訂閱專區 技術分析 焦點新聞評析 拓墣觀點 TechNews Smart AI 活動專區 常見問題 半導體 晶圓 晶片 IC 設計 封裝測試 處理器 GPU 記憶體 零組件 光電科技 面板 電池 3C周邊 AI 人工智慧 Claude Apple Intelligence DeepSeek Gemini Copilot ChatGPT Perplexity Grok 財經 財報 證券 房地產 Fintech 加密貨幣 金融政策 國際貿易 國際金融 支付方案 尖端科技 奈米 衛星通訊 汽車科技 航太科技 機器人 軍事科技 材料 無人機 環境科學 醫療科技 生物科技 科技生活 科技教育 能源科技 太陽能 風力 核能 電力儲存 企業永續 科技人才 系列專題 Token 戰爭：AI 推論時代的結構性大洗牌 光速革命 2026：矽光子與 CPO 領航 AI 下半場 AI 全方位解析：看懂任務分類、硬體門檻與你的產業卡位戰 能源即算力！2026 資料中心電源保衛戰 川普重返白宮一年，全球科技規則如何改變？ AI 晶片封裝技術革命 晶片戰場的隱形冠軍：先進封裝需求背後，一場決定全球 AI 命脈的設備軍備競賽 財報快訊 企業部落格 市場動態 關於我們 內容合作單位 菁英人才招募中 廣告合作 TN Smart 半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 作者 中央社 | 發布日期 2026 年 05 月 01 日 9:59 | 分類 IC 設計 , 半導體 , 晶圓 | edit Loading... Now Translating . . . 半導體通膨趨勢成形，因應成本高漲，包括晶圓代工及 IC 設計廠紛紛調漲價格，對於智慧手機等消費產品市場影響逐步顯現，智慧手機等今年出貨量恐面臨衰退壓力。 半導體廠法人說明會陸續登場，成本壓力及產品價格策略成為法人關注的焦點。晶圓代工廠除將持續投入技術開發及擴充產能，中東緊張局勢也造成能源和物流等成本升高。 晶圓代工廠 力積電 已搶先於今年1月調漲驅動IC及感測器代工價格，3月調漲功率元件代工價格， 世界 先進跟進於4月調漲代工價格， 聯電 也於4月通知客戶，將於下半年調整價格。 不僅晶圓代工價格調漲，後段封測價格也傳出漲價消息，IC設計廠紛紛決定調漲產品售價，減緩成本升高的影響， 盛群 3月已通知客戶， 聯發科 透露將藉由嚴謹的定價策略，目標將全年毛利率維持在44.5%至47.5%區間。 觀察目前整體市況依然呈現不同調的態勢，AI相關市場需求持續強勁，消費電子市場需求相對疲弱，IC設計廠不打算全面調漲產品價格。 雅特力-KY認為，近期微控制器（MCU）市場掀起一波漲價潮，並不是終端市場強勁需求所帶動，而是AI需求強勁占用產能，以及原材料漲價所致，雅特力-KY僅會適度漲價，力求毛利率持穩。 盛群認為，目前經濟情勢並未變好，需求僅穩定，因應晶圓代工與封測漲價10%至15%，盛群將僅調漲低毛利產品售價，期能讓毛利回歸合理。 繼記憶體價格飆漲後，晶圓代工和IC設計紛紛調漲價格，半導體通膨趨勢成形，使得智慧手機等消費產品市場，面臨成本升高的壓力進一步加劇。廠商除將資源集中於高階產品因應，需求也開始趨緩，聯發科預估，今年手機出貨量恐減少15%。漲價對市場需求的影響，未來是否進一步擴大，備受市場關注。 （作者：張建中；首圖來源：shutterstock） 文章看完覺得有幫助，何不給我們一個鼓勵 請我們喝杯咖啡 想請我們喝幾杯咖啡？ 每杯咖啡 65 元 x 1 x 3 x 5 x 您的咖啡贊助將是讓我們持續走下去的動力 總金額共新臺幣 0 元 《關於請喝咖啡的 Q &amp; A》 留給我們的話 取消 確認 從這裡可透過《Google 新聞》追蹤 TechNews 科技新知，時時更新 科技新報粉絲團 加入好友 訂閱免費電子報 關鍵字: 半導體通路 , 晶圓代工 , 智慧手機 , 漲價 Post navigation ← 抓無人機不靠雷達，波蘭測試「聲學感測器」揪出隱形威脅 當「好公司」成為一種人設？拆解 B 型企業的道德溢價與認證背後的機制失靈 → 我們偵測 到您有啟用 AD Block 請您暫停使用AD Block，以支持我們持續能提供更多新聞資訊與優質的閱讀環境。 新報特企 焦點動態 系列專題 AI 推論的 Token 戰爭 小龍蝦點燃「算力即營收」新紀元！Vera Rubin 引爆台美供應鏈一次看 代理 AI 重塑晶片架構！「成本才是王道」，ASIC、CPU 與記憶體牆成新戰場 從 SaaS 到 TaaS：AI 時代為何你不是付月費，而是 Token？ VIP 全預觀 本田續約廣汽十年：從技術輸出到技術汲取的合資 2.0 模式 從馬路到水路，小米申請新能源車水下推進器專利 FEV 與微軟部署車端小語言模型，確保離線語音服務與高效運用記憶體 全球儲能產業發展趨勢：政策、法規與標準化 1.6T 世代：通訊關鍵元件洗牌與台灣廠商切入路徑 本週熱門 數學界天翻地覆，代數幾何 87 年懸案「雅可比猜想」遭 Claude 證偽 焦慮、肥胖、不婚不生，研究：人類演化無法適應現代社會 全球水域含氧量迅速流失，科學家警告「水體脫氧」恐不可逆 根本沒有 100%「美國製造」路由器，廠商群起申請豁免使 FCC 禁令漸鬆 海洋蠕蟲超硬顎部揭密，科學家首度定義全新「生體金屬」 一天喝五杯咖啡也無妨？研究揭開咖啡的護肝潛力 喝咖啡能護心？美國心臟協會揭每日黃金杯數，警告避開三大飲用地雷 是太空垃圾也是天然實驗場！SpaceX 火箭殘骸 8/5 將墜入月球表面 財訊快報 宜特6月營收月增10.5% 漢唐6月營收87.43 億元 台灣大6月營收月增5.4% 科嘉-KY6月營收月減17.3% 康控-KY6月營收月減4.3% 漢磊6月營收6.20 億元 嘉晶6月營收月增3.3% 中華電6月營收月增9.3% 中環6月營收6.39 億元 台積電6月營收月增6.2% 更多&gt;&gt; 編輯精選 [ 專欄 ] 美國與中國分居最大出口市場與進口來源國下的台灣貿易結構 [ 專欄 ] 記憶體價格上漲，難成為美國政府鬆綁中國管制的理由 [ 專題 ] 小龍蝦點燃「算力即營收」新紀元！Vera Rubin 引爆台美供應鏈一次看 [ 專題 ] 代理 AI 重塑晶片架構！「成本才是王道」，ASIC、CPU 與記憶體牆成新戰場 [ 專題 ] 從 SaaS 到 TaaS：AI 時代為何你不是付月費，而是 Token？ [ 專欄 ] 「中小微企業多元振興發展計畫」落實，對提高台灣經濟韌性有重大幫助 [ 專訪 ] AI 資料傳輸量暴增！WD 談「兩大儲存挑戰」：關鍵在分層式架構 [ 專欄 ] 鼓勵「不勞而獲」降稅政策只會擴大台灣社會失衡 FB 粉絲團 我的最愛 趕快加入最愛頁面 Facebook 成為我們的小粉絲 RSS 即時更新新知 相關連結 Facebook 功能 文章 RSS 訂閱 迴響 RSS 訂閱 © 2013-2026 TechNews Inc. All rights reserved. | 關於我們 | 使用條款 | 隱私權政策 | 著作權與授權轉載 登入裝置已達上限 親愛的會員, 您的帳戶已經在其他裝置進行登入，於是系統將自動把您的帳戶登出本裝置。 若需要繼續瀏覽網站，請 重新登入 網站 若非您本人的操作，為保障您的帳戶安全，請您儘快至會員中心 修改密碼 × 請您暫停使用AD Block，以支持我們持續能提供更多新聞資訊與優質的閱讀環境。</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -527,6 +545,12 @@
           <t>Success</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>d970a92d732b9934c7e2d6a264f99fc947e20ef78a234dcc7de6a81e794b3864</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -536,23 +560,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 日報 - 工商時報</t>
+          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development - 中央社 CNA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.ctee.com.tw/news/20260304700096-439901</t>
+          <t>https://www.cna.com.tw/postwrite/eng/432806</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Thu, 07 May 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>中央社 CNA</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 日報 - 工商時報 前往主要內容 會員 會員中心 登出 電子報 影音特區 讀報區 首頁 即時 開闔次選單 即時首頁 要聞 證券 金融 稅法 產業 房市 國際 兩岸 科技 生活 要聞 開闔次選單 要聞首頁 政經焦點 總經趨勢 稅務法務 綜合要聞 前瞻一周 證券 開闔次選單 證券首頁 上市櫃 陸港股市 國際股市 產業焦點 期貨 權證 亮點個股 專家看盤 台股逐洞賽 重要指數 重大訊息 財經行事曆 金融 開闔次選單 金融首頁 金融話題 外匯市場 牌告匯率 金融科技 銀行動態 保險脈動 數據觀測 金融人物 理財 開闔次選單 理財首頁 理財新訊 基金 ETF 生活消費 信用卡 退休理財 統一發票 產業 開闔次選單 產業首頁 半導體 科技動態 綜合產業 生技醫療 CEO專訪 職場達人 房市 開闔次選單 房市首頁 房市焦點 區域亮點 名家攻略 居住安全 觀點評論 市場動態 國際 開闔次選單 國際首頁 全球政經 全球市場 議題觀點 國際產業 Global Scan 全球財經周報 大宗商品行情 兩岸 開闔次選單 兩岸首頁 政情動向 兩岸焦點 大陸財經 大陸產業 China Scan 陸港市場 觀點分析 言論 開闔次選單 言論首頁 社論 總經經濟 產業脈動 國際經貿 企業管理 社會觀察 奇思妙想 作者群 樂活 開闔次選單 樂活首頁 美食饗宴 旅遊休閒 生活風格 愛車天地 養生保健 時尚消費 藝文特區 書房 開闔次選單 書房首頁 書房嚴選 名人書單 好書推薦 英文進修 雜誌精選 年度好書 專題 開闔次選單 專題首頁 上市櫃6月營收 大陸經濟新局 台灣半導體風雲 上市櫃Q1營收 生技ESG革命 新世代夯話題 財經人物專訪 商情 開闔次選單 商情首頁 智慧機械 大健康 金融理財 房市建材 科技綠能 消費時尚 產學管顧 社企公益 活動 開闔次選單 活動首頁 台南機械展 台中AI展 台灣權王 服務業大評鑑 數位金融獎 ETF論壇 中華電信論壇 多元信託 期貨與選擇權 永續校園徵影 搜尋 首頁 日報 工商時報 全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO 全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO 2026.03.04 03:00 工商時報 呂雪彗 通寶半導體 安謀 智原科技 IC設計 Arm注資 通寶半導體公司董事長暨執行長沈軾榮表示，通寶半導體為全台唯一獲Arm投資的 IC 設計公司。圖／通寶半導體提供 切換文字大小 複製文章連結 分享至臉書 以Line分享 加入Google來源 參與討論 友善列印 已將目前網頁的網址複製到您的剪貼簿！ 通寶半導體設計公司簡介 台灣IC設計領域傳出國際策略投資合作捷報，通寶半導體（QBit Semiconductor）公司3日宣布，已完成B輪募資，並獲全球半導體架構大廠安謀公司（Arm Limited）參與投資，成為目前全台唯一獲得Arm投資的IC設計公司。 安謀現成為通寶十大股東之一，至於安謀持股比例及金額，4月下旬召開法說會可望對外說明，未來通寶擬計畫跨足無人機及機器人市場。 通寶半導體同時宣布，隨著募資完成營運規模擴大，計畫於今年第四季向臺灣證券交易所申請IPO上市，進一步邁向資本市場新里程碑，實際時程仍須視主管機關核准及市場狀況而定。 通寶半導體為專攻多功能列印機及事務機系統晶片的IC設計公司，其客戶主要市場遍及美國、日本、中國跟台灣。除Arm參與投資外，據悉，通寶半導體在A輪募資時，台灣政府法人機構持有通寶半導體約6％股權，包括國發基金持股2.7％，以及台肥、工研院等公股事業合計持股比例約6％，還有智原科技等半導體產業加入，整體A輪投資人持股比例約為通寶已發行股權10％。 對於這項注資，Arm全球執行副總裁暨商務長Will Abbey表示，透過與通寶的合作，可以結合先進影像處理、控制與安全能力，以支持列印及影像市場的創新。此類合作展現Arm更廣泛的策略，亦即推動具差異化的解決方案，從高效能系統延伸至更具成本效益的裝置，同時為各類產品建立成長基礎。 通寶半導體創辦人暨執行長沈軾榮也表示，很榮幸成為獲得Arm唯一投資的台灣半導體設計公司，未來通寶將持續深化在印表機影像市場的布局，並拓展至更廣泛的影像相關應用領域。 將工商時報加入Google偏好來源 相關新聞 大盤震盪 拉回擇優布局台股ETF 美股走勢分歧 晶片股台積電ADR持續承壓 《基金》6檔國內半導體ETF夯 受益人數突破43.8萬人創新高 您可能感興趣的話題 留言討論 熱門日報新聞 more 台股聞到「洗籌碼、殺斷頭」的味道！「四貸同堂」族哀嚎 指數何時反彈名師劃重點 大摩喊記憶體供需缺口未收斂 Q3漲勢未歇 南亞科、華邦電、旺宏有戲唱 台股融資大退散 短線反彈契機已到？專家估8月有望戰季線 公股逢低撿便宜 重倉大型權值電子股 買超前十強3檔ETF卡位 竟是同一家 金管會出手 嚴管四貸同堂 專題推薦 返回頁首 網站選單開關 顏色主題切換 LOADING 熱門新聞 TOP 3 more 台股崩盤不敢買？孫慶龍股災做對一件事 52萬竟變成8千萬 未來十年最看好這2檔 台股聞到「洗籌碼、殺斷頭」的味道！「四貸同堂」族哀嚎 指數何時反彈名師劃重點 期貨最新報價7／29期交所夜盤行情 本網頁已閒置超過3分鐘。請點撃框外背景，或右側關閉按鈕(X)，即可回到網頁。 關閉 關閉廣告</t>
+          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development | 中央社訊息平台 財經訊息平台 知訊台 好生活 影像空間 客戶頻道 中文稿 英文稿 電信 簡介 投稿 投稿 中文稿 英文稿 電信 簡介 平台簡介 服務辦法 投稿流程 收款方式 供稿啓事 新聞稿寫作原則 其他服務 財經訊息平台 知訊台 歡迎公司行號投遞新聞訊息！詳洽業務行銷中心 人工服務時間為週一至週六9:30-12:00、14:00-18:30 如有週日發稿需求請於週六18:00前完成刊登程序。 了解更多 訊息來源：國立陽明交通大學 轉載網址 更多訊息 Matsu’s “Blue Tears” Inspire NYCU Breakthrough in Next-Generation Luminescent Materials NYCU Partners with Kneron to Advance Edge AI Education and Real-World Deployment NYCU and Changhua County Launch Smart Agriculture App to Help Farmers Monitor Crops with AI NYCU Team Wins Taiwan Title at Red Bull Basement, Heads to Silicon Valley for Global Finals NYCU Study Finds Belly Fat May Signal Hidden Heart Failure Risk—Even at Normal Weight 首頁 英文稿 NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development 發稿時間：2026/05/07 14:14:32 (中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide. The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management. The program is designed for working professionals, engineers, and learners seeking to deepen their expertise or enter the rapidly evolving semiconductor field. Courses will be delivered online in a modular, stackable format, allowing learners to tailor their studies to their professional goals and industry needs. The Semiconductor Academy is a flexible, industry-aligned portfolio of Purdue University micro-credentials developed in collaboration with faculty from NYCU in Taiwan to help upskill the global semiconductor workforce. As one of Taiwan’s leading universities in electrical engineering, computer science, photonics, AI, and semiconductor research, NYCU has long played a central role in nurturing talent for Taiwan’s semiconductor industry and the Hsinchu Science Park ecosystem. Through the Semiconductor Academy, NYCU faculty will contribute academic expertise and real-world industry perspectives drawn from Taiwan’s globally influential semiconductor ecosystem, offering international learners a unique window into the technologies and manufacturing practices shaping the future of chips and AI computing. “Semiconductor innovation requires a deep understanding of the entire technology stack,” said Mark Lundstrom, Don and Carol Scifres Distinguished Professor of Electrical and Computer Engineering at Purdue University. “By bringing together the strengths of both Purdue and NYCU, the Semiconductor Academy provides learners with a rigorous, globally informed perspective on the technologies shaping the future of the industry.” The collaboration also reflects NYCU’s broader internationalization strategy and its commitment to strengthening global partnerships in semiconductors, AI, and emerging technologies. Covering topics from chip design and semiconductor materials to packaging and supply chain management, the Semiconductor Academy’s two-hour modular courses allow learners to build industry-relevant skills at their own pace. According to Purdue, the Semiconductor Academy is part of a broader expansion of semiconductor professional education aimed at addressing rising workforce demands across the global chip industry. Each course in the academy will feature approximately 2 hours of focused learning content and be accessible through flexible online formats. The academy will also be featured on SEMI University (SEMI U), a global digital learning platform serving semiconductor professionals and organizations worldwide. Topics planned for the initial course offerings include: 。Chip Design for AI 。Packaging, Reliability and Characterization 。IC Design, EDA and Analog 。Semiconductor Materials and Devices 。Supply Chain Management and Leadership in the Semiconductor Industry Additional semiconductor professional education courses developed by Purdue are expected to launch in summer 2026, including transistor fundamentals, nanolithography, RF design, and data analysis for semiconductor applications. The launch ceremony for the Semiconductor Academy was held via livestream between Purdue and NYCU, underscoring the growing importance of international collaboration in building the future semiconductor workforce. 文章附檔 For more NYCU News, please visit the official NYCU website. 訊息平台 平台簡介 | 服務辦法 | 投稿流程 | 收款方式 | 供稿啟事 | 新聞稿寫作原則 | 其他服務 關於中央社 公司簡介 | 企業識別 | 公開資訊 | 設置條例摘要 | 隱私權聲明 | 聯絡我們 友善連結 曾虛白新聞獎基金會 | 公職人員及關係人補助交易身分關係公開及查詢平臺 中央社網站 中央通訊社 | Focus Taiwan | フォーカス台湾 | Fokus Taiwan 關注更多 iOS app 下載 | Android app 下載 | Focus Taiwan APP | 全球中央雜誌 | 文化+ | 淨零碳排 | 新聞學院 | 中央社電子報 產品與服務 產品總覽 | 客戶頻道 | 影像空間 | 訊息平台 | 財經訊息平台 | 知訊台 本平台資料均由投稿單位輸入後對外公布，資料如有錯誤、遺漏或虛偽不實，均由投稿單位負責 copyright © 2021 中央通訊社版權所有</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -561,6 +589,12 @@
           <t>Success</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>f4068be0c01a90821295bd0289181ff02d813688f755753fa888b3135406f94d</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -570,33 +604,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå-¨çICæ°åµéçµèºç£åå°é«çæ-é - å°åå¸é»è-¦åæ¥­åæ¥­å-¬æ Taipei Computer Association</t>
+          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.tca.org.tw/news_detail.php?n=2454&amp;t=h</t>
+          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fri, 02 Jan 2026 08:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå ¨çICæ°åµéçµèºç£åå°é«çæ é - å°åå¸é»è ¦åæ¥­åæ¥­å ¬æ Taipei Computer Association æå¡ç»å ¥ å å ¥TCA äººææå ç«å §æå° èªè­ TCA æ¬æç°¡ä» å¤§äºç´ çµç¹æ¶æ§ çç£äº å°æ¥­è¯ç æå¡æå ç¢æ¥­æ¨å»£ å±è¦½æé· åé¡ç«¶è³½ æ°åµæ´»å è¨ç«è³æº åå¥½é£çµ æ°èä¸­å¿ ç±éæ°è äººç©æ¡è¨ª æå¡å°è¨ª æ´»åæ å ± å½±åæ«¥çª TCA Video Gallery TCA Photo Gallery ç«å §æå° × æå° éé ç±éæ°è ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå ¨çICæ°åµéçµèºç£åå°é«çæ é IC Taiwan Grand Challengeåéæ¼CES 2025å±ä¸­ä¹TTAåå®¶é¤¨ä»ç´¹ç«¶è³½ åå®¶ç§å­¸åæè¡å§å¡æï¼NSTCï¼æå°çåéåµæ°ç«¶è³½IC Taiwan Grand Challengeï¼ICTGCï¼å°èå ¨çæ°åµå±æ InnoVEX ä¸»è¾¦å®ä½âå°åå¸é»è ¦å ¬æï¼TCAï¼æ¼ CES 2026 æéå ±åååä¸ç³»ååéäº¤æµæ´»åã é¢å° AI ç¡¬é«ãæ©å¨äººãå é²æ¶çèé«ç§æåµæ°å¿«éæ¼é²çå ¨çæµªæ½®ï¼InnoVEX æçºä½çºåéæ°åµå°æ¥äºæ´²æå é²ç§æç¢æ¥­çééµå ¥å£ï¼æ­¤æ¬¡ ICTGC x InnoVEX åéæ¨å»£è¡åé¤äºå¨CESå±æäº®ç¸ï¼ä¹å¾å°æ¼ 1 æ 13 æ¥å¨ç½è°·èè¾¦å°å ´æ´»åï¼åå©æ´å¤ç½è°·åéæ·±å ¥äºè§£å¦ä½ä¸²é£å°ç£å¨åå°é«è AI é åçä¸çç´è³æºï¼å±ç¾å°ç£æ¨åè·¨ååä½èæ¯æä¸ä¸ä»£ééµæè¡çæ±ºå¿èæ¿è«¾ã ICTGCãInnoVEXå°æ¼CES 2026é éç»å ´ å»£éå ¨çæ°åµèè¨TTAåå®¶é¤¨ å¨ CES 2026å±ææéï¼ IC Taiwan Grand Challengeï¼ICTGCï¼å°ææå ¨çåµæ°å±æInnoVEX å°äº®ç¸æ¼CES Eureka Park ç Taiwan Tech Arenaï¼TTAï¼åå®¶é¤¨ï¼Booth Venetian Expo, Hall G â 62201ï¼ãTTA çºåç§ææ¼ CES è¨­ç«çå®æ¹å±åï¼éå®å ·åç ç©¶å°åèæªä¾æ·±ç§ææ½åçæ°åµåéï¼æ¯å¹´å¸å¼å ¨çæè³äººãåéåªé«èç§æé è¢åè¨ªã ICTGC åéä¹å°æ¼ TTA Stage æ·±å ¥ä»ç´¹èºç£å¯ä¸å ·æå®æ´è¼å°æ©å¶ãå¯æ·±å ¥å°æ¥ç¢æ¥­éä¹åå°é«æ°åµç«¶è³½ï¼åä»¥ç²çæ°åµæ¡ä¾åäº«ICTGCå¦ä½çºæ°åµæä¾å¾è¨­è¨å°éç¢çå®æ´å éæ¯æã åéè§å±è äº¦æ­¡è¿èè¨ç¾å ´è InnoVEX åICTGC åéäº¤æµï¼ç­è§£è³æºéçµèç«¶è³½çå¾µä»¶åèæ¹å¼ã ICTGC 2026 å ¨çå¾µä»¶éè·ï¼å©æ»åéæ°åµéµçµç½å³¶ ICTGC ç¾æ­£éæ¾å ¨çå ±åï¼ç³è«æªæ­¢æ¥çº 2026 å¹´ 2 æ 28 æ¥ãæ­¡è¿ä¾èª AIãæ©å¨äººãåå°é«æè¡ãææ¸¬ç³»çµ±ãæ¬¡ä¸ä»£éç®ãæ·±ç§æç­é åçæ©ææ°åµãå­¸ç åéèæè¡éç¼è æäº¤å ·æ½åçåµæ°æç¨ææ¡ã çºåå©åéæ°åµæ´å¤§å½±é¿åãå éæè¡è½å°ï¼å ¥é¸åéå°æ¼ 2026 å¹´ 6 æ 2 è³ 5 æ¥å¨å°åèè¡ç COMPUTEX TAIPEI è InnoVEX æ°åµå±ä¸­ï¼ç²å¾å è²»åå±æ©æã ä½çºäºæ´²ææ¨æ§ç B2B ç§æå±ï¼COMPUTEX çµå InnoVEX ä¸ç«å¼çåµæå°æ¥èåéåªåèå°ï¼è®åéææ©æç´æ¥éçµè£½é å¤¥ä¼´ãåå°é«ä¾æéãåµæè³æºèåéè²·ä¸»ï¼çºå¸å±åå°é«ç¢æ¥­éä¹ééµè·³æ¿ãééICTGCè¨ç«ï¼ç²çåéå¯æææå°ç£åå°é«çæ ç³»ï¼å ±åéç¼å ·åéç«¶ç­ååµæ°è§£æ±ºæ¹æ¡ã å ±åç¶²åï¼ictaiwanchallenge.org ICTGCé¦åº¦ç½è°·ç»å ´ã1 æ 13 æ¥ææInnoVEXèè¾¦è«å£æ·±åå°ç½åå°é«èAIåä½ å»¶çºCESåéæ¨å»£åè½ï¼ICTGCå°æ¼2026å¹´1æ13æ¥é¦åº¦å¨ç½è°·Palo AltoçStartup Island TAIWAN â Silicon Valley Hubèè¾¦ãBridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergiesãè«å£ãè«å£å¯èç½è°·åµæ¥­è ãæè³äººèæè¡å°å®¶ï¼æ¢è¨å¦ä½åç¨å°ç£åå°é«èAIä¾æéè³æºï¼å¼·ååµæ°è½å°èåéåä½ï¼æ´æ¼ç¾å ´çºæèè¶£åèæ·±åº¦ä»ç´¹å°ä»ç´¹ç«¶è³½å¾µä»¶å §å®¹èè©é¸éé»ï¼åæåæ¡ä¾åäº«ã åéåéäº¦å¯èç±åå æ­¤è«å£ï¼äºè§£æ´å¤æ¼å°ç£ COMPUTEX/InnoVEX å±åºè³è¨ï¼åå©å ¶ææ¡æåé²å ¥å¸å ´çè·¯å¾ä¸¦èèºç£ICTç¢æ¥­çæ ç³»å»ºç«å¯¦è³ªé£çµã æ­¤æ¬¡æ´»åè«å£é¤äºéè«åä½è¬è Laura Swan-Silicon Catalyst Ventures å ±ååå¤¥äººï¼Andy Lombard-Tesoro Venture Capital ç®¡çåå¤¥äºº, Janis Skriveris-Plug and Play Ventures æè³ç¸½ç£æ¨é«ç§æè² è²¬äººä»¥åSam Fok-femtoAI å ±ååµè¾¦äººæ¨å·è¡é·ï¼å°åå¸é»è ¦å ¬ææ¥æ«»å§¿å¯ç¸½å¹¹äºå°å¸¶é åéæä¾ç½è°·æ°åµäººå£«æ´å¤éµçµå°ç£çè³æºï¼å ±åèå£¯æé·ã ç¾å ´å°åæé²è¡å ¨çç´æ­ï¼é è¨å°å¸å¼å ¨çç¸éæ°åµäººå£«è§çãç´æ­é£çµçºï¼https://www.youtube.com/live/ruXS6oe7WNA æ´»åè³è¨ Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies 2026 å¹´ 1 æ 13 æ¥ï¼ææäºï¼ï½ä¸å 5:00ï¼PSTï¼ Startup Island TAIWAN â Silicon Valley Hub 299 California Ave STE 300, Palo Alto, CA 94306 U.S.A. åèç¶²åï¼ ãBridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergiesãè«å£ ï¼ç¼ä½æéï¼2026-01-02ï¼ ååè¡¨é  è½å¯ ã åå° ã åäº« å»¶ä¼¸é±è® InnoVEX 2026 ç«¶è³½ç»å ´ AVITICãPlug and PlayãPwCé¦æ³¢ç¹å¥çé½ç¼ï¼è¯æè³¦è½æ°åµéæåéçåè½é å®ç¢é³ä¿èè£äºé·æ¥ä»»çäºé· æè¨±å ±åè´åç¢æ¥­åéå äººç©æ¡è¨ª åç§æç¢å­¸èæå¾·çèé· : æ¨åç¢å­¸åä½è®ç ç¼ææè½å° æ°ä»»çç£äºæ¡è¨ªç³»åå ±å°(7)-æ¬æçäºæ¨å®ç¢æºé«é£å æ©è£äºé· : ãè³éè¨çµåçæãæ¯å°ç£æªä¾ç«¶ç­åªå¢ æ°ä»»çç£äºæ¡è¨ªç³»åå ±å°(6)-æ¬æçäºæ¨éææ©å¨äººé»è­å¿ çéé· : Edge AIæ¯å°ç£æ©å¨äººç¢æ¥­å½éè¶ è»çæ©æ ï¼ æ´å¤è¨æ¯ æå¡å°è¨ª TCAæå¡ä¼æ¥­å°è¨ª -å±¹å²ç§æï¼Eleosï¼ TCAæå¡ä¼æ¥­å°è¨ª -é²ä¸æè¾° TCAæå¡ä¼æ¥­å°è¨ª -å°ç£è³æç§æ ï¼ æ´å¤è¨æ¯ å»£å®£æå é±ç§æ¿ç­ è¯çµ¡æå äº¤éä½ç½® æå¡eåé Â© 2002ï¼2026 å°åå¸é»è ¦åæ¥­åæ¥­å ¬æ çæ¬ææ</t>
-        </is>
-      </c>
+          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>科技產業資訊室</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Success</t>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Download failed</t>
         </is>
       </c>
     </row>
@@ -608,23 +644,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>中國 IC 設計市佔已超車台灣！IDC 揭 2026 半導體十大趨勢：地緣政治如何重塑供應鏈？ | TechOrange 科技報橘</t>
+          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 工商時報</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://techorange.com/2025/12/05/2026-semiconductor/</t>
+          <t>https://www.ctee.com.tw/news/20260304700096-439901</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Fri, 05 Dec 2025 08:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Wed, 04 Mar 2026 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>工商時報</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>中國 IC 設計市佔已超車台灣！IDC 揭 2026 半導體十大趨勢：地緣政治如何重塑供應鏈？ | TechOrange 科技報橘 Skip to content Podcast Apple Podcast Spotify Youtube 聯絡我們 活力徵才 Podcast Apple Podcast Spotify Youtube 聯絡我們 活力徵才 Search 最新文章 AI 人工智慧 AI 機器人 智慧製造 新零售 金融科技 資安 主題特展 2026 AI 智慧大工廠論壇——台中場 2026 科技金融論壇 AI 智慧大工廠論壇－高雄場 2026 AI Agent 新工作革命論壇 AI 智慧大工廠論壇－台南場 AI 機器人產業論壇 AI Ready 數據治理論壇 AI 智慧大工廠論壇－台北場 科技風暴金融高峰論壇 AI 人才年會 TO Highlight 直擊 COMPUTEX 2026 台北國際電腦展 透視 NVIDIA GTC 2026 穩定幣新秩序：科技供應鏈與全球新金融的世紀博弈 2026 AI Impacts 趨勢觀察報告 AI 機器人全球 7 大勢力關鍵報告：透視 Global 300+ 企業系統生態 AI Agent 上工中──你準備好和 AI 當同事了嗎？ 資料治理 = AI 時代的戰略基礎設施 你用的 AI 安全嗎？揭開資安攻擊的新破口 2025 AI 工具應用報告 AI 機器人產業生態分布圖：透視台灣 100 大領軍企業 2025 企業主管 AI 技能趨勢報告 全新一週 Youtube Apple Podcast Spotify 最新文章 AI 人工智慧 AI 機器人 智慧製造 新零售 金融科技 資安 主題特展 2026 AI 智慧大工廠論壇——台中場 2026 科技金融論壇 AI 智慧大工廠論壇－高雄場 2026 AI Agent 新工作革命論壇 AI 智慧大工廠論壇－台南場 AI 機器人產業論壇 AI Ready 數據治理論壇 AI 智慧大工廠論壇－台北場 科技風暴金融高峰論壇 AI 人才年會 TO Highlight 直擊 COMPUTEX 2026 台北國際電腦展 透視 NVIDIA GTC 2026 穩定幣新秩序：科技供應鏈與全球新金融的世紀博弈 2026 AI Impacts 趨勢觀察報告 AI 機器人全球 7 大勢力關鍵報告：透視 Global 300+ 企業系統生態 AI Agent 上工中──你準備好和 AI 當同事了嗎？ 資料治理 = AI 時代的戰略基礎設施 你用的 AI 安全嗎？揭開資安攻擊的新破口 2025 AI 工具應用報告 AI 機器人產業生態分布圖：透視台灣 100 大領軍企業 2025 企業主管 AI 技能趨勢報告 全新一週 Youtube Apple Podcast Spotify 最新文章 AI 人工智慧 AI 機器人 智慧製造 新零售 金融科技 資安 主題特展 2026 AI 智慧大工廠論壇——台中場 2026 科技金融論壇 AI 智慧大工廠論壇－高雄場 2026 AI Agent 新工作革命論壇 AI 智慧大工廠論壇－台南場 AI 機器人產業論壇 AI Ready 數據治理論壇 AI 智慧大工廠論壇－台北場 科技風暴金融高峰論壇 AI 人才年會 TO Highlight 直擊 COMPUTEX 2026 台北國際電腦展 透視 NVIDIA GTC 2026 穩定幣新秩序：科技供應鏈與全球新金融的世紀博弈 2026 AI Impacts 趨勢觀察報告 AI 機器人全球 7 大勢力關鍵報告：透視 Global 300+ 企業系統生態 資料治理 = AI 時代的戰略基礎設施 AI Agent 上工中──你準備好和 AI 當同事了嗎？ 你用的 AI 安全嗎？揭開資安攻擊的新破口 2025 AI 工具應用報告 AI 機器人產業生態分布圖：透視台灣 100 大領軍企業 2025 企業主管 AI 技能趨勢報告 機器人新同事已上工！人機互動最新模式 全新一週 Youtube Apple Podcast Spotify About Us 徵才 聯絡我們 最新文章 AI 人工智慧 AI 機器人 智慧製造 新零售 金融科技 資安 主題特展 2026 AI 智慧大工廠論壇——台中場 2026 科技金融論壇 AI 智慧大工廠論壇－高雄場 2026 AI Agent 新工作革命論壇 AI 智慧大工廠論壇－台南場 AI 機器人產業論壇 AI Ready 數據治理論壇 AI 智慧大工廠論壇－台北場 科技風暴金融高峰論壇 AI 人才年會 TO Highlight 直擊 COMPUTEX 2026 台北國際電腦展 透視 NVIDIA GTC 2026 穩定幣新秩序：科技供應鏈與全球新金融的世紀博弈 2026 AI Impacts 趨勢觀察報告 AI 機器人全球 7 大勢力關鍵報告：透視 Global 300+ 企業系統生態 資料治理 = AI 時代的戰略基礎設施 AI Agent 上工中──你準備好和 AI 當同事了嗎？ 你用的 AI 安全嗎？揭開資安攻擊的新破口 2025 AI 工具應用報告 AI 機器人產業生態分布圖：透視台灣 100 大領軍企業 2025 企業主管 AI 技能趨勢報告 機器人新同事已上工！人機互動最新模式 全新一週 Youtube Apple Podcast Spotify About Us 徵才 聯絡我們 Search 半導體/零組件 中國 IC 設計市佔已超車台灣！IDC 揭 2026 半導體十大趨勢：地緣政治如何重塑供應鏈？ 李昀蔚 2025-12-05 分享本文 IDC 在今（12/5）發布 2026 年全球半導體市場十大趨勢預測，預期 2026 年全球半導體市場將維持雙位數成長動能，年成長率達 11%。 「2026 年半導體產業將從爆發性復甦邁向穩健擴張的階段，」IDC 資深研究經理曾冠瑋表示，為了滿足指數級增長的運算需求，從 IC 設計、晶圓製造到先進封裝的整體價值鏈正處於高產能利用率狀態，供應鏈上下游的緊密協作，將是確保 AI 晶片順利量產與效能突破的關鍵。 針對 2026 年全球半導體市場，IDC 歸納十大趨勢。 趨勢一：2026 年半導體市場持續強勁，年成長率將達 11% 根據 IDC 預測，2028 年全球半導體市場規模將突破 1 兆美元，2030 年更將達到 1.2 兆美元。這股由 AI 驅動的投資週期，將抵銷部分總體經濟的不確定性。 不過，市場必須留意記憶體價格上漲的趨勢，若價格持續走高，可能影響 2026 下半年的市場動能。 趨勢二：AI 晶片需求旺盛，運算應用領域年增 18% 領跑市場 曾冠瑋分析，運算類別佔據半導體市場營收比重將持續攀升，預計 2025-2026 年市佔達 60%，其中 AI 伺服器核心晶片受惠於雲端訓練與邊緣推論需求的同步爆發，預計成長 32%。 相對地，車用（Automotive）與消費性（Consumer）市場因庫存調整與成本上升，展望較為保守。 趨勢三：亞太區 IC 設計年成長 11%，中國市佔擴大至 45% 確立領先 IDC 預估 2026 年亞太區 IC 設計市場將成長 11%，不過正面臨歷史性的結構轉變，因為中國 IC 設計產值已於 2025 年正式超越台灣，確立其市場領先地位。 IDC 預測，2026 年中國市佔率將進一步擴大至 45%，台灣則調整至 40%，此消長態勢源自中國在美方制裁下，仍積極發展本土 AI 晶片、高階手機處理器，加上虛擬貨幣與安防晶片需求強勁，因此帶動當地營收呈現倍數級成長。 趨勢四：先進製程帶動晶圓代工市場成長 20%，台積電市佔將達 73% 先進製程是 2026 年晶圓代工市場成長的核心引擎，預計推動整體產值成長 20%。隨著 AI 晶片算力需求增長，台積電預期市佔率將攀升至 73%，且維持 22-26% 的高成長率。 在資本支出方面，IDC 預估台積電將達 480 億至 500 億美元，主要用於擴充 3nm、2nm 產能及為 1.6nm 做準備。台積電 2nm 預計於 2025 年底達到月產能 8 萬片。三星與 Intel 則分別在韓國華城、美國德州及俄亥俄州積極布局，試圖在 2027-2028 年的 AI 晶片商機中搶佔一席之地。 趨勢五：成熟製程市況回溫，產能利用率將穩於八成 IDC 預估 2026 年平均產能利用率將穩定維持在 80% 以上，特別是中國晶圓廠，受惠於國產替代政策以及驅動 IC、PMIC 等訂單回流，產能利用率預期將保持在 90% 以上的高檔水位。至於台灣、韓國等非中國地區，則受惠於消費性電子復甦，利用率約維持在 80%。 趨勢六：地緣政治重塑半導體供應鏈，美中日晶圓代工產能擴張加速 全球半導體產能版圖正走向區域多元化，美國、中國與日本的晶圓產能年複合成長率（CAGR）預計將分別達到 9.8%、9.8% 與 10% 的新高水位。 中國面對美方先進製程設備禁令，將資源集中擴充受限較小的成熟製程，並加速扶植國產設備供應鏈，預計最快在 2028 年其「所有製程總產能」將超越台灣居全球之冠，並於 2029 年達到 37% 的全球市佔率。 在美國方面，台積電亞利桑那州廠進展順利，一廠（P1）已開始量產，二廠（P2A）預計於 2027 年上半年正式量產 3nm 製程，P2B 則鎖定 2027 年底至 2028 年加入 2nm 行列。 日本亦展現重返半導體強國決心，除台積電熊本廠外，日本政府也全力支持新創晶片製造商 Rapidus。雖然目前日本全球產能佔比僅約 2.5% 至 3%，但在先進製程的戰略地位將顯著提升。 趨勢七：2026 OSAT 市場成長 11%，台美 AI 晶片封裝比重持續攀升 地緣政治重塑全球封測版圖，預計 2026 年 OSAT 市場將成長 11%。中國在「半導體自主化」政策推動下，要求 IC 設計與晶圓製造盡量採用在地供應鏈，推動中國 OSAT 市佔率預計將從過去的 30% 攀升至 2029 年的 33%。 然而，高階 AI 晶片封裝仍由台灣與美國大廠掌握優勢。值得注意的是，若以包含晶圓代工廠先進封裝（Foundry-based packaging）的「封裝總市值」重新排名，受惠於 CoWoS 與 InFO 的高價值貢獻，台積電預計將在 2026 年超越傳統封測廠，成為全球封裝市值的實質龍頭。 趨勢八：CoWoS 先進封裝擴張持續，產能年增 72% 仍供不應求 先進封裝產能擴張將是 2026 年的主旋律。IDC 預測，台積電 2026 年底 CoWoS 月產能將來到 11 萬片，但面對 NVIDIA、AMD 等巨頭將主力晶片全數投入 3nm 製程且 100% 採用先進封裝，市場供需依然吃緊。 這股外溢效應將為 OSAT 廠帶來機會：日月光與矽品憑藉與台積電的長期合作，預計在 2025 年中旬開始有明顯的訂單放量；Intel 雖積極推廣封裝代工，但考量玻璃基板與高階封裝的良率需達 90% 以上才具經濟效益，預期要到 2027 年才能在 CSP 自研晶片市場中見到顯著貢獻。 趨勢九：雲端軍備競賽白熱化，AI 伺服器加速器製造市場暴增 78% AI 加速器市場預計迎來爆發性成長。受惠於 Google TPU、AWS Trainium 等 CSP 自研晶片需求，IDC 預估 2026 年 ASIC 市場年增率將高達 173%。 長期而言，為了優化 TCO，CSP 與模型開發商將持續擴大 ASIC 採用比例，推動 ASIC 在 2024-2029 年的年均複合成長率達到 67%。然而，GPU 並不會因此失勢，因為隨著「影像生成」的需求大增，未來的 AI 電影與即時影像運算需要極具彈性的通用算力，這將是 GPU 長期難以被取代的護城河，也讓 GPU 的年均複合成長率仍維持 56% 的高成長動能。 趨勢十：Foundry、non-memory IDM、OSAT、Photomask 產業同步成長，Foundry2.0市 場將成長 14% 針對市場擔憂的「AI 泡沫化」，IDC 認為 2026 年發生機率偏低，主因在於 AI 基礎建設並非無限制擴張，而是受到「電力供應」與「能源網架構」的物理限制。CSP 業者無法在缺乏電力配套下無限採購晶片，這種物理上的「調節閥」反而讓半導體出貨維持在相對健康、理性的成長軌道，避免了過度庫存堆積導致的瞬間崩盤。 2026 年全球半導體產業將延續雙位數成長，從爆發期邁入「穩健擴張」階段。在這段過程中，地緣政治帶來的供應鏈重組、中國產能的強勢崛起，以及 AI 基礎建設是否會因電力瓶頸而調整節奏，將是決定產業走向的關鍵變數。 議題標籤 熱門文章 追蹤我們 追蹤 Google News TO 會員電子報 還在靠社群媒體追新聞嗎？馬上訂閱電子報，最新科技趨勢、熱門活動不漏接！ 點我訂閱 感謝訂閱！請隨時注意信箱的最新資訊 訂閱發生異常，請稍候再試或聯繫客服信箱 [email protected] 訂閱即同意 個資蒐集聲明 ，並允許 Fusionmedium 使用您的個人資料，及接收不定期活動資訊。 更多分類文章 出口暴增 75% 卻僅增千個職缺：南韓半導體高中爆紅，高薪職涯入口背後藏什麼風險？ 李昀蔚 2026-06-29 近 1,000 億電晶體塞進指甲大小晶片：IBM 0.7 奈米技術亮相，靠 3D 堆疊超車先進製程競賽 李昀蔚 2026-06-26 推論成本砍半、9 個月做出來：OpenAI 首款自研 AI 晶片 Jalapeño 想換到什麼？ 廖紹伶 2026-06-25 高通揭 AI 資料中心新藍圖：Meta 買單、Modular 補上軟體層，同步洽談 ByteDance 客製晶片 李昀蔚 2026-06-25 隱私條款 資訊安全政策 聯絡我們 活力徵才 生活報橘 公民報橘 隱私條款 資訊安全政策 聯絡我們 活力徵才 生活報橘 公民報橘 Facebook Youtube Linkedin Instagram Copyright © 2026 流線傳媒股份有限公司 All rights reserved. 為提供您更好的網站服務，本網站會使用 Cookies 及其他相關技術優化用戶體驗，繼續瀏覽本網站即表示您同意上述聲明 了解隱私權政策 同意並關閉視窗 Manage consent Close Privacy Overview This website uses cookies to improve your experience while you navigate through the website. Out of these, the cookies that are categorized as necessary are stored on your browser as they are essential for the working of basic functionalities of the website. We also use third-party cookies that help us analyze and understand how you use this website. These cookies will be stored in your browser only with your consent. You also have the option to opt-out of these cookies. But opting out of some of these cookies may affect your browsing experience. Necessary Necessary Always Enabled Necessary cookies are absolutely essential for the website to function properly. These cookies ensure basic functionalities and security features of the website, anonymously. Cookie Duration Description cookielawinfo-checkbox-analytics 11 months This cookie is set by GDPR Cookie Consent plugin. The cookie is used to store the user consent for the cookies in the category "Analytics". cookielawinfo-checkbox-functional 11 months The cookie is set by GDPR cookie consent to record the user consent for the cookies in the category "Functional". cookielawinfo-checkbox-necessary 11 months This cookie is set by GDPR Cookie Consent plugin. The cookies is used to store the user consent for the cookies in the category "Necessary". cookielawinfo-checkbox-others 11 months This cookie is set by GDPR Cookie Consent plugin. The cookie is used to store the user consent for the cookies in the category "Other. cookielawinfo-checkbox-performance 11 months This cookie is set by GDPR Cookie Consent plugin. The cookie is used to store the user consent for the cookies in the category "Performance". viewed_cookie_policy 11 months The cookie is set by the GDPR Cookie Consent plugin and is used to store whether or not user has consented to the use of cookies. It does not store any personal data. Functional Functional Functional cookies help to perform certain functionalities like sharing the content of the website on social media platforms, collect feedbacks, and other third-party features. Performance Performance Performance cookies are used to understand and analyze the key performance indexes of the website which helps in delivering a better user experience for the visitors. Analytics Analytics Analytical cookies are used to understand how visitors interact with the website. These cookies help provide information on metrics the number of visitors, bounce rate, traffic source, etc. Advertisement Advertisement Advertisement cookies are used to provide visitors with relevant ads and marketing campaigns. These cookies track visitors across websites and collect information to provide customized ads. Others Others Other uncategorized cookies are those that are being analyzed and have not been classified into a category as yet. SAVE &amp; ACCEPT</t>
+          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 日報 - 工商時報 前往主要內容 會員 會員中心 登出 電子報 影音特區 讀報區 首頁 即時 開闔次選單 即時首頁 要聞 證券 金融 稅法 產業 房市 國際 兩岸 科技 生活 要聞 開闔次選單 要聞首頁 政經焦點 總經趨勢 稅務法務 綜合要聞 前瞻一周 證券 開闔次選單 證券首頁 上市櫃 陸港股市 國際股市 產業焦點 期貨 權證 亮點個股 專家看盤 台股逐洞賽 重要指數 重大訊息 財經行事曆 金融 開闔次選單 金融首頁 金融話題 外匯市場 牌告匯率 金融科技 銀行動態 保險脈動 數據觀測 金融人物 理財 開闔次選單 理財首頁 理財新訊 基金 ETF 生活消費 信用卡 退休理財 統一發票 產業 開闔次選單 產業首頁 半導體 科技動態 綜合產業 生技醫療 CEO專訪 職場達人 房市 開闔次選單 房市首頁 房市焦點 區域亮點 名家攻略 居住安全 觀點評論 市場動態 國際 開闔次選單 國際首頁 全球政經 全球市場 議題觀點 國際產業 Global Scan 全球財經周報 大宗商品行情 兩岸 開闔次選單 兩岸首頁 政情動向 兩岸焦點 大陸財經 大陸產業 China Scan 陸港市場 觀點分析 言論 開闔次選單 言論首頁 社論 總經經濟 產業脈動 國際經貿 企業管理 社會觀察 奇思妙想 作者群 樂活 開闔次選單 樂活首頁 美食饗宴 旅遊休閒 生活風格 愛車天地 養生保健 時尚消費 藝文特區 書房 開闔次選單 書房首頁 書房嚴選 名人書單 好書推薦 英文進修 雜誌精選 年度好書 專題 開闔次選單 專題首頁 上市櫃6月營收 大陸經濟新局 台灣半導體風雲 上市櫃Q1營收 生技ESG革命 新世代夯話題 財經人物專訪 商情 開闔次選單 商情首頁 智慧機械 大健康 金融理財 房市建材 科技綠能 消費時尚 產學管顧 社企公益 活動 開闔次選單 活動首頁 台南機械展 台中AI展 台灣權王 服務業大評鑑 數位金融獎 ETF論壇 中華電信論壇 多元信託 期貨與選擇權 永續校園徵影 搜尋 首頁 日報 工商時報 全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO 全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO 2026.03.04 03:00 工商時報 呂雪彗 通寶半導體 安謀 智原科技 IC設計 Arm注資 通寶半導體公司董事長暨執行長沈軾榮表示，通寶半導體為全台唯一獲Arm投資的 IC 設計公司。圖／通寶半導體提供 切換文字大小 複製文章連結 分享至臉書 以Line分享 加入Google來源 參與討論 友善列印 已將目前網頁的網址複製到您的剪貼簿！ 通寶半導體設計公司簡介 台灣IC設計領域傳出國際策略投資合作捷報，通寶半導體（QBit Semiconductor）公司3日宣布，已完成B輪募資，並獲全球半導體架構大廠安謀公司（Arm Limited）參與投資，成為目前全台唯一獲得Arm投資的IC設計公司。 安謀現成為通寶十大股東之一，至於安謀持股比例及金額，4月下旬召開法說會可望對外說明，未來通寶擬計畫跨足無人機及機器人市場。 通寶半導體同時宣布，隨著募資完成營運規模擴大，計畫於今年第四季向臺灣證券交易所申請IPO上市，進一步邁向資本市場新里程碑，實際時程仍須視主管機關核准及市場狀況而定。 通寶半導體為專攻多功能列印機及事務機系統晶片的IC設計公司，其客戶主要市場遍及美國、日本、中國跟台灣。除Arm參與投資外，據悉，通寶半導體在A輪募資時，台灣政府法人機構持有通寶半導體約6％股權，包括國發基金持股2.7％，以及台肥、工研院等公股事業合計持股比例約6％，還有智原科技等半導體產業加入，整體A輪投資人持股比例約為通寶已發行股權10％。 對於這項注資，Arm全球執行副總裁暨商務長Will Abbey表示，透過與通寶的合作，可以結合先進影像處理、控制與安全能力，以支持列印及影像市場的創新。此類合作展現Arm更廣泛的策略，亦即推動具差異化的解決方案，從高效能系統延伸至更具成本效益的裝置，同時為各類產品建立成長基礎。 通寶半導體創辦人暨執行長沈軾榮也表示，很榮幸成為獲得Arm唯一投資的台灣半導體設計公司，未來通寶將持續深化在印表機影像市場的布局，並拓展至更廣泛的影像相關應用領域。 將工商時報加入Google偏好來源 相關新聞 大盤震盪 拉回擇優布局台股ETF 美股走勢分歧 晶片股台積電ADR持續承壓 《基金》6檔國內半導體ETF夯 受益人數突破43.8萬人創新高 您可能感興趣的話題 留言討論 熱門日報新聞 more 台股聞到「洗籌碼、殺斷頭」的味道！「四貸同堂」族哀嚎 指數何時反彈名師劃重點 大摩喊記憶體供需缺口未收斂 Q3漲勢未歇 南亞科、華邦電、旺宏有戲唱 台股融資大退散 短線反彈契機已到？專家估8月有望戰季線 公股逢低撿便宜 重倉大型權值電子股 買超前十強3檔ETF卡位 竟是同一家 金管會出手 嚴管四貸同堂 專題推薦 返回頁首 網站選單開關 顏色主題切換 LOADING 熱門新聞 TOP 3 more 台股崩盤不敢買？孫慶龍股災做對一件事 52萬竟變成8千萬 未來十年最看好這2檔 台股聞到「洗籌碼、殺斷頭」的味道！「四貸同堂」族哀嚎 指數何時反彈名師劃重點 期貨最新報價7／29期交所夜盤行情 本網頁已閒置超過3分鐘。請點撃框外背景，或右側關閉按鈕(X)，即可回到網頁。 關閉 關閉廣告</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -633,6 +673,12 @@
           <t>Success</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>07bad44a832864eb1272dcab2762e4e86697da67fbc05a5934fb00417467b485</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -642,23 +688,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>瑞昱半導體網通音訊IC領先 全球電子產品仰賴台灣實力 - 財經新聞 - PChome Online 新聞</t>
+          <t>ICTGC競賽首登矽谷 進軍CES廣邀全球IC新創鏈結臺灣半導體生態鏈 - tca.org.tw</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://news.pchome.com.tw/finance/sunmedia/20260330/index-77484256473773329003.html</t>
+          <t>https://www.tca.org.tw/news_detail.php?n=2454&amp;t=h</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mon, 30 Mar 2026 07:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>Fri, 02 Jan 2026 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tca.org.tw</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>瑞昱半導體網通音訊IC領先 全球電子產品仰賴台灣實力 - 財經新聞 - PChome Online 新聞 股市 PChome 合作媒體 說明 (登入) 首頁 專題 政治 社會 財經 科技 國際 職場 運勢 星座 健康 娛樂 體育 生活 上班族 消費 旅遊 雜誌 汽車 政府 大陸 快訊 財部：台版肥咖CRS申報 筆數金額齊增 中國實施跨國鎮壓 總統：與美強化國防合作 友達第2季每股賺0.18元 投入新技術活化資產 熊本強震見台日情誼 台人送鳳梨酥感謝日人伸援手 # 農民曆 # 今日運勢 # 金融股配息 今日天氣 空氣品質 今日運勢 樂透開獎 彰化縣 一週天氣預報(07/30 05:00發布) 臺北市 33° 32° / 34° 週五 34° / 28° 週六 35° / 28° 農曆 丙午年六月十七 宜: 祭祀,求職應聘 忌: 祈福,拜神求子 更多 獅子座 工作運 更多 【幸運色】 淡粉 【小人】 獅子 2026-07-29 樂透彩中獎號碼 更多 大樂透 8 19 24 26 32 43 47 39樂合彩 5 14 32 33 36 115年 05~06月 統一發票中獎號碼 詳情 2026-07-30 空氣品質指標 更多 臺北市士林 普通 AQI : 64 PM2.5 : 15 臺北市松山 普通 AQI : 62 PM2.5 : 14 最新 google熱搜-新竹氣爆 熱門 名人被打臉事件 HOT 人氣新聞 人氣財經新聞 女性失智症盛行率比男性高！醫揭4可能原因 更年期後應警惕 杜拜國際金融中心在 2026 年上半年取得引領業界的佳績，鞏固其於中東、非洲及南亞地區環球金融領域的領先地位 熊本7.1強震後餘震不斷 熊本市西區測得最大震度4 Google個人AI代理 Gemini Spark將在台開放 立委曝綠營幹部親屬赴陸失聯 陸委會：循機制了解 強震後熊本縣內增至14死 其中2人因地震「直接死亡」 熊本7.1強震後餘震不斷 又再兩起有感地震 Lockton 正式成立全球數據中心及數字基礎設施業務部門 曾獲2014世足金手套 德國門神諾伊爾可能下季退休 老針車翻轉新活力！彰化榮家8旬嬤用古董裁縫機實踐自主復能 監院指兩岸教育交流失衡 陸委會：強化中共統戰識讀 紅十字會設熊本地震捐款專區 首波撥1千萬日圓馳援 FIFA擬成立子公司賣股權 歐足總砲轟、亞足聯表失望 2026臺南夏日音樂節-將軍吼 本周六日強勢來襲！ 周邊交通與各項管制措施懶人包全攻略 央廣推新住民共創平台 用AI突破語言隔閡 《鐵拳教育》金武烈首爾見面會秒殺！海外首站9月獻台灣 高國輝肯定悍將上半季撐到最後 打擊找跳出的契機 韓職王彥程連兩場優質先發 奪個人本季第9勝 王順和重感冒大巨蛋開轟 打擊更有力添信心 熊本強震停電斷水又遇酷暑 政府發首批移動式冷氣 【台股盤後】台股多空激戰震盪逾1700點 終場下跌105點失守4萬點 川寶布局TGV 完成成孔後電鍍金屬化設備試機 台股多空激戰震盪逾1700點 終場下跌105點失守4萬點 AI基建掀物流商機 中菲行：高價值空運快速成長 熊本強震衝擊九州製造業 豐田、Sony等持續停工檢查 台北市新案房價抗跌 信義區每坪226萬實登居冠 越南土地革命篇－與鹹水共生 稻蝦輪作逆境求生 AI基建掀物流商機 中菲行：高價值空運快速成長 8月台股期指跌58點 三大法人賣超台股508.73億元 星巴克同店銷售額連4季成長 上調全年財務展望 越南現象篇－九龍江星光不浪漫 海水倒灌成農民夢魘 8月電子期跌 金融期漲 日月光投控第2季獲利同期新高 先進封測營收優預期 夏慕尼哈根達斯聯名推「情人節套餐」 台北市新案房價抗跌 信義區每坪226萬實登居冠 台股4萬點失守！台積電撐盤收2205元 台股震盪 童子賢：別盯著綠紅聖誕樹、AI長期不泡沫 王品集團夏慕尼加速展店 目標明年底達21店 台股震盪 童子賢：別盯著綠紅聖誕樹、AI長期不泡沫 NEW 最新 新聞 最新影音新聞 友達第2季每股賺0.18元 投入新技術活化資產 財部：台版肥咖CRS申報 筆數金額齊增 苦茶油驗出苯駢芘超標！永豐餘生技退費方式 韓國7月出口額估年增59% 晶片熱潮支撐動能不減 央行理事：若台股降溫 憂資金由股轉房推升房價 央行理事：若台股降溫 憂資金由股轉房推升房價 外資賣超483億元 調節元大台灣50逾6萬張居冠 韓國7月出口額估年增59% 晶片熱潮支撐動能不減 阿里山林鐵x台啤5年 開發第五種品牌雙聯名釀造出二萬天晴新品 日月光：目前封測製程重心在台灣 待時機擴展美國 經濟部、勞動部共審 強迫勞動貨品機制公布 台達電今年資本支出上看700億元 擬新增海外營運據點 台達電上半年獲利創高 鄭平：下半年成長沒有太大問題 台灣大有望併凱擘？林之晨：勢必會評估 台達電資本支出上看700億 擬新增海外營運據點 停進巴紐天然氣 經長：現貨可調整、長約仍需履約 市調：明年DRAM供給續吃緊 NAND Flash轉寬鬆 日月光投控資本支出估105億美元 先進封測營收明年再翻倍 日月光資本支出估105億美元 先進封測營收明年再翻倍 台積電洩密案 2前工程師各判10年、6年定讞 苦茶油驗出苯駢芘超標！永豐餘生技退費方式 韓國7月出口額估年增59% 晶片熱潮支撐動能不減 永慶房屋首年72萬收入保障 新鮮人藍婉云零經驗拚出百萬年薪 央行理事：若台股降溫 憂資金由股轉房推升房價 蔣萬安為何提倒閣？他曝3關鍵：當然衝第一 2026咖啡產業職涯論壇8月6日中山堂登場！跨域結合AI與品牌經營 即日起免費報名 豪雨災害農損現金救助 農業處呼籲屏東縣各鄉鎮市公所加速完成初勘 兒少柳營體驗多元學習！以射擊培養專注及自律 中國實施跨國鎮壓 總統：與美強化國防合作 屏東縣衛生局守護青少年健康！全面禁電子煙、未滿20歲嚴禁購菸 夏莉絲案涉案行為人終身不得擔任教保人員、廢照重罰235萬！北市教育局籲停止政治操作：勿抹煞基層努力 阿里山林鐵x台啤5年 開發第五種品牌雙聯名釀造出二萬天晴新品 吳玉琴返鄉參選鹿草鄉長 盼打造健康家園 影／不讓貧窮限制夢想 彰化家扶獎助學金點亮孩子未來 台積電核心關鍵技術內鬼案 主嫌陳力銘判刑10年定讞 梁詠琪現場驚喜「催生」Lulu 許曦文曝媽媽小S吃醋內幕 血跡一路通往森林！7公尺巨蟒肚子鼓鼓 剖開全村嚇壞 融資租賃業納金保法 163件申訴2大類為主 國海院首度發布MDImageNet高品質海廢資料集 鄭淑分體恤高齢長輩 太保市公所x監理所、衛生所推動高齡換照一站式服務 新聞 財經 2026-03-30 11:49:24 新聞來源 : 商傳媒 回應 瑞昱半導體網通音訊IC領先 全球電子產品仰賴台灣實力 圖／本報資料庫 商傳媒 ｜何映辰／台北報導 台灣積體電路設計大廠瑞昱半導體（Realtek Semiconductor Corp）在全球網通與音訊積體電路（IC）市場扮演關鍵角色，其技術實力驅動著個人電腦與消費性電子產品的發展，並連結台灣IC設計產業在全球供應鏈中的重要地位。該公司以無晶圓廠（fabless）模式運作，專精於設計與行銷通訊、多媒體及周邊裝置所需的各類晶片。 瑞昱半導體的產品線多元，涵蓋乙太網路控制器、Wi-Fi解決方案、音訊編解碼器及高畫質多媒體晶片。這些高效能晶片支援數據傳輸、音訊處理與多媒體操控，廣泛應用於全球主機板、筆記型電腦、路由器及智慧裝置中。華碩（Asus）、技嘉（Gigabyte）、微星（MSI）等主要OEM客戶皆將瑞昱的解決方案整合至其產品。在乙太網路晶片領域，瑞昱提供支援 Gigabit、2.5G及5G速度的區域網路（LAN）介面卡，在PC主機板與網通設備市場佔據主導地位。此外，其ALC系列音訊編解碼器則嵌入在數百萬台筆記型電腦與桌上型電腦中，負責處理高傳真音效。 面對英特爾（Intel）、博通（Broadcom）及聯發科（MediaTek）等巨頭的競爭，瑞昱透過快速創新與穩固的OEM客戶關係，在成本效益高且出貨量龐大的消費性及PC市場取得競爭優勢。該公司專注於乙太網路實體層（Ethernet PHY）與音訊數位類比轉換器（DAC）等利基市場，並在這些類別中掌握顯著市佔。北極星市場情報（NorthStar Market Insights）資深財經編輯艾蕾娜·瓦茲奎茲博士（Dr. Elena Vasquez）曾表示，瑞昱半導體將可靠的晶片設計與物聯網（IoT）、5G及消費性電子產品的持久需求連結起來。 當前市場對瑞昱通訊IC的需求，正受惠於5G基礎設施、邊緣運算及物聯網裝置的擴張，而居家及辦公網路升級也持續推動乙太網路晶片的銷售。此外，8K串流與AI工作負載所需的頻寬，亦刺激對高速區域網路解決方案的需求。在供應鏈方面，瑞昱半導體仰賴台灣半導體產業聚落的支援，包括與台積電（TSMC）等晶圓代工夥伴的合作。對於尋求亞洲科技領袖投資機會的北美投資者而言，瑞昱半導體提供了一個穩定且具代表性的選項，能有效平衡以美國為中心的晶片製造商。 然而，瑞昱也面臨多重風險。其中，圍繞台灣的地緣政治緊張局勢，因其地理位置及對區域晶圓代工廠的依賴，被視為主要潛在風險。激烈的市場競爭亦對利潤造成壓力，尤其當競爭對手在高端市場加速創新時。半導體產業的週期性需求則導致營收波動，PC出貨量放緩會直接影響其業績。瑞昱必須持續投入研發，才能在中階市場維持其成本領先地位。該公司目前正積極投入Wi-Fi 7與PCIe Gen5技術的採用進程。 新聞關鍵字： 半導體 、 瑞昱 、 5G 、 AI 、 IC設計 、 intel 、 代工 、 台積電 、 微星 、 技嘉 記者：商傳媒 更多財經新聞 » 延伸閱讀 微星電競主機Woot狂砍900美元 搶攻暑期玩家市場 (商傳媒2026-07-29 09:26:14) MSI 2026 夏季健檢開跑 筆電、掌機等 6 六項產品皆提供免費健檢服務 (巴哈姆特 GNN2026-07-27 18:46:41) 慶祝品牌 40 週年 MSI 微星推出互動體驗小遊戲「超級組裝挑戰賽」 (巴哈姆特 GNN2026-07-27 18:46:23) 微星科技推出《玩具總動員》「蛋頭先生造型顯卡支撐架」 即日起限量開賣 (巴哈姆特 GNN2026-07-24 18:11:08) 微星推第六代 AMD EPYC 伺服器 搶攻 AI 與資料中心市場 (商傳媒2026-07-24 10:48:52) 超微AI大會一次看 Helios機櫃進入量產台廠受惠 (中央社2026-07-24 06:57:06) 聯手搶攻 AI 商機！微星 與 資策會 展開策略合作 共推 AI PC 與 Edge AI 應用 加速企業智慧化升級 (警政時報2026-07-23 13:09:46) 三星 OLED 電競螢幕殺出 300 美元震撼價 搶攻平價遊戲市場 (商傳媒2026-07-21 09:33:58) 微星科技與資策會展開策略合作 共推 AI PC 與 Edge AI 應用 加速企業智慧化升級 (威傳媒2026-07-16 21:44:24) 微星：RTX Spark高階款供不應求 首批貨接近完售 (中央商情2026-07-16 20:00:30) 最新財經新聞 友達第2季每股賺0.18元 投入新技術活化資產 (中央社 2026-07-30 17:38:52) 財部：台版肥咖CRS申報 筆數金額齊增 (中央社 2026-07-30 17:37:50) 苦茶油驗出苯駢芘超標！永豐餘生技退費方式 (今日新聞 2026-07-30 17:36:19) 韓國7月出口額估年增59% 晶片熱潮支撐動能不減 (中央商情 2026-07-30 17:35:48) 央行理事：若台股降溫 憂資金由股轉房推升房價 (中央商情 2026-07-30 17:34:25) 央行理事：若台股降溫 憂資金由股轉房推升房價 (中央社 2026-07-30 17:32:46) 外資賣超483億元 調節元大台灣50逾6萬張居冠 (中央社 2026-07-30 17:31:44) 韓國7月出口額估年增59% 晶片熱潮支撐動能不減 (中央社 2026-07-30 17:30:40) 阿里山林鐵x台啤5年 開發第五種品牌雙聯名釀造出二萬天晴新品 (台灣好報 2026-07-30 17:25:20) 日月光：目前封測製程重心在台灣 待時機擴展美國 (中央社 2026-07-30 17:18:22) 經濟部、勞動部共審 強迫勞動貨品機制公布 (今日新聞 2026-07-30 17:12:40) 台達電今年資本支出上看700億元 擬新增海外營運據點 (中央商情 2026-07-30 17:08:39) 台達電上半年獲利創高 鄭平：下半年成長沒有太大問題 (中央商情 2026-07-30 17:08:37) 台灣大有望併凱擘？林之晨：勢必會評估 (中央社 2026-07-30 17:08:13) 台達電資本支出上看700億 擬新增海外營運據點 (中央社 2026-07-30 17:07:09) 停進巴紐天然氣 經長：現貨可調整、長約仍需履約 (中央社 2026-07-30 16:47:29) 市調：明年DRAM供給續吃緊 NAND Flash轉寬鬆 (中央社 2026-07-30 16:38:22) 日月光投控資本支出估105億美元 先進封測營收明年再翻倍 (中央商情 2026-07-30 16:29:57) 日月光資本支出估105億美元 先進封測營收明年再翻倍 (中央社 2026-07-30 16:29:09) 台積電洩密案 2前工程師各判10年、6年定讞 (中央商情 2026-07-30 16:16:33) 人氣財經新聞 【台股盤後】台股多空激戰震盪逾1700點 終場下跌105點失守4萬點 (中央商情) 川寶布局TGV 完成成孔後電鍍金屬化設備試機 (中央商情) 台股多空激戰震盪逾1700點 終場下跌105點失守4萬點 (中央社) AI基建掀物流商機 中菲行：高價值空運快速成長 (中央商情) 熊本強震衝擊九州製造業 豐田、Sony等持續停工檢查 (中央社) 台北市新案房價抗跌 信義區每坪226萬實登居冠 (中央商情) 越南土地革命篇－與鹹水共生 稻蝦輪作逆境求生 (中央社) AI基建掀物流商機 中菲行：高價值空運快速成長 (中央社) 8月台股期指跌58點 (中央社) 三大法人賣超台股508.73億元 (中央社) 星巴克同店銷售額連4季成長 上調全年財務展望 (中央社) 越南現象篇－九龍江星光不浪漫 海水倒灌成農民夢魘 (中央社) 8月電子期跌 金融期漲 (中央社) 日月光投控第2季獲利同期新高 先進封測營收優預期 (中央商情) 夏慕尼哈根達斯聯名推「情人節套餐」 (今日新聞) 台北市新案房價抗跌 信義區每坪226萬實登居冠 (中央社) 台股4萬點失守！台積電撐盤收2205元 (今日新聞) 台股震盪 童子賢：別盯著綠紅聖誕樹、AI長期不泡沫 (中央社) 王品集團夏慕尼加速展店 目標明年底達21店 (中央社) 台股震盪 童子賢：別盯著綠紅聖誕樹、AI長期不泡沫 (中央商情) 熊本強震 中信銀與東京之星銀捐5千萬日圓 (今日新聞) 日企財報亮眼率日經指數收漲 SK海力士拖累韓股收低 (中央社) 熊本6.8地震 經長：主要受影響半導體業 (今日新聞) 日月光投控資本支出估105億美元 先進封測營收明年再翻倍 (中央商情) 台灣大種福電滿10年 綠能公益收入估破億元 (中央社) 轉虧為盈！友達Q2賺13.4億元 EPS 0.18元 (今日新聞) 日月光第2季獲利210億同期新高 先進封測營收超預期 (中央社) 星巴克同店銷售額連4季成長 上調全年財務展望 (中央商情) 日月光資本支出估105億美元 先進封測營收明年再翻倍 (中央社) 美國消費者信用分數創一年新高 信用卡拖欠率趨緩 (商傳媒) 限制強迫勞動貨品輸入 龔明鑫：審定會由經部勞部共審 (中央商情) 台積電洩密案 2前工程師各判10年、6年定讞 (中央商情) 肯塔基州西部將建AI資料中心 獲逾千億美元私人投資 (商傳媒) 新台幣貶8.8分 收32.454元 (中央商情) 市調：明年DRAM供給續吃緊 NAND Flash轉寬鬆 (中央社) 高通估Q4獲利不如預期 看好AI業務填補蘋果營收下滑 (中央商情) 停進巴紐天然氣 經長：現貨可調整、長約仍需履約 (中央社) 熊本強震衝擊九州製造業 豐田、Sony等持續停工檢查 (中央商情) 限制強迫勞動貨品輸入 龔明鑫：審定會由經部勞部共審 (中央社) 新台幣貶8.8分 收32.454元 (中央社) IBM 報告：AI 驅動網路攻擊暴增 56% 數據外洩成本飆近 500 萬美元 (商傳媒) 助熊本災後重建 中國信託銀行與日本東京之星銀行捐款5000萬日圓 (上報) 華爾街力挺加密永續合約 美國監管立場現轉機 (商傳媒) 台股收跌105點失守4萬點大關 台積電終場2205元、國巨收跌停 (上報) 台達電資本支出上看700億 擬新增海外營運據點 (中央社) 美晶片法注資格芯 3 億美元 強化 AI 晶片光子互連技術 (商傳媒) 台灣大有望併凱擘？林之晨：勢必會評估 (中央社) 歐元走軟助攻美元投資者 居留權計畫成本最高省6萬美元 (商傳媒) 菲國博弈營收受監管與通膨夾擊 今年恐陷7%衰退 (商傳媒) 台新新光金攜手台新銀 捐3000萬日圓馳援日本熊本震災重建 (品觀點) 台達電上半年獲利創高 鄭平：下半年成長沒有太大問題 (中央商情) 輝達擴大AI與先進技術佈局 聖荷西租賃新廠房搶進研發 (商傳媒) 台達電今年資本支出上看700億元 擬新增海外營運據點 (中央商情) 烏克蘭煉油廠攻擊戰術轉變 美法情報助鎖定俄關鍵設施 (商傳媒) 日月光：目前封測製程重心在台灣 待時機擴展美國 (中央社) 從企業經營看房市政策！百夫長集團主席陳志彬博士解析限貸令 (三星傳媒) 經濟部、勞動部共審 強迫勞動貨品機制公布 (今日新聞) 中信銀與東京之星銀行捐5000萬日圓 盼助熊本受災民眾重建家園 (品觀點) 韓國7月出口額估年增59% 晶片熱潮支撐動能不減 (中央社) 阿里山林鐵x台啤5年 開發第五種品牌雙聯名釀造出二萬天晴新品 (台灣好報) 外資賣超483億元 調節元大台灣50逾6萬張居冠 (中央社) 永豐金證券邀巴逆逆、前外資分析師程正樺開講 談AI泡沫迷思與反指標陷阱 (品觀點) 洛克希德馬丁擴廠增700職位 強化美國軍備產能 (商傳媒) 日股7月跌逾11％！法人看好抵禦波動風險 點名「NIPPON」結構性優勢 (品觀點) 央行理事：若台股降溫 憂資金由股轉房推升房價 (中央社) 財部：台版肥咖CRS申報 筆數金額齊增 (中央社) 苦茶油驗出苯駢芘超標！永豐餘生技退費方式 (今日新聞) 友達第2季每股賺0.18元 投入新技術活化資產 (中央社) 國泰世華銀：油價風險加劇美國聯準會9月升息壓力 (中央商情) 台股反彈無力收跌105點 失守4萬點大關 (中央商情) 日經：SpaceX供應鏈去中 排除中國籍員工設備 (中央商情) AI晶片需求強勁 三星電子Q2營利暴增19倍創歷史新高 (中央商情) 三星電子財報報喜 激勵韓股Kospi指數盤中強彈逾5% (中央商情) 日本2027年4月起食品消費稅首次降至1% 為期2年 (中央商情) 韓國電信KT遭駭致未經用戶授權小額支付 遭罰12億元 (中央商情) 開源基金會3年投入3億元 提升台灣供應鏈影響力 (中央商情) 美國限制先進機器人進口 北京稱將反制 (中央商情) 北市攜手美國20州辦商機媒合會 助台美經貿發展 (中央商情) 男女平均所得差距 財政部統計2024年縮小至1.54倍 (中央商情) 英國宣布3636億核潛艦計畫 支持國防與青年就業 (中央商情) 權值股領軍 台股盤中強彈逾千點觸及41000點 (中央社) 緯創布局AI基建 台南算力中心估2027年首季建置完成 (中央社) 研調：熊本地震JASM停機 台積電第3季營收影響應有限 (中央社) 索尼擬收購騰龍 相機鏡頭市場可能洗牌 (中央社) AI晶片需求強勁 三星電子Q2營利暴增19倍創歷史新高 (中央社) AI投資隱憂衝擊亞股 聯準會按兵不動增利率不確定性 (中央社) 高通估Q4獲利不如預期 看好AI業務填補蘋果營收下滑 (中央社) 美國限制先進機器人進口 北京稱將反制 (中央社) 男女平均所得差距 財政部統計2024年縮小至1.54倍 (中央社) 三星電子財報報喜 激勵韓股Kospi指數盤中強彈逾5% (中央社) 台股跌105.88點 (中央社) 國泰世華銀：油價風險加劇美國聯準會9月升息壓力 (中央社) 開源基金會3年投入3億元 提升台灣供應鏈影響力 (中央社) 索尼擬收購騰龍 相機鏡頭市場可能洗牌 (中央商情) Meta 重押 AI 拖累股價大跌 投資人憂回報不如預期 (商傳媒) 台股反彈無力收跌105點 失守4萬點大關 (中央社) 美利率凍！美元跌後反彈 台幣早盤貶快1角 (今日新聞) 美禁國外機器人進口 業者看台廠供應鏈具3大優勢受惠 (中央社) 看台股暴跌 國安基金操盤手：若失序會處理 (今日新聞) 援助熊本災後重建 台新新光金捐3千萬日圓 (今日新聞) 新台幣午盤貶9分 暫收32.456元 (中央社) 【台股盤中】權值股領軍 台股殺完融資後強彈逾千點 (中央商情) momo富昇物流徵百名司機 績優年薪上看百萬元 (中央社) 韓國金融界推4措施應對槓桿ETF 分散再平衡交易 (中央社) AI新十大建設 教育、醫療、司法導入成果 (今日新聞) AI投資隱憂衝擊亞股 聯準會按兵不動增利率不確定性 (中央商情) 紐約聯準銀行：美國高評級公司債市場運作失能達近三年高點 (商傳媒) 慧榮：下半年持續強勁成長 全年營收估增逾100% (中央商情) 台股歷次盤中跌逾2千點 法人：後市表現佳 (今日新聞) 韓國金融界推4措施應對槓桿ETF 分散再平衡交易 (中央商情) 慧榮：下半年持續強勁成長 全年營收估增逾100% (中央社) 緯創布局AI基建 台南算力中心估2027年首季建置完成 (中央商情) 美商藝電執行長年薪3865萬美元 員工平均薪資305倍引議論 (商傳媒) Plaid 推出創新 AI 模型 深層解讀用戶金融軌跡 (商傳媒) 美眾院通過國防法案引爭議 美以軍事合作非「合併」 (商傳媒) 聯準會決策在即 美元面臨下行風險 豐業銀行示警 (商傳媒) 方舟投資連兩日加碼加密概念股 押寶 CLARITY Act 立法利多 (商傳媒) 萊茵河乾旱水位創低 歐洲油化品供應鏈陷停擺危機 (商傳媒) 美國3億美元注資格芯 劍指矽光子技術發展 (商傳媒) 高通膨與中東戰火施壓 美國聯準會連續五次維持利率不變 (商傳媒) 美國利率連5凍 聯準會主席華許：沒有降通膨的魔法棒！ (品觀點) Rhodium Group：美2030年代新增發電量 政策左右再生能源或天然氣 (商傳媒) 美銀證券集團重申維諦技術買入評級 目標價 440 美元 (商傳媒) 美加關稅戰升溫 加拿大總理強調穩定能源供應以維信譽 (商傳媒) NEC首季財報亮眼 AI業務「Blue Stella」營收強勁成長 (商傳媒) AI用電需求噴發 核能發電股重回投資人視線 (商傳媒) 3COINS插旗臺北複製日本平價策略 誓成「雜貨界優衣庫」 (商傳媒) 投資美股領股息需留意 加拿大免稅儲蓄帳戶揭美國預扣稅陷阱 (商傳媒) 看戲兼做公益！創世兒童劇8/15登場 (商傳媒) 傳伊朗採購中國製攜帶型防空飛彈 中國外交部否認軍售消息 (商傳媒) OpenAI奧特曼會晤美國會議員 談AI風險與發布科研用新模型 (商傳媒) 伊朗發射飛彈襲美基地 川普嗆聲、國際油價跳漲 (商傳媒) 美國證管會控地產信託詐欺 創辦人挪用近 500 萬美元 (商傳媒) 伊朗數週內將獲中國製肩射飛彈 最多400套加劇區域失衡 (商傳媒) BMW傳全球裁員8,000人 加速轉型因應中國電動車競爭 (商傳媒) 能源巨頭求售美國 Explorer 輸油管道股權 估值逾 35 億美元 (商傳媒) 美國關稅衝擊巴西雞蛋出口逾四成 禽類業承壓轉向新市場 (商傳媒) 北美REITs第二季財報報喜 Morguard獲利轉正、Primaris戰略奏效 (商傳媒) 加密貨幣基金經理逃稅判囚三年 須賠償逾 340 萬美元 (商傳媒) AI 巨頭聯手呼籲：美國應主導國際 AI 監管減速 (商傳媒) 【金屬盤後】金價漲 銅價跌 (中央商情) 空中光電板1／屋頂光電新制恐有變數？迷糊上路代價高 「這類住宅」衝擊最大 (周刊王) 阿特曼：AI代理失控如科幻事件 真切感受到威脅 (中央商情) 空中光電板2／屋頂種電政策成敗「管委會」扛？ 沒錢維護下場慘淪「空中廢棄物」 (周刊王) 台股早盤震盪逾千點 台積電上漲40元 (中央商情) 聯準會利率連5凍 外界關注華許如何兌現降通膨承諾 (中央商情) 【盤前焦點】美股下挫費半摔逾5% 法人估台股打底時間拉長 (中央商情) Fed按兵不動「3官員、市場皆不買單」！會議5大要點一次看 (周刊王) 台股早盤震盪逾千點 台積電上漲40元 (中央社) 美高梅Q2營收創紀錄 賭城大道與數位業務表現亮眼 (商傳媒) 聯準會利率連5凍 外界關注華許如何兌現降通膨承諾 (中央社) 新台幣開盤貶1.4分 為32.38元 (中央社) Fed按兵不動引發憂慮！道瓊暴跌逾1千點 創去年4月以來最大單日跌幅 (周刊王) 中東情勢推升油價助長通膨擔憂 美股重挫半導體類股承壓 (商傳媒) 台股急拉站回4萬點 開盤後翻紅漲逾360點 (今日新聞) 泰國現象篇－魚販生計受衝擊 漁村世代斷裂 (中央社) 美股下挫費半摔逾5% 法人估台股打底時間拉長 (中央社) 全球矽晶圓出貨創14季新高 AI需求強勁 (中央社) 台股開盤漲9.76點 (中央社) 泰國公民運動篇－保育母親之河 湄公河學校揭露重金屬污染 (中央社) 台股逆轉！早盤跌634點隨後強彈逾千點 (今日新聞) 油價飆漲 VIX 恐慌指數攀升 納斯達克在聯準會前重挫 (商傳媒) 快訊／台股開盤震盪 一度下挫逾600點、失守4萬點大關 (上報) 美國好市多油價為何能壓到極低？ (草根影響力新視野) 新加坡祭出9億坡元振興方案 多管齊下鞏固經濟競爭力 (商傳媒) AI類股賣壓籠罩 台積電盤中重挫4.1%半導體供應鏈受創 (商傳媒) 烏克蘭襲擊俄國兩大煉油廠 全球能源供應隱憂再起 (商傳媒) 伊朗突襲約旦美軍基地與荷莫茲海峽 油價急升美財政部宣布制裁 (商傳媒) 台積電、台灣50還能買嗎？黃世聰曝抄底關鍵條件 (品觀點) 聯準會分歧美元承壓 日銀決策將左右日圓匯率動向 (商傳媒) 美國原油庫存意外驟降720萬桶 市場關注油價走向 (商傳媒) 聯準會會議後美股續跌 那指連六黑 半導體指數重挫逾5% (商傳媒) 聯準會利率按兵不動 9比3分歧投票 市場料9月升息機率降 (商傳媒) 美元指數延續回檔走勢 聯準會凍息推升匯市波動 (商傳媒) 中東空襲推升油價飆漲近7% 埃克森美孚股價揚3.3% (商傳媒) 美國原油庫存銳減720萬桶創多年新低 國際油價應聲勁揚 (商傳媒) 歐洲股市走低：精品業績喜憂參半，油價攀升科技股續弱 (商傳媒) Binance.US 擬申請美 CFTC 牌照 搶攻美國預測市場業務 (商傳媒) 聯準會維持利率不變 全球股市重挫那指跌逾1.7% (商傳媒) 美國原油庫存大幅銳減720萬桶 油價看漲消費者成本增 (商傳媒) 台股勉強站回4萬點 何時止跌先看3大指標 (卡優新聞) 電玩遊戲課金有祕笈 信用卡賺回20%決殺技 (卡優新聞) 學貸利率降至0.775% 臺銀8/1起受理申請 (卡優新聞) 友達ADR29日上漲0.14美元漲幅1.96%折台股23.63元 (中央商情) 日月光投控ADR29日下跌2.81美元跌幅8.28%折台股503.61元 (中央商情) AI軍備競賽開銷驚人 Meta第二季現金流大減91% (中央社) 中華電信ADR29日下跌0.11美元跌幅0.25%折台股139.59元 (中央商情) 聯電ADR29日下跌0.25美元跌幅1.44%折台股110.76元 (中央商情) 美國揚言打擊伊朗 國際油價大幅上揚 (中央社) 【歐股盤後】互有漲跌 (中央商情) 【美股盤後】收低 (中央商情) 台積電ADR29日下跌17.64美元跌幅4.50%折台股2425.31元 (中央商情) 基準利率不動美債殖利率飆高 通膨難解拖累道瓊大跌 (中央社) 聯準會利率不動但分歧加劇 9月升息機率破5成 (中央社) 晶片股拋售潮未止 美股收黑費半跌逾5% (中央社) 聯準會利率不變3票反對 華許形容決策過程如家庭爭吵 (中央社) 【能源盤後】上揚 (中央商情) 美伊戰火推升油價 聯準會續觀望利率連5凍 (中央社) 台灣大攜可樂旅遊搶進BNPL先買後付市場 (自立晚報) 金管會推金融大回饋提22項目 (自立晚報) 行動版 電腦版 分類新聞 最新 政治 社會 財經 科技 娛樂 體育 生活 國際 健康 寵物 情商 星座 職場 流行 新聞人物 政治 社會 娛樂 體育 科技 國際 財經 新聞專題 精選專題 星座 算命 農民曆 擇日 對獎 樂透 統一發票 氣象 今日天氣 一週天氣 旅遊天氣 國際天氣 天氣圖 警特報 影音新聞 政治 社會 財經 科技 娛樂 體育 生活 國際 健康 消費 旅遊 其他 新聞照片 政治 社會 財經 科技 娛樂 生活 國際 健康 消費 旅遊 大陸 其他 雜誌 總覽 政治 投資 管理 消費 好生活 藝文 公益 愛地球 關鍵字 最新關鍵字</t>
+          <t>ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå ¨çICæ°åµéçµèºç£åå°é«çæ é - å°åå¸é»è ¦åæ¥­åæ¥­å ¬æ Taipei Computer Association æå¡ç»å ¥ å å ¥TCA äººææå ç«å §æå° èªè­ TCA æ¬æç°¡ä» å¤§äºç´ çµç¹æ¶æ§ çç£äº å°æ¥­è¯ç æå¡æå ç¢æ¥­æ¨å»£ å±è¦½æé· åé¡ç«¶è³½ æ°åµæ´»å è¨ç«è³æº åå¥½é£çµ æ°èä¸­å¿ ç±éæ°è äººç©æ¡è¨ª æå¡å°è¨ª æ´»åæ å ± å½±åæ«¥çª TCA Video Gallery TCA Photo Gallery ç«å §æå° × æå° éé ç±éæ°è ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå ¨çICæ°åµéçµèºç£åå°é«çæ é IC Taiwan Grand Challengeåéæ¼CES 2025å±ä¸­ä¹TTAåå®¶é¤¨ä»ç´¹ç«¶è³½ åå®¶ç§å­¸åæè¡å§å¡æï¼NSTCï¼æå°çåéåµæ°ç«¶è³½IC Taiwan Grand Challengeï¼ICTGCï¼å°èå ¨çæ°åµå±æ InnoVEX ä¸»è¾¦å®ä½âå°åå¸é»è ¦å ¬æï¼TCAï¼æ¼ CES 2026 æéå ±åååä¸ç³»ååéäº¤æµæ´»åã é¢å° AI ç¡¬é«ãæ©å¨äººãå é²æ¶çèé«ç§æåµæ°å¿«éæ¼é²çå ¨çæµªæ½®ï¼InnoVEX æçºä½çºåéæ°åµå°æ¥äºæ´²æå é²ç§æç¢æ¥­çééµå ¥å£ï¼æ­¤æ¬¡ ICTGC x InnoVEX åéæ¨å»£è¡åé¤äºå¨CESå±æäº®ç¸ï¼ä¹å¾å°æ¼ 1 æ 13 æ¥å¨ç½è°·èè¾¦å°å ´æ´»åï¼åå©æ´å¤ç½è°·åéæ·±å ¥äºè§£å¦ä½ä¸²é£å°ç£å¨åå°é«è AI é åçä¸çç´è³æºï¼å±ç¾å°ç£æ¨åè·¨ååä½èæ¯æä¸ä¸ä»£ééµæè¡çæ±ºå¿èæ¿è«¾ã ICTGCãInnoVEXå°æ¼CES 2026é éç»å ´ å»£éå ¨çæ°åµèè¨TTAåå®¶é¤¨ å¨ CES 2026å±ææéï¼ IC Taiwan Grand Challengeï¼ICTGCï¼å°ææå ¨çåµæ°å±æInnoVEX å°äº®ç¸æ¼CES Eureka Park ç Taiwan Tech Arenaï¼TTAï¼åå®¶é¤¨ï¼Booth Venetian Expo, Hall G â 62201ï¼ãTTA çºåç§ææ¼ CES è¨­ç«çå®æ¹å±åï¼éå®å ·åç ç©¶å°åèæªä¾æ·±ç§ææ½åçæ°åµåéï¼æ¯å¹´å¸å¼å ¨çæè³äººãåéåªé«èç§æé è¢åè¨ªã ICTGC åéä¹å°æ¼ TTA Stage æ·±å ¥ä»ç´¹èºç£å¯ä¸å ·æå®æ´è¼å°æ©å¶ãå¯æ·±å ¥å°æ¥ç¢æ¥­éä¹åå°é«æ°åµç«¶è³½ï¼åä»¥ç²çæ°åµæ¡ä¾åäº«ICTGCå¦ä½çºæ°åµæä¾å¾è¨­è¨å°éç¢çå®æ´å éæ¯æã åéè§å±è äº¦æ­¡è¿èè¨ç¾å ´è InnoVEX åICTGC åéäº¤æµï¼ç­è§£è³æºéçµèç«¶è³½çå¾µä»¶åèæ¹å¼ã ICTGC 2026 å ¨çå¾µä»¶éè·ï¼å©æ»åéæ°åµéµçµç½å³¶ ICTGC ç¾æ­£éæ¾å ¨çå ±åï¼ç³è«æªæ­¢æ¥çº 2026 å¹´ 2 æ 28 æ¥ãæ­¡è¿ä¾èª AIãæ©å¨äººãåå°é«æè¡ãææ¸¬ç³»çµ±ãæ¬¡ä¸ä»£éç®ãæ·±ç§æç­é åçæ©ææ°åµãå­¸ç åéèæè¡éç¼è æäº¤å ·æ½åçåµæ°æç¨ææ¡ã çºåå©åéæ°åµæ´å¤§å½±é¿åãå éæè¡è½å°ï¼å ¥é¸åéå°æ¼ 2026 å¹´ 6 æ 2 è³ 5 æ¥å¨å°åèè¡ç COMPUTEX TAIPEI è InnoVEX æ°åµå±ä¸­ï¼ç²å¾å è²»åå±æ©æã ä½çºäºæ´²ææ¨æ§ç B2B ç§æå±ï¼COMPUTEX çµå InnoVEX ä¸ç«å¼çåµæå°æ¥èåéåªåèå°ï¼è®åéææ©æç´æ¥éçµè£½é å¤¥ä¼´ãåå°é«ä¾æéãåµæè³æºèåéè²·ä¸»ï¼çºå¸å±åå°é«ç¢æ¥­éä¹ééµè·³æ¿ãééICTGCè¨ç«ï¼ç²çåéå¯æææå°ç£åå°é«çæ ç³»ï¼å ±åéç¼å ·åéç«¶ç­ååµæ°è§£æ±ºæ¹æ¡ã å ±åç¶²åï¼ictaiwanchallenge.org ICTGCé¦åº¦ç½è°·ç»å ´ã1 æ 13 æ¥ææInnoVEXèè¾¦è«å£æ·±åå°ç½åå°é«èAIåä½ å»¶çºCESåéæ¨å»£åè½ï¼ICTGCå°æ¼2026å¹´1æ13æ¥é¦åº¦å¨ç½è°·Palo AltoçStartup Island TAIWAN â Silicon Valley Hubèè¾¦ãBridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergiesãè«å£ãè«å£å¯èç½è°·åµæ¥­è ãæè³äººèæè¡å°å®¶ï¼æ¢è¨å¦ä½åç¨å°ç£åå°é«èAIä¾æéè³æºï¼å¼·ååµæ°è½å°èåéåä½ï¼æ´æ¼ç¾å ´çºæèè¶£åèæ·±åº¦ä»ç´¹å°ä»ç´¹ç«¶è³½å¾µä»¶å §å®¹èè©é¸éé»ï¼åæåæ¡ä¾åäº«ã åéåéäº¦å¯èç±åå æ­¤è«å£ï¼äºè§£æ´å¤æ¼å°ç£ COMPUTEX/InnoVEX å±åºè³è¨ï¼åå©å ¶ææ¡æåé²å ¥å¸å ´çè·¯å¾ä¸¦èèºç£ICTç¢æ¥­çæ ç³»å»ºç«å¯¦è³ªé£çµã æ­¤æ¬¡æ´»åè«å£é¤äºéè«åä½è¬è Laura Swan-Silicon Catalyst Ventures å ±ååå¤¥äººï¼Andy Lombard-Tesoro Venture Capital ç®¡çåå¤¥äºº, Janis Skriveris-Plug and Play Ventures æè³ç¸½ç£æ¨é«ç§æè² è²¬äººä»¥åSam Fok-femtoAI å ±ååµè¾¦äººæ¨å·è¡é·ï¼å°åå¸é»è ¦å ¬ææ¥æ«»å§¿å¯ç¸½å¹¹äºå°å¸¶é åéæä¾ç½è°·æ°åµäººå£«æ´å¤éµçµå°ç£çè³æºï¼å ±åèå£¯æé·ã ç¾å ´å°åæé²è¡å ¨çç´æ­ï¼é è¨å°å¸å¼å ¨çç¸éæ°åµäººå£«è§çãç´æ­é£çµçºï¼https://www.youtube.com/live/ruXS6oe7WNA æ´»åè³è¨ Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies 2026 å¹´ 1 æ 13 æ¥ï¼ææäºï¼ï½ä¸å 5:00ï¼PSTï¼ Startup Island TAIWAN â Silicon Valley Hub 299 California Ave STE 300, Palo Alto, CA 94306 U.S.A. åèç¶²åï¼ ãBridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergiesãè«å£ ï¼ç¼ä½æéï¼2026-01-02ï¼ ååè¡¨é  è½å¯ ã åå° ã åäº« å»¶ä¼¸é±è® InnoVEX 2026 ç«¶è³½ç»å ´ AVITICãPlug and PlayãPwCé¦æ³¢ç¹å¥çé½ç¼ï¼è¯æè³¦è½æ°åµéæåéçåè½é å®ç¢é³ä¿èè£äºé·æ¥ä»»çäºé· æè¨±å ±åè´åç¢æ¥­åéå äººç©æ¡è¨ª åç§æç¢å­¸èæå¾·çèé· : æ¨åç¢å­¸åä½è®ç ç¼ææè½å° æ°ä»»çç£äºæ¡è¨ªç³»åå ±å°(7)-æ¬æçäºæ¨å®ç¢æºé«é£å æ©è£äºé· : ãè³éè¨çµåçæãæ¯å°ç£æªä¾ç«¶ç­åªå¢ æ°ä»»çç£äºæ¡è¨ªç³»åå ±å°(6)-æ¬æçäºæ¨éææ©å¨äººé»è­å¿ çéé· : Edge AIæ¯å°ç£æ©å¨äººç¢æ¥­å½éè¶ è»çæ©æ ï¼ æ´å¤è¨æ¯ æå¡å°è¨ª TCAæå¡ä¼æ¥­å°è¨ª -å±¹å²ç§æï¼Eleosï¼ TCAæå¡ä¼æ¥­å°è¨ª -é²ä¸æè¾° TCAæå¡ä¼æ¥­å°è¨ª -å°ç£è³æç§æ ï¼ æ´å¤è¨æ¯ å»£å®£æå é±ç§æ¿ç­ è¯çµ¡æå äº¤éä½ç½® æå¡eåé Â© 2002ï¼2026 å°åå¸é»è ¦åæ¥­åæ¥­å ¬æ çæ¬ææ</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -667,74 +717,12 @@
           <t>Success</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IC semiconductor</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ç¾è¡ç¦é»ï¼ON Semiconductor(ON.US) | 23:32:11(GMT+8) - å°è¦è²¡ç¶</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://www.ttv.com.tw/finance/view/042026232332134174FF5E00432693B2142340DE48AAE792/587</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Fri, 24 Apr 2026 07:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>ç¾è¡ç¦é»ï¼ON Semiconductor(ON.US) | 23:32:11(GMT+8) - å°è¦è²¡ç¶ é»æé¡¯ç¤º è²¡ç¶å°ç¯ç®è¡¨ å°è¦è²¡ç¶å°ç²çµ²å å°è¦æ°è ç¾è¡ç¦é»ï¼ON Semiconductor(ON.US) | 23:32:11(GMT+8) 2026/4/24 åéè¡å¸ MoneyDJæ°è 2026-04-23 23:32:13 æ¸ä½å §å®¹ä¸­å¿ ç¼ä½ON Semiconductorï¼ON.USï¼è¡å¹ç¤ä¸­è¡¨ç¾å¼·å¢ï¼æäº¤å¹ä¾å°97.78ç¾å ï¼æ¼²å¹ é9.87%ï¼ç¤ä¸­æé«è§¸å98.62ç¾å ï¼æäº¤éçº649,794è¡ï¼åå¹96.30ç¾å ã å¾ç¤ä¸­èµ°å¢ä¾çï¼è³éæé¡¯ç©æ¥µæ¹§å ¥ï¼ä¹åæ å¸å ´å°å ¬å¸å¾å¸è¡¨ç¾æ±æåå¤æå¾ ãON Semiconductoræ¯ä¸å®¶æä¾é»æºç®¡çèææ¸¬è§£æ±ºæ¹æ¡çåå°é«å ¬å¸ï¼ç¢åæ¶µèSiCèGaNåçåå°é«ãåé¡ææ¸¬å¨ä»¥åé¡æ¯ICï¼æç¨ç¯åéåæ±½è»ãå·¥æ¥­èè³æä¸­å¿ç­é åã æ­¤æ¬¡è¡å¹ä¸æï¼åæ åºå¸å ´çå¥½å ¶å¨AIè³æä¸­å¿èé«å£é»åè½æé åçæé·æ½åãé¨èé«æè½éç®èé»åæçéæ±æçºæåï¼ON Semiconductoræèåçå ä»¶èææ¸¬æè¡å¸å±ï¼å ·ååå ¥é«æé·æç¨å¸å ´çåªå¢ï¼ä¹è®æè³äººå°å ¶æªä¾çéç©ºéç¢çæ´å¤æ³åã å¾ç¢æ¥­è¶¨å¢ä¾çï¼åå°é«éæ±æ­£åæ æ¼AIä¼ºæå¨èè³æä¸­å¿æ´å»ºå¸¶åï¼ç¸éä¾æéä¸­çå å­¸æª¢æ¸¬ãæ¸¬è©¦ä»¥åé«å£é é»é åä¹åæ­¥è½è¶¨æ´»çµ¡ãå¦ä¸æ¹é¢ï¼SiemensèTSMCå¨AIé© åæ¶çè¨­è¨ä¸çåä½æçºæ´å¤§ï¼åéåºå£æ¸æèåéåªé«å ±å°äº¦é¡¯ç¤ºï¼åå°é«è¨å®åè½æ­£å¨ååãå¨æ´é«å¸æ³éæ­¥æ¹åä¹ä¸ï¼ä¹é²ä¸æ­¥æ¯æON Semiconductorå¨æè¡å¯¦åèå®¢æ¶å¸å±ä¸çåªå¢ï¼ä¸¦å¼·åå¸å ´å°å ¶å¾çºç²å©è¡¨ç¾çæå¾ ã è³æä¾æºï¼ MoneyDJçè²¡ç¶² æ­¡è¿å å ¥ å°è¦è²¡ç¶å°ç²çµ²å ï¼ ç±éé»é± » ä¸æGalaxyæ°åç¼è¡¨ ç§ä¸æ¬¾æºçæ©åå ¨æ°æºæ §æé¶ ãç¾è¡ãéçææ¸æ¶é« AIææå¼ç§æè¡ä¸è· åçå ä»¶ä¾éæªè®ï¼å¼·èä¸åå¹´çæ¶å¢å¹ æåªä¸åå¹´ ç·¯åµæ´å¤§æ°äºæ¥­ï¼ç¼æåé·æç²å©è½å çæ¬çç¼7.1å¼·é å°ç©é»åæäº æ¥BBUå¤§å®¢æ¶è¡åºï¼é ç¥¥æªä¾ä¸å¹´AIæç¨æä¿è­ å¸å±AIãHPCåæ© è¶ è±æå¹´çºæ´Flip Chipç¢è½ ç¾ç³»CPUæ°å¹³å°äº¦å°ååï¼éé´»åç±çè¿æé· ç¤¾ç¾¤åäº« » èºç£é»è¦äºæ¥­è¡ä»½æéå ¬å¸ çæ¬ææã©2015 Taiwan Television Enterprise, Ltd. All Rights Reserved. é»æé¡¯ç¤º åéè¡å¸ ç§æèå éèå¸å ´ ç¢æ¥­åæ  è²¡ç¶è³è¨ çæ´»è¬è±¡ ç¾é£æ¶è²» â²TOPâ²</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>IC semiconductor</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>【即時新聞】這「1檔」半導體轉強，NVTS最新漲2.94%還能追嗎？ | CMoney投資網誌</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://cmnews.com.tw/article/newsyoudeservetoknow-d463d065-3823-11f1-bf7c-8951ef46c39f</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Wed, 15 Apr 2026 07:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>【即時新聞】這「1檔」半導體轉強，NVTS最新漲2.94%還能追嗎？ | CMoney投資網誌 清空 搜尋紀錄 全部清除 取消 開始使用 投資網誌 登入 台股 新聞快訊 盤中獵報 籌碼k線專欄 ETF/期貨/原物料 美股 美股研究報告 美股新聞 美股財報會議 美股入門 大師選股 美股K線 Alpha's Newsletter 基金 基金新聞 基金排行 熱門 研究報告 理財達人 小資女艾蜜莉 不敗教主陳重銘 權證小哥 林恩如 阿格力 沈萬鈞 愛德恩小朋友 朱家泓x林穎 大俠武林 張捷 股市隱者 老簡免費文章 不魯 順流小畢 BC股倉 股人阿勳 Sara 無聊詹 蔡斯 怪博士 Dr.Selena好老公選股 美股夢想家施雅棠 尼克萊 春燕來了 新手入門 投資策略 基本分析 技術分析 籌碼分析 生活理財 生活理財 投資心得 退休規劃 CMoney官方 Money錢 林奇芬 狄驤 葉芷娟 李勛 金融人類學徒 清流君 美股航海王 游庭皓 張遠 存股攻城獅-聰聰 學投資，也學人生 人生學習 【即時新聞】這「1檔」半導體轉強，NVTS最新漲2.94%還能追嗎？ 首頁 美股 美股新聞 【即時新聞】這「1檔」半導體轉強，NVTS最新漲2.94%還能追嗎？ 權知道 我們重視「知」的權利 不惜抽絲剝繭、深入調查 只為讓投資人不錯過重要的投資訊息 權知道 2026-04-15 01:03 405 NVTS 近期市場對次世代半導體技術的關注度持續提升，其中專注於純粹次世代半導體技術的 Navitas Semiconductor (NVTS) 成為焦點。該公司致力推動「電氣化世界」願景，以全球首創的氮化鎵（GaN）功率 IC 及獨特的溝槽式平面碳化矽（SiC）技術在產業中佔據一席之地，旨在支援更高效能與潔淨能源的永續發展。 隨著市場熱度增加，相關衍生性金融商品也受到資金留意，例如 Tradr 每日2倍做多 NVTS 主動型 ETF（代號：NVTX）。最新資料顯示，該檔 ETF 預計於 2025 年 12 月 17 日進行除息，配息總額約為 3.5155 美元，這為關注該個股波動性與資金流向的資深投資人，提供了另一個觀察市場情緒與籌碼動能的參考指標。 Navitas Semiconductor (NVTS) ：近期個股表現 基本面亮點 Navitas Semiconductor (NVTS) 主要研發超高效能的半導體解決方案，其營運與業務重點包含： 核心技術：專注於氮化鎵（GaN）與碳化矽（SiC）技術，提供高功率密度的解決方案。 產品應用：功率 IC 高度整合了驅動、控制與保護功能，主要應用於行動裝置、消費性電子、企業級應用及電動車（eMobility）等新能源領域。 營收結構：目前公司營運版圖涵蓋美國、歐洲與亞洲等地，其中最大宗的營收來源為中國市場。 近期股價變化 根據 2026 年 4 月 13 日的最新交易數據顯示，該股價呈現震盪走高的格局。當日開盤價為 9.37 美元，盤中最高觸及 9.86 美元，最低來到 9.12 美元，終場收在 9.82 美元，單日上漲 0.28 美元，漲幅達 2.94%。在交易量方面，當日成交量為 13,571,257 股，較前一交易日的成交量變動幅度為 -8.25%。 總結而言，Navitas Semiconductor 在次世代功率半導體領域具備明確的技術佈局，相關主動型 ETF 亦反映出市場對其資金動能的關注。後續投資人可持續追蹤該公司在中國市場的營收表現，以及終端消費電子與電動車市場的供需動態，作為評估 (NVTS) 長期營運發展與潛在風險的重要依據。 文章相關標籤 Top50美股新聞 美股 美股新聞快訊 本文內容轉載 於此 關於作者 權知道 我們重視「知」的權利 不惜抽絲剝繭、深入調查 只為讓投資人不錯過重要的投資訊息 作者文章 【即時新聞】台達電(2308)獲利狂增88%！法說前夕，這「5檔概念股」多空交戰？ 【即時新聞】晶豪科(3006)爆量震盪多空激戰！這「3檔概念股」資金輪動誰接棒？ 【即時新聞】宇瞻(8271)爆量急跌逾7%，這「2檔記憶體概念股」盤中多空激戰！ 更多文章 今日最熱 1 【台股盤後】漲價題材陸續追繳，加權一度回測半年線 2 輝達「循環融資」疑慮發酵，牽動全球晶片股，這7檔重挫台股一度大跌逾2,000點 3 【股市爆料同學會專屬】－開戶領 30 天籌碼 K 線 VIP 4 記憶體股重挫解析：長鑫科技（CXMT）掛牌引爆全球賣壓 5 崩盤怎麼辦？「腳麻動不了」也要活下來：顧好情緒4步驟＋看懂大盤籌碼訊號 全站最新 【00405A】07/30 操作日報｜揮刀出清國巨，資金轉進台達電 19minutes ago 【00406A】07/30 操作日報｜資金轉向金融傳產避險？ 20minutes ago 【ETF籌碼日報】官股大買0050，外資、自營商大賣0050達119億 31minutes ago 2026.7.29 期指實戰錄 - VVIP 限定 anhour ago 2026.7.28 期指實戰錄 - VVIP 限定 anhour ago 最熱 最新 作者 1 【即時新聞】台達電(2308)獲利狂增88%！法說前夕，這「5檔概念股」多空交戰？ 2 【即時新聞】晶豪科(3006)爆量震盪多空激戰！這「3檔概念股」資金輪動誰接棒？ 3 【即時新聞】宇瞻(8271)爆量急跌逾7%，這「2檔記憶體概念股」盤中多空激戰！ 更多文章 1 【00405A】07/30 操作日報｜揮刀出清國巨，資金轉進台達電 2 【00406A】07/30 操作日報｜資金轉向金融傳產避險？ 3 【ETF籌碼日報】官股大買0050，外資、自營商大賣0050達119億 1 【台股盤後】漲價題材陸續追繳，加權一度回測半年線 2 輝達「循環融資」疑慮發酵，牽動全球晶片股，這7檔重挫台股一度大跌逾2,000點 3 【股市爆料同學會專屬】－開戶領 30 天籌碼 K 線 VIP 收藏內容 讓好文不錯過 立即收藏 取消 前往綁定 取消 確定購買 要永久刪除文章嗎 「」將被永久刪除，且這項操作無法復原。 取消 永久刪除 您尚未登入 登入會員才能編輯或管理文章，請先登入再進入此頁 取消 登入</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>3ccc8d408c7b8b6a576a6c109f4331f3fdb5cb914a2a24b036a161f9c12492a9</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete V2.2 base web understanding layer
</commit_message>
<xml_diff>
--- a/output/result.xlsx
+++ b/output/result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,37 +476,53 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
+          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 - TechNews 科技新報</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
+          <t>https://finance.technews.tw/2026/05/01/semiconductor-inflation-trend-takes-shape-wafer-foundries-ic-design-price-hikes/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
+          <t>Fri, 01 May 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>科技產業資訊室</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>TechNews 科技新報</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>半導體通膨趨勢成形，因應成本高漲，包括晶圓代工及 IC 設計廠紛紛調漲價格，對於智慧手機等消費產品市場影響逐步顯現，智慧手機等今年出貨量恐面臨衰退壓力。
+半導體廠法人說明會陸續登場，成本壓力及產品價格策略成為法人關注的焦點。晶圓代工廠除將持續投入技術開發及擴充產能，中東緊張局勢也造成能源和物流等成本升高。
+晶圓代工廠
+已搶先於今年1月調漲驅動IC及感測器代工價格，3月調漲功率元件代工價格，
+先進跟進於4月調漲代工價格，
+也於4月通知客戶，將於下半年調整價格。
+不僅晶圓代工價格調漲，後段封測價格也傳出漲價消息，IC設計廠紛紛決定調漲產品售價，減緩成本升高的影響，
+3月已通知客戶，
+透露將藉由嚴謹的定價策略，目標將全年毛利率維持在44.5%至47.5%區間。
+觀察目前整體市況依然呈現不同調的態勢，AI相關市場需求持續強勁，消費電子市場需求相對疲弱，IC設計廠不打算全面調漲產品價格。
+雅特力-KY認為，近期微控制器（MCU）市場掀起一波漲價潮，並不是終端市場強勁需求所帶動，而是AI需求強勁占用產能，以及原材料漲價所致，雅特力-KY僅會適度漲價，力求毛利率持穩。
+盛群認為，目前經濟情勢並未變好，需求僅穩定，因應晶圓代工與封測漲價10%至15%，盛群將僅調漲低毛利產品售價，期能讓毛利回歸合理。
+繼記憶體價格飆漲後，晶圓代工和IC設計紛紛調漲價格，半導體通膨趨勢成形，使得智慧手機等消費產品市場，面臨成本升高的壓力進一步加劇。廠商除將資源集中於高階產品因應，需求也開始趨緩，聯發科預估，今年手機出貨量恐減少15%。漲價對市場需求的影響，未來是否進一步擴大，備受市場關注。</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Download failed</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4e78b80beb620f39c678da1b8dd8d665db0c4dc4072aef4c8de7eb9abd8d246e</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -516,27 +532,45 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 - TechNews 科技新報</t>
+          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development - 中央社 CNA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://finance.technews.tw/2026/05/01/semiconductor-inflation-trend-takes-shape-wafer-foundries-ic-design-price-hikes/</t>
+          <t>https://www.cna.com.tw/postwrite/eng/432806</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fri, 01 May 2026 07:00:00 GMT</t>
+          <t>Thu, 07 May 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TechNews 科技新報</t>
+          <t>中央社 CNA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 | TechNews 科技新報 搜尋： 登入 註冊 登出 VIP會員 Menu Skip to content 會員專區 訂閱專區 技術分析 焦點新聞評析 拓墣觀點 TechNews Smart AI 活動專區 常見問題 半導體 晶圓 晶片 IC 設計 封裝測試 處理器 GPU 記憶體 零組件 光電科技 面板 電池 3C周邊 AI 人工智慧 Claude Apple Intelligence DeepSeek Gemini Copilot ChatGPT Perplexity Grok 財經 財報 證券 房地產 Fintech 加密貨幣 金融政策 國際貿易 國際金融 支付方案 尖端科技 奈米 衛星通訊 汽車科技 航太科技 機器人 軍事科技 材料 無人機 環境科學 醫療科技 生物科技 科技生活 科技教育 能源科技 太陽能 風力 核能 電力儲存 企業永續 科技人才 系列專題 Token 戰爭：AI 推論時代的結構性大洗牌 光速革命 2026：矽光子與 CPO 領航 AI 下半場 AI 全方位解析：看懂任務分類、硬體門檻與你的產業卡位戰 能源即算力！2026 資料中心電源保衛戰 川普重返白宮一年，全球科技規則如何改變？ AI 晶片封裝技術革命 晶片戰場的隱形冠軍：先進封裝需求背後，一場決定全球 AI 命脈的設備軍備競賽 財報快訊 企業部落格 市場動態 關於我們 內容合作單位 菁英人才招募中 廣告合作 TN Smart 半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 作者 中央社 | 發布日期 2026 年 05 月 01 日 9:59 | 分類 IC 設計 , 半導體 , 晶圓 | edit Loading... Now Translating . . . 半導體通膨趨勢成形，因應成本高漲，包括晶圓代工及 IC 設計廠紛紛調漲價格，對於智慧手機等消費產品市場影響逐步顯現，智慧手機等今年出貨量恐面臨衰退壓力。 半導體廠法人說明會陸續登場，成本壓力及產品價格策略成為法人關注的焦點。晶圓代工廠除將持續投入技術開發及擴充產能，中東緊張局勢也造成能源和物流等成本升高。 晶圓代工廠 力積電 已搶先於今年1月調漲驅動IC及感測器代工價格，3月調漲功率元件代工價格， 世界 先進跟進於4月調漲代工價格， 聯電 也於4月通知客戶，將於下半年調整價格。 不僅晶圓代工價格調漲，後段封測價格也傳出漲價消息，IC設計廠紛紛決定調漲產品售價，減緩成本升高的影響， 盛群 3月已通知客戶， 聯發科 透露將藉由嚴謹的定價策略，目標將全年毛利率維持在44.5%至47.5%區間。 觀察目前整體市況依然呈現不同調的態勢，AI相關市場需求持續強勁，消費電子市場需求相對疲弱，IC設計廠不打算全面調漲產品價格。 雅特力-KY認為，近期微控制器（MCU）市場掀起一波漲價潮，並不是終端市場強勁需求所帶動，而是AI需求強勁占用產能，以及原材料漲價所致，雅特力-KY僅會適度漲價，力求毛利率持穩。 盛群認為，目前經濟情勢並未變好，需求僅穩定，因應晶圓代工與封測漲價10%至15%，盛群將僅調漲低毛利產品售價，期能讓毛利回歸合理。 繼記憶體價格飆漲後，晶圓代工和IC設計紛紛調漲價格，半導體通膨趨勢成形，使得智慧手機等消費產品市場，面臨成本升高的壓力進一步加劇。廠商除將資源集中於高階產品因應，需求也開始趨緩，聯發科預估，今年手機出貨量恐減少15%。漲價對市場需求的影響，未來是否進一步擴大，備受市場關注。 （作者：張建中；首圖來源：shutterstock） 文章看完覺得有幫助，何不給我們一個鼓勵 請我們喝杯咖啡 想請我們喝幾杯咖啡？ 每杯咖啡 65 元 x 1 x 3 x 5 x 您的咖啡贊助將是讓我們持續走下去的動力 總金額共新臺幣 0 元 《關於請喝咖啡的 Q &amp; A》 留給我們的話 取消 確認 從這裡可透過《Google 新聞》追蹤 TechNews 科技新知，時時更新 科技新報粉絲團 加入好友 訂閱免費電子報 關鍵字: 半導體通路 , 晶圓代工 , 智慧手機 , 漲價 Post navigation ← 抓無人機不靠雷達，波蘭測試「聲學感測器」揪出隱形威脅 當「好公司」成為一種人設？拆解 B 型企業的道德溢價與認證背後的機制失靈 → 我們偵測 到您有啟用 AD Block 請您暫停使用AD Block，以支持我們持續能提供更多新聞資訊與優質的閱讀環境。 新報特企 焦點動態 系列專題 AI 推論的 Token 戰爭 小龍蝦點燃「算力即營收」新紀元！Vera Rubin 引爆台美供應鏈一次看 代理 AI 重塑晶片架構！「成本才是王道」，ASIC、CPU 與記憶體牆成新戰場 從 SaaS 到 TaaS：AI 時代為何你不是付月費，而是 Token？ VIP 全預觀 本田續約廣汽十年：從技術輸出到技術汲取的合資 2.0 模式 從馬路到水路，小米申請新能源車水下推進器專利 FEV 與微軟部署車端小語言模型，確保離線語音服務與高效運用記憶體 全球儲能產業發展趨勢：政策、法規與標準化 1.6T 世代：通訊關鍵元件洗牌與台灣廠商切入路徑 本週熱門 數學界天翻地覆，代數幾何 87 年懸案「雅可比猜想」遭 Claude 證偽 焦慮、肥胖、不婚不生，研究：人類演化無法適應現代社會 全球水域含氧量迅速流失，科學家警告「水體脫氧」恐不可逆 根本沒有 100%「美國製造」路由器，廠商群起申請豁免使 FCC 禁令漸鬆 海洋蠕蟲超硬顎部揭密，科學家首度定義全新「生體金屬」 一天喝五杯咖啡也無妨？研究揭開咖啡的護肝潛力 喝咖啡能護心？美國心臟協會揭每日黃金杯數，警告避開三大飲用地雷 是太空垃圾也是天然實驗場！SpaceX 火箭殘骸 8/5 將墜入月球表面 財訊快報 宜特6月營收月增10.5% 漢唐6月營收87.43 億元 台灣大6月營收月增5.4% 科嘉-KY6月營收月減17.3% 康控-KY6月營收月減4.3% 漢磊6月營收6.20 億元 嘉晶6月營收月增3.3% 中華電6月營收月增9.3% 中環6月營收6.39 億元 台積電6月營收月增6.2% 更多&gt;&gt; 編輯精選 [ 專欄 ] 美國與中國分居最大出口市場與進口來源國下的台灣貿易結構 [ 專欄 ] 記憶體價格上漲，難成為美國政府鬆綁中國管制的理由 [ 專題 ] 小龍蝦點燃「算力即營收」新紀元！Vera Rubin 引爆台美供應鏈一次看 [ 專題 ] 代理 AI 重塑晶片架構！「成本才是王道」，ASIC、CPU 與記憶體牆成新戰場 [ 專題 ] 從 SaaS 到 TaaS：AI 時代為何你不是付月費，而是 Token？ [ 專欄 ] 「中小微企業多元振興發展計畫」落實，對提高台灣經濟韌性有重大幫助 [ 專訪 ] AI 資料傳輸量暴增！WD 談「兩大儲存挑戰」：關鍵在分層式架構 [ 專欄 ] 鼓勵「不勞而獲」降稅政策只會擴大台灣社會失衡 FB 粉絲團 我的最愛 趕快加入最愛頁面 Facebook 成為我們的小粉絲 RSS 即時更新新知 相關連結 Facebook 功能 文章 RSS 訂閱 迴響 RSS 訂閱 © 2013-2026 TechNews Inc. All rights reserved. | 關於我們 | 使用條款 | 隱私權政策 | 著作權與授權轉載 登入裝置已達上限 親愛的會員, 您的帳戶已經在其他裝置進行登入，於是系統將自動把您的帳戶登出本裝置。 若需要繼續瀏覽網站，請 重新登入 網站 若非您本人的操作，為保障您的帳戶安全，請您儘快至會員中心 修改密碼 × 請您暫停使用AD Block，以支持我們持續能提供更多新聞資訊與優質的閱讀環境。</t>
+          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development
+發稿時間：2026/05/07 14:14:32
+(中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide.
+The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management.
+The program is designed for working professionals, engineers, and learners seeking to deepen their expertise or enter the rapidly evolving semiconductor field. Courses will be delivered online in a modular, stackable format, allowing learners to tailor their studies to their professional goals and industry needs.
+The Semiconductor Academy is a flexible, industry-aligned portfolio of Purdue University micro-credentials developed in collaboration with faculty from NYCU in Taiwan to help upskill the global semiconductor workforce.
+As one of Taiwan’s leading universities in electrical engineering, computer science, photonics, AI, and semiconductor research, NYCU has long played a central role in nurturing talent for Taiwan’s semiconductor industry and the Hsinchu Science Park ecosystem.
+Through the Semiconductor Academy, NYCU faculty will contribute academic expertise and real-world industry perspectives drawn from Taiwan’s globally influential semiconductor ecosystem, offering international learners a unique window into the technologies and manufacturing practices shaping the future of chips and AI computing.
+“Semiconductor innovation requires a deep understanding of the entire technology stack,” said Mark Lundstrom, Don and Carol Scifres Distinguished Professor of Electrical and Computer Engineering at Purdue University. “By bringing together the strengths of both Purdue and NYCU, the Semiconductor Academy provides learners with a rigorous, globally informed perspective on the technologies shaping the future of the industry.” The collaboration also reflects NYCU’s broader internationalization strategy and its commitment to strengthening global partnerships in semiconductors, AI, and emerging technologies.
+Covering topics from chip design and semiconductor materials to packaging and supply chain management, the Semiconductor Academy’s two-hour modular courses allow learners to build industry-relevant skills at their own pace.
+According to Purdue, the Semiconductor Academy is part of a broader expansion of semiconductor professional education aimed at addressing rising workforce demands across the global chip industry. Each course in the academy will feature approximately 2 hours of focused learning content and be accessible through flexible online formats. The academy will also be featured on SEMI University (SEMI U), a global digital learning platform serving semiconductor professionals and organizations worldwide.
+Topics planned for the initial course offerings include:
+。Chip Design for AI
+。Packaging, Reliability and Characterization
+。IC Design, EDA and Analog
+。Semiconductor Materials and Devices
+。Supply Chain Management and Leadership in the Semiconductor Industry
+Additional semiconductor professional education courses developed by Purdue are expected to launch in summer 2026, including transistor fundamentals, nanolithography, RF design, and data analysis for semiconductor applications. The launch ceremony for the Semiconductor Academy was held via livestream between Purdue and NYCU, underscoring the growing importance of international collaboration in building the future semiconductor workforce.
+For more NYCU News, please visit the official NYCU website.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -547,7 +581,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>d970a92d732b9934c7e2d6a264f99fc947e20ef78a234dcc7de6a81e794b3864</t>
+          <t>99c1b51e2e4344e6fd4461f48b7839df56167ecec2c97ec84fb1251345ae320e</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -560,41 +594,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development - 中央社 CNA</t>
+          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.cna.com.tw/postwrite/eng/432806</t>
+          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 07:00:00 GMT</t>
+          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>中央社 CNA</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development | 中央社訊息平台 財經訊息平台 知訊台 好生活 影像空間 客戶頻道 中文稿 英文稿 電信 簡介 投稿 投稿 中文稿 英文稿 電信 簡介 平台簡介 服務辦法 投稿流程 收款方式 供稿啓事 新聞稿寫作原則 其他服務 財經訊息平台 知訊台 歡迎公司行號投遞新聞訊息！詳洽業務行銷中心 人工服務時間為週一至週六9:30-12:00、14:00-18:30 如有週日發稿需求請於週六18:00前完成刊登程序。 了解更多 訊息來源：國立陽明交通大學 轉載網址 更多訊息 Matsu’s “Blue Tears” Inspire NYCU Breakthrough in Next-Generation Luminescent Materials NYCU Partners with Kneron to Advance Edge AI Education and Real-World Deployment NYCU and Changhua County Launch Smart Agriculture App to Help Farmers Monitor Crops with AI NYCU Team Wins Taiwan Title at Red Bull Basement, Heads to Silicon Valley for Global Finals NYCU Study Finds Belly Fat May Signal Hidden Heart Failure Risk—Even at Normal Weight 首頁 英文稿 NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development 發稿時間：2026/05/07 14:14:32 (中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide. The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management. The program is designed for working professionals, engineers, and learners seeking to deepen their expertise or enter the rapidly evolving semiconductor field. Courses will be delivered online in a modular, stackable format, allowing learners to tailor their studies to their professional goals and industry needs. The Semiconductor Academy is a flexible, industry-aligned portfolio of Purdue University micro-credentials developed in collaboration with faculty from NYCU in Taiwan to help upskill the global semiconductor workforce. As one of Taiwan’s leading universities in electrical engineering, computer science, photonics, AI, and semiconductor research, NYCU has long played a central role in nurturing talent for Taiwan’s semiconductor industry and the Hsinchu Science Park ecosystem. Through the Semiconductor Academy, NYCU faculty will contribute academic expertise and real-world industry perspectives drawn from Taiwan’s globally influential semiconductor ecosystem, offering international learners a unique window into the technologies and manufacturing practices shaping the future of chips and AI computing. “Semiconductor innovation requires a deep understanding of the entire technology stack,” said Mark Lundstrom, Don and Carol Scifres Distinguished Professor of Electrical and Computer Engineering at Purdue University. “By bringing together the strengths of both Purdue and NYCU, the Semiconductor Academy provides learners with a rigorous, globally informed perspective on the technologies shaping the future of the industry.” The collaboration also reflects NYCU’s broader internationalization strategy and its commitment to strengthening global partnerships in semiconductors, AI, and emerging technologies. Covering topics from chip design and semiconductor materials to packaging and supply chain management, the Semiconductor Academy’s two-hour modular courses allow learners to build industry-relevant skills at their own pace. According to Purdue, the Semiconductor Academy is part of a broader expansion of semiconductor professional education aimed at addressing rising workforce demands across the global chip industry. Each course in the academy will feature approximately 2 hours of focused learning content and be accessible through flexible online formats. The academy will also be featured on SEMI University (SEMI U), a global digital learning platform serving semiconductor professionals and organizations worldwide. Topics planned for the initial course offerings include: 。Chip Design for AI 。Packaging, Reliability and Characterization 。IC Design, EDA and Analog 。Semiconductor Materials and Devices 。Supply Chain Management and Leadership in the Semiconductor Industry Additional semiconductor professional education courses developed by Purdue are expected to launch in summer 2026, including transistor fundamentals, nanolithography, RF design, and data analysis for semiconductor applications. The launch ceremony for the Semiconductor Academy was held via livestream between Purdue and NYCU, underscoring the growing importance of international collaboration in building the future semiconductor workforce. 文章附檔 For more NYCU News, please visit the official NYCU website. 訊息平台 平台簡介 | 服務辦法 | 投稿流程 | 收款方式 | 供稿啟事 | 新聞稿寫作原則 | 其他服務 關於中央社 公司簡介 | 企業識別 | 公開資訊 | 設置條例摘要 | 隱私權聲明 | 聯絡我們 友善連結 曾虛白新聞獎基金會 | 公職人員及關係人補助交易身分關係公開及查詢平臺 中央社網站 中央通訊社 | Focus Taiwan | フォーカス台湾 | Fokus Taiwan 關注更多 iOS app 下載 | Android app 下載 | Focus Taiwan APP | 全球中央雜誌 | 文化+ | 淨零碳排 | 新聞學院 | 中央社電子報 產品與服務 產品總覽 | 客戶頻道 | 影像空間 | 訊息平台 | 財經訊息平台 | 知訊台 本平台資料均由投稿單位輸入後對外公布，資料如有錯誤、遺漏或虛偽不實，均由投稿單位負責 copyright © 2021 中央通訊社版權所有</t>
-        </is>
-      </c>
+          <t>科技產業資訊室</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>f4068be0c01a90821295bd0289181ff02d813688f755753fa888b3135406f94d</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Download failed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -604,37 +634,48 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
+          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 工商時報</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
+          <t>https://www.ctee.com.tw/news/20260304700096-439901</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
+          <t>Wed, 04 Mar 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>科技產業資訊室</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>工商時報</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>通寶半導體設計公司簡介
+台灣IC設計領域傳出國際策略投資合作捷報，通寶半導體（QBit Semiconductor）公司3日宣布，已完成B輪募資，並獲全球半導體架構大廠安謀公司（Arm Limited）參與投資，成為目前全台唯一獲得Arm投資的IC設計公司。
+安謀現成為通寶十大股東之一，至於安謀持股比例及金額，4月下旬召開法說會可望對外說明，未來通寶擬計畫跨足無人機及機器人市場。
+通寶半導體同時宣布，隨著募資完成營運規模擴大，計畫於今年第四季向臺灣證券交易所申請IPO上市，進一步邁向資本市場新里程碑，實際時程仍須視主管機關核准及市場狀況而定。
+通寶半導體為專攻多功能列印機及事務機系統晶片的IC設計公司，其客戶主要市場遍及美國、日本、中國跟台灣。除Arm參與投資外，據悉，通寶半導體在A輪募資時，台灣政府法人機構持有通寶半導體約6％股權，包括國發基金持股2.7％，以及台肥、工研院等公股事業合計持股比例約6％，還有智原科技等半導體產業加入，整體A輪投資人持股比例約為通寶已發行股權10％。
+對於這項注資，Arm全球執行副總裁暨商務長Will Abbey表示，透過與通寶的合作，可以結合先進影像處理、控制與安全能力，以支持列印及影像市場的創新。此類合作展現Arm更廣泛的策略，亦即推動具差異化的解決方案，從高效能系統延伸至更具成本效益的裝置，同時為各類產品建立成長基礎。
+通寶半導體創辦人暨執行長沈軾榮也表示，很榮幸成為獲得Arm唯一投資的台灣半導體設計公司，未來通寶將持續深化在印表機影像市場的布局，並拓展至更廣泛的影像相關應用領域。
+將工商時報加入Google偏好來源</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Download failed</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>aff1f2ed85b1eadb7b7db5280b1d2c6999979931eb2ac141ac79151a4983936d</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -644,27 +685,51 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 工商時報</t>
+          <t>ICTGC競賽首登矽谷 進軍CES廣邀全球IC新創鏈結臺灣半導體生態鏈 - tca.org.tw</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.ctee.com.tw/news/20260304700096-439901</t>
+          <t>https://www.tca.org.tw/news_detail.php?n=2454&amp;t=h</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 08:00:00 GMT</t>
+          <t>Fri, 02 Jan 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>工商時報</t>
+          <t>tca.org.tw</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 日報 - 工商時報 前往主要內容 會員 會員中心 登出 電子報 影音特區 讀報區 首頁 即時 開闔次選單 即時首頁 要聞 證券 金融 稅法 產業 房市 國際 兩岸 科技 生活 要聞 開闔次選單 要聞首頁 政經焦點 總經趨勢 稅務法務 綜合要聞 前瞻一周 證券 開闔次選單 證券首頁 上市櫃 陸港股市 國際股市 產業焦點 期貨 權證 亮點個股 專家看盤 台股逐洞賽 重要指數 重大訊息 財經行事曆 金融 開闔次選單 金融首頁 金融話題 外匯市場 牌告匯率 金融科技 銀行動態 保險脈動 數據觀測 金融人物 理財 開闔次選單 理財首頁 理財新訊 基金 ETF 生活消費 信用卡 退休理財 統一發票 產業 開闔次選單 產業首頁 半導體 科技動態 綜合產業 生技醫療 CEO專訪 職場達人 房市 開闔次選單 房市首頁 房市焦點 區域亮點 名家攻略 居住安全 觀點評論 市場動態 國際 開闔次選單 國際首頁 全球政經 全球市場 議題觀點 國際產業 Global Scan 全球財經周報 大宗商品行情 兩岸 開闔次選單 兩岸首頁 政情動向 兩岸焦點 大陸財經 大陸產業 China Scan 陸港市場 觀點分析 言論 開闔次選單 言論首頁 社論 總經經濟 產業脈動 國際經貿 企業管理 社會觀察 奇思妙想 作者群 樂活 開闔次選單 樂活首頁 美食饗宴 旅遊休閒 生活風格 愛車天地 養生保健 時尚消費 藝文特區 書房 開闔次選單 書房首頁 書房嚴選 名人書單 好書推薦 英文進修 雜誌精選 年度好書 專題 開闔次選單 專題首頁 上市櫃6月營收 大陸經濟新局 台灣半導體風雲 上市櫃Q1營收 生技ESG革命 新世代夯話題 財經人物專訪 商情 開闔次選單 商情首頁 智慧機械 大健康 金融理財 房市建材 科技綠能 消費時尚 產學管顧 社企公益 活動 開闔次選單 活動首頁 台南機械展 台中AI展 台灣權王 服務業大評鑑 數位金融獎 ETF論壇 中華電信論壇 多元信託 期貨與選擇權 永續校園徵影 搜尋 首頁 日報 工商時報 全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO 全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO 2026.03.04 03:00 工商時報 呂雪彗 通寶半導體 安謀 智原科技 IC設計 Arm注資 通寶半導體公司董事長暨執行長沈軾榮表示，通寶半導體為全台唯一獲Arm投資的 IC 設計公司。圖／通寶半導體提供 切換文字大小 複製文章連結 分享至臉書 以Line分享 加入Google來源 參與討論 友善列印 已將目前網頁的網址複製到您的剪貼簿！ 通寶半導體設計公司簡介 台灣IC設計領域傳出國際策略投資合作捷報，通寶半導體（QBit Semiconductor）公司3日宣布，已完成B輪募資，並獲全球半導體架構大廠安謀公司（Arm Limited）參與投資，成為目前全台唯一獲得Arm投資的IC設計公司。 安謀現成為通寶十大股東之一，至於安謀持股比例及金額，4月下旬召開法說會可望對外說明，未來通寶擬計畫跨足無人機及機器人市場。 通寶半導體同時宣布，隨著募資完成營運規模擴大，計畫於今年第四季向臺灣證券交易所申請IPO上市，進一步邁向資本市場新里程碑，實際時程仍須視主管機關核准及市場狀況而定。 通寶半導體為專攻多功能列印機及事務機系統晶片的IC設計公司，其客戶主要市場遍及美國、日本、中國跟台灣。除Arm參與投資外，據悉，通寶半導體在A輪募資時，台灣政府法人機構持有通寶半導體約6％股權，包括國發基金持股2.7％，以及台肥、工研院等公股事業合計持股比例約6％，還有智原科技等半導體產業加入，整體A輪投資人持股比例約為通寶已發行股權10％。 對於這項注資，Arm全球執行副總裁暨商務長Will Abbey表示，透過與通寶的合作，可以結合先進影像處理、控制與安全能力，以支持列印及影像市場的創新。此類合作展現Arm更廣泛的策略，亦即推動具差異化的解決方案，從高效能系統延伸至更具成本效益的裝置，同時為各類產品建立成長基礎。 通寶半導體創辦人暨執行長沈軾榮也表示，很榮幸成為獲得Arm唯一投資的台灣半導體設計公司，未來通寶將持續深化在印表機影像市場的布局，並拓展至更廣泛的影像相關應用領域。 將工商時報加入Google偏好來源 相關新聞 大盤震盪 拉回擇優布局台股ETF 美股走勢分歧 晶片股台積電ADR持續承壓 《基金》6檔國內半導體ETF夯 受益人數突破43.8萬人創新高 您可能感興趣的話題 留言討論 熱門日報新聞 more 台股聞到「洗籌碼、殺斷頭」的味道！「四貸同堂」族哀嚎 指數何時反彈名師劃重點 大摩喊記憶體供需缺口未收斂 Q3漲勢未歇 南亞科、華邦電、旺宏有戲唱 台股融資大退散 短線反彈契機已到？專家估8月有望戰季線 公股逢低撿便宜 重倉大型權值電子股 買超前十強3檔ETF卡位 竟是同一家 金管會出手 嚴管四貸同堂 專題推薦 返回頁首 網站選單開關 顏色主題切換 LOADING 熱門新聞 TOP 3 more 台股崩盤不敢買？孫慶龍股災做對一件事 52萬竟變成8千萬 未來十年最看好這2檔 台股聞到「洗籌碼、殺斷頭」的味道！「四貸同堂」族哀嚎 指數何時反彈名師劃重點 期貨最新報價7／29期交所夜盤行情 本網頁已閒置超過3分鐘。請點撃框外背景，或右側關閉按鈕(X)，即可回到網頁。 關閉 關閉廣告</t>
+          <t>ICTGC競賽首登矽谷 進軍CES廣邀全球IC新創鏈結臺灣半導體生態鏈
+IC Taiwan Grand Challenge團隊於CES 2025展中之TTA國家館介紹競賽
+國家科學及技術委員會（NSTC）指導的國際創新競賽IC Taiwan Grand Challenge（ICTGC）將與全球新創展會 InnoVEX 主辦單位—台北市電腦公會（TCA）於 CES 2026 期間共同啟動一系列國際交流活動。
+面對 AI 硬體、機器人、先進晶片與高科技創新快速演進的全球浪潮，InnoVEX 持續作為國際新創對接亞洲最先進科技產業的關鍵入口，此次 ICTGC x InnoVEX 國際推廣行動除了在CES展會亮相，之後將於 1 月 13 日在矽谷舉辦專場活動，協助更多矽谷團隊深入了解如何串連台灣在半導體與 AI 領域的世界級資源，展現台灣推動跨國合作與支持下一代關鍵技術的決心與承諾。
+ICTGC、InnoVEX將於CES 2026領銜登場 廣邀全球新創蒞臨TTA國家館
+在 CES 2026展會期間， IC Taiwan Grand Challenge（ICTGC）將攜手全球創新展會InnoVEX 將亮相於CES Eureka Park 的 Taiwan Tech Arena（TTA）國家館（Booth Venetian Expo, Hall G — 62201）。TTA 為國科會於 CES 設立的官方展區，鎖定具備研究導向與未來深科技潛力的新創團隊，每年吸引全球投資人、國際媒體與科技領袖參訪。
+ICTGC 團隊也將於 TTA Stage 深入介紹臺灣唯一具有完整輔導機制、可深入對接產業鏈之半導體新創競賽，及以獲獎新創案例分享ICTGC如何為新創提供從設計到量產的完整加速支持。
+國際觀展者亦歡迎蒞臨現場與 InnoVEX 及ICTGC 團隊交流，瞭解資源鏈結與競賽的徵件參與方式。
+ICTGC 2026 全球徵件開跑！助攻國際新創鍵結矽島
+ICTGC 現正開放全球報名，申請截止日為 2026 年 2 月 28 日。歡迎來自 AI、機器人、半導體技術、感測系統、次世代運算、深科技等領域的早期新創、學研團隊與技術開發者提交具潛力的創新應用提案。
+為協助國際新創擴大影響力、加速技術落地，入選團隊將於 2026 年 6 月 2 至 5 日在台北舉行的 COMPUTEX TAIPEI 與 InnoVEX 新創展中，獲得免費參展機會。
+作為亞洲指標性的 B2B 科技展，COMPUTEX 結合 InnoVEX 一站式的創投對接與國際媒合舞台，讓團隊有機會直接鏈結製造夥伴、半導體供應鏈、創投資源與國際買主，為布局半導體產業鏈之關鍵跳板。透過ICTGC計畫，獲獎團隊可望攜手台灣半導體生態系，共同開發具國際競爭力創新解決方案。
+報名網址：ictaiwanchallenge.org
+ICTGC首度矽谷登場　1 月 13 日攜手InnoVEX舉辦論壇深化台矽半導體與AI合作
+延續CES國際推廣動能，ICTGC將於2026年1月13日首度在矽谷Palo Alto的Startup Island TAIWAN – Silicon Valley Hub舉辦「Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies」論壇。論壇匯聚矽谷創業者、投資人與技術專家，探討如何善用台灣半導體與AI供應鏈資源，強化創新落地與國際合作，更於現場為有興趣參與深度介紹將介紹競賽徵件內容與評選重點，及成功案例分享。
+國際團隊亦可藉由參加此論壇，了解更多於台灣 COMPUTEX/InnoVEX 展出資訊，協助其掌握成功進入市場的路徑並與臺灣ICT產業生態系建立實質連結。
+此次活動論壇除了邀請四位講者Laura Swan-Silicon Catalyst Ventures 共同合夥人，Andy Lombard-Tesoro Venture Capital 管理合夥人, Janis Skriveris-Plug and Play Ventures 投資總監暨高科技負責人以及Sam Fok-femtoAI 共同創辦人暨執行長，台北市電腦公會楊櫻姿副總幹事將帶領團隊提供矽谷新創人士更多鍵結台灣的資源，共同茁壯成長。
+現場將同時進行全球直播，預計將吸引全球相關新創人士觀看。直播連結為：
+Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies
+2026 年 1 月 13 日（星期二）｜下午 5:00（PST）
+Startup Island TAIWAN – Silicon Valley Hub
+299 California Ave STE 300, Palo Alto, CA 94306 U.S.A.
+參考網址：
+「Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies」論壇
+（發佈時間：2026-01-02）</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -675,7 +740,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>07bad44a832864eb1272dcab2762e4e86697da67fbc05a5934fb00417467b485</t>
+          <t>3e2cc7646f4acb278718f9a379e3fb9ff2aef32d2c4329d4a62d582c839ad49d</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -688,27 +753,50 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ICTGC競賽首登矽谷 進軍CES廣邀全球IC新創鏈結臺灣半導體生態鏈 - tca.org.tw</t>
+          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development - 中央社 CNA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.tca.org.tw/news_detail.php?n=2454&amp;t=h</t>
+          <t>https://www.cna.com.tw/postwrite/eng/432806</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fri, 02 Jan 2026 08:00:00 GMT</t>
+          <t>Thu, 07 May 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>tca.org.tw</t>
+          <t>中央社 CNA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå ¨çICæ°åµéçµèºç£åå°é«çæ é - å°åå¸é»è ¦åæ¥­åæ¥­å ¬æ Taipei Computer Association æå¡ç»å ¥ å å ¥TCA äººææå ç«å §æå° èªè­ TCA æ¬æç°¡ä» å¤§äºç´ çµç¹æ¶æ§ çç£äº å°æ¥­è¯ç æå¡æå ç¢æ¥­æ¨å»£ å±è¦½æé· åé¡ç«¶è³½ æ°åµæ´»å è¨ç«è³æº åå¥½é£çµ æ°èä¸­å¿ ç±éæ°è äººç©æ¡è¨ª æå¡å°è¨ª æ´»åæ å ± å½±åæ«¥çª TCA Video Gallery TCA Photo Gallery ç«å §æå° × æå° éé ç±éæ°è ICTGCç«¶è³½é¦ç»ç½è°· é²è»CESå»£éå ¨çICæ°åµéçµèºç£åå°é«çæ é IC Taiwan Grand Challengeåéæ¼CES 2025å±ä¸­ä¹TTAåå®¶é¤¨ä»ç´¹ç«¶è³½ åå®¶ç§å­¸åæè¡å§å¡æï¼NSTCï¼æå°çåéåµæ°ç«¶è³½IC Taiwan Grand Challengeï¼ICTGCï¼å°èå ¨çæ°åµå±æ InnoVEX ä¸»è¾¦å®ä½âå°åå¸é»è ¦å ¬æï¼TCAï¼æ¼ CES 2026 æéå ±åååä¸ç³»ååéäº¤æµæ´»åã é¢å° AI ç¡¬é«ãæ©å¨äººãå é²æ¶çèé«ç§æåµæ°å¿«éæ¼é²çå ¨çæµªæ½®ï¼InnoVEX æçºä½çºåéæ°åµå°æ¥äºæ´²æå é²ç§æç¢æ¥­çééµå ¥å£ï¼æ­¤æ¬¡ ICTGC x InnoVEX åéæ¨å»£è¡åé¤äºå¨CESå±æäº®ç¸ï¼ä¹å¾å°æ¼ 1 æ 13 æ¥å¨ç½è°·èè¾¦å°å ´æ´»åï¼åå©æ´å¤ç½è°·åéæ·±å ¥äºè§£å¦ä½ä¸²é£å°ç£å¨åå°é«è AI é åçä¸çç´è³æºï¼å±ç¾å°ç£æ¨åè·¨ååä½èæ¯æä¸ä¸ä»£ééµæè¡çæ±ºå¿èæ¿è«¾ã ICTGCãInnoVEXå°æ¼CES 2026é éç»å ´ å»£éå ¨çæ°åµèè¨TTAåå®¶é¤¨ å¨ CES 2026å±ææéï¼ IC Taiwan Grand Challengeï¼ICTGCï¼å°ææå ¨çåµæ°å±æInnoVEX å°äº®ç¸æ¼CES Eureka Park ç Taiwan Tech Arenaï¼TTAï¼åå®¶é¤¨ï¼Booth Venetian Expo, Hall G â 62201ï¼ãTTA çºåç§ææ¼ CES è¨­ç«çå®æ¹å±åï¼éå®å ·åç ç©¶å°åèæªä¾æ·±ç§ææ½åçæ°åµåéï¼æ¯å¹´å¸å¼å ¨çæè³äººãåéåªé«èç§æé è¢åè¨ªã ICTGC åéä¹å°æ¼ TTA Stage æ·±å ¥ä»ç´¹èºç£å¯ä¸å ·æå®æ´è¼å°æ©å¶ãå¯æ·±å ¥å°æ¥ç¢æ¥­éä¹åå°é«æ°åµç«¶è³½ï¼åä»¥ç²çæ°åµæ¡ä¾åäº«ICTGCå¦ä½çºæ°åµæä¾å¾è¨­è¨å°éç¢çå®æ´å éæ¯æã åéè§å±è äº¦æ­¡è¿èè¨ç¾å ´è InnoVEX åICTGC åéäº¤æµï¼ç­è§£è³æºéçµèç«¶è³½çå¾µä»¶åèæ¹å¼ã ICTGC 2026 å ¨çå¾µä»¶éè·ï¼å©æ»åéæ°åµéµçµç½å³¶ ICTGC ç¾æ­£éæ¾å ¨çå ±åï¼ç³è«æªæ­¢æ¥çº 2026 å¹´ 2 æ 28 æ¥ãæ­¡è¿ä¾èª AIãæ©å¨äººãåå°é«æè¡ãææ¸¬ç³»çµ±ãæ¬¡ä¸ä»£éç®ãæ·±ç§æç­é åçæ©ææ°åµãå­¸ç åéèæè¡éç¼è æäº¤å ·æ½åçåµæ°æç¨ææ¡ã çºåå©åéæ°åµæ´å¤§å½±é¿åãå éæè¡è½å°ï¼å ¥é¸åéå°æ¼ 2026 å¹´ 6 æ 2 è³ 5 æ¥å¨å°åèè¡ç COMPUTEX TAIPEI è InnoVEX æ°åµå±ä¸­ï¼ç²å¾å è²»åå±æ©æã ä½çºäºæ´²ææ¨æ§ç B2B ç§æå±ï¼COMPUTEX çµå InnoVEX ä¸ç«å¼çåµæå°æ¥èåéåªåèå°ï¼è®åéææ©æç´æ¥éçµè£½é å¤¥ä¼´ãåå°é«ä¾æéãåµæè³æºèåéè²·ä¸»ï¼çºå¸å±åå°é«ç¢æ¥­éä¹ééµè·³æ¿ãééICTGCè¨ç«ï¼ç²çåéå¯æææå°ç£åå°é«çæ ç³»ï¼å ±åéç¼å ·åéç«¶ç­ååµæ°è§£æ±ºæ¹æ¡ã å ±åç¶²åï¼ictaiwanchallenge.org ICTGCé¦åº¦ç½è°·ç»å ´ã1 æ 13 æ¥ææInnoVEXèè¾¦è«å£æ·±åå°ç½åå°é«èAIåä½ å»¶çºCESåéæ¨å»£åè½ï¼ICTGCå°æ¼2026å¹´1æ13æ¥é¦åº¦å¨ç½è°·Palo AltoçStartup Island TAIWAN â Silicon Valley Hubèè¾¦ãBridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergiesãè«å£ãè«å£å¯èç½è°·åµæ¥­è ãæè³äººèæè¡å°å®¶ï¼æ¢è¨å¦ä½åç¨å°ç£åå°é«èAIä¾æéè³æºï¼å¼·ååµæ°è½å°èåéåä½ï¼æ´æ¼ç¾å ´çºæèè¶£åèæ·±åº¦ä»ç´¹å°ä»ç´¹ç«¶è³½å¾µä»¶å §å®¹èè©é¸éé»ï¼åæåæ¡ä¾åäº«ã åéåéäº¦å¯èç±åå æ­¤è«å£ï¼äºè§£æ´å¤æ¼å°ç£ COMPUTEX/InnoVEX å±åºè³è¨ï¼åå©å ¶ææ¡æåé²å ¥å¸å ´çè·¯å¾ä¸¦èèºç£ICTç¢æ¥­çæ ç³»å»ºç«å¯¦è³ªé£çµã æ­¤æ¬¡æ´»åè«å£é¤äºéè«åä½è¬è Laura Swan-Silicon Catalyst Ventures å ±ååå¤¥äººï¼Andy Lombard-Tesoro Venture Capital ç®¡çåå¤¥äºº, Janis Skriveris-Plug and Play Ventures æè³ç¸½ç£æ¨é«ç§æè² è²¬äººä»¥åSam Fok-femtoAI å ±ååµè¾¦äººæ¨å·è¡é·ï¼å°åå¸é»è ¦å ¬ææ¥æ«»å§¿å¯ç¸½å¹¹äºå°å¸¶é åéæä¾ç½è°·æ°åµäººå£«æ´å¤éµçµå°ç£çè³æºï¼å ±åèå£¯æé·ã ç¾å ´å°åæé²è¡å ¨çç´æ­ï¼é è¨å°å¸å¼å ¨çç¸éæ°åµäººå£«è§çãç´æ­é£çµçºï¼https://www.youtube.com/live/ruXS6oe7WNA æ´»åè³è¨ Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies 2026 å¹´ 1 æ 13 æ¥ï¼ææäºï¼ï½ä¸å 5:00ï¼PSTï¼ Startup Island TAIWAN â Silicon Valley Hub 299 California Ave STE 300, Palo Alto, CA 94306 U.S.A. åèç¶²åï¼ ãBridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergiesãè«å£ ï¼ç¼ä½æéï¼2026-01-02ï¼ ååè¡¨é  è½å¯ ã åå° ã åäº« å»¶ä¼¸é±è® InnoVEX 2026 ç«¶è³½ç»å ´ AVITICãPlug and PlayãPwCé¦æ³¢ç¹å¥çé½ç¼ï¼è¯æè³¦è½æ°åµéæåéçåè½é å®ç¢é³ä¿èè£äºé·æ¥ä»»çäºé· æè¨±å ±åè´åç¢æ¥­åéå äººç©æ¡è¨ª åç§æç¢å­¸èæå¾·çèé· : æ¨åç¢å­¸åä½è®ç ç¼ææè½å° æ°ä»»çç£äºæ¡è¨ªç³»åå ±å°(7)-æ¬æçäºæ¨å®ç¢æºé«é£å æ©è£äºé· : ãè³éè¨çµåçæãæ¯å°ç£æªä¾ç«¶ç­åªå¢ æ°ä»»çç£äºæ¡è¨ªç³»åå ±å°(6)-æ¬æçäºæ¨éææ©å¨äººé»è­å¿ çéé· : Edge AIæ¯å°ç£æ©å¨äººç¢æ¥­å½éè¶ è»çæ©æ ï¼ æ´å¤è¨æ¯ æå¡å°è¨ª TCAæå¡ä¼æ¥­å°è¨ª -å±¹å²ç§æï¼Eleosï¼ TCAæå¡ä¼æ¥­å°è¨ª -é²ä¸æè¾° TCAæå¡ä¼æ¥­å°è¨ª -å°ç£è³æç§æ ï¼ æ´å¤è¨æ¯ å»£å®£æå é±ç§æ¿ç­ è¯çµ¡æå äº¤éä½ç½® æå¡eåé Â© 2002ï¼2026 å°åå¸é»è ¦åæ¥­åæ¥­å ¬æ çæ¬ææ</t>
+          <t>Matsu’s “Blue Tears” Inspire NYCU Breakthrough in Next-Generation Luminescent Materials
+NYCU Partners with Kneron to Advance Edge AI Education and Real-World Deployment
+NYCU and Changhua County Launch Smart Agriculture App to Help Farmers Monitor Crops with AI
+NYCU Team Wins Taiwan Title at Red Bull Basement, Heads to Silicon Valley for Global Finals
+NYCU Study Finds Belly Fat May Signal Hidden Heart Failure Risk—Even at Normal Weight
+NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development
+發稿時間：2026/05/07 14:14:32
+(中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide.
+The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management.
+The program is designed for working professionals, engineers, and learners seeking to deepen their expertise or enter the rapidly evolving semiconductor field. Courses will be delivered online in a modular, stackable format, allowing learners to tailor their studies to their professional goals and industry needs.
+The Semiconductor Academy is a flexible, industry-aligned portfolio of Purdue University micro-credentials developed in collaboration with faculty from NYCU in Taiwan to help upskill the global semiconductor workforce.
+As one of Taiwan’s leading universities in electrical engineering, computer science, photonics, AI, and semiconductor research, NYCU has long played a central role in nurturing talent for Taiwan’s semiconductor industry and the Hsinchu Science Park ecosystem.
+Through the Semiconductor Academy, NYCU faculty will contribute academic expertise and real-world industry perspectives drawn from Taiwan’s globally influential semiconductor ecosystem, offering international learners a unique window into the technologies and manufacturing practices shaping the future of chips and AI computing.
+“Semiconductor innovation requires a deep understanding of the entire technology stack,” said Mark Lundstrom, Don and Carol Scifres Distinguished Professor of Electrical and Computer Engineering at Purdue University. “By bringing together the strengths of both Purdue and NYCU, the Semiconductor Academy provides learners with a rigorous, globally informed perspective on the technologies shaping the future of the industry.” The collaboration also reflects NYCU’s broader internationalization strategy and its commitment to strengthening global partnerships in semiconductors, AI, and emerging technologies.
+Covering topics from chip design and semiconductor materials to packaging and supply chain management, the Semiconductor Academy’s two-hour modular courses allow learners to build industry-relevant skills at their own pace.
+According to Purdue, the Semiconductor Academy is part of a broader expansion of semiconductor professional education aimed at addressing rising workforce demands across the global chip industry. Each course in the academy will feature approximately 2 hours of focused learning content and be accessible through flexible online formats. The academy will also be featured on SEMI University (SEMI U), a global digital learning platform serving semiconductor professionals and organizations worldwide.
+Topics planned for the initial course offerings include:
+。Chip Design for AI
+。Packaging, Reliability and Characterization
+。IC Design, EDA and Analog
+。Semiconductor Materials and Devices
+。Supply Chain Management and Leadership in the Semiconductor Industry
+Additional semiconductor professional education courses developed by Purdue are expected to launch in summer 2026, including transistor fundamentals, nanolithography, RF design, and data analysis for semiconductor applications. The launch ceremony for the Semiconductor Academy was held via livestream between Purdue and NYCU, underscoring the growing importance of international collaboration in building the future semiconductor workforce.
+For more NYCU News, please visit the official NYCU website.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -719,10 +807,50 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3ccc8d408c7b8b6a576a6c109f4331f3fdb5cb914a2a24b036a161f9c12492a9</t>
+          <t>18fb0777c7251bbf53690d6e918ab35a43212a286e270a47638a96b4e1d35bf9</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>科技產業資訊室</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Download failed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add logging system for AutoSearch V2.5
</commit_message>
<xml_diff>
--- a/output/result.xlsx
+++ b/output/result.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,10 +488,8 @@
           <t>https://finance.technews.tw/2026/05/01/semiconductor-inflation-trend-takes-shape-wafer-foundries-ic-design-price-hikes/</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Fri, 01 May 2026 07:00:00 GMT</t>
-        </is>
+      <c r="D2" s="1" t="n">
+        <v>46143.29166666666</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -552,7 +554,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development
+          <t>Matsu’s “Blue Tears” Inspire NYCU Breakthrough in Next-Generation Luminescent Materials
+NYCU Partners with Kneron to Advance Edge AI Education and Real-World Deployment
+NYCU and Changhua County Launch Smart Agriculture App to Help Farmers Monitor Crops with AI
+NYCU Team Wins Taiwan Title at Red Bull Basement, Heads to Silicon Valley for Global Finals
+NYCU Study Finds Belly Fat May Signal Hidden Heart Failure Risk—Even at Normal Weight
+NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development
 發稿時間：2026/05/07 14:14:32
 (中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide.
 The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management.
@@ -581,7 +588,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>99c1b51e2e4344e6fd4461f48b7839df56167ecec2c97ec84fb1251345ae320e</t>
+          <t>18fb0777c7251bbf53690d6e918ab35a43212a286e270a47638a96b4e1d35bf9</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -753,100 +760,33 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development - 中央社 CNA</t>
+          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.cna.com.tw/postwrite/eng/432806</t>
+          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 07:00:00 GMT</t>
+          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>中央社 CNA</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Matsu’s “Blue Tears” Inspire NYCU Breakthrough in Next-Generation Luminescent Materials
-NYCU Partners with Kneron to Advance Edge AI Education and Real-World Deployment
-NYCU and Changhua County Launch Smart Agriculture App to Help Farmers Monitor Crops with AI
-NYCU Team Wins Taiwan Title at Red Bull Basement, Heads to Silicon Valley for Global Finals
-NYCU Study Finds Belly Fat May Signal Hidden Heart Failure Risk—Even at Normal Weight
-NYCU and Purdue Launch Global Semiconductor Academy to Advance AI and Chip Talent Development
-發稿時間：2026/05/07 14:14:32
-(中央社訊息服務20260507 14:14:32)As the global semiconductor race accelerates in the AI era, National Yang Ming Chiao Tung University (NYCU) and Purdue University have jointly launched the Semiconductor Academy, a new online professional education initiative designed to cultivate next-generation semiconductor talent and expand access to industry-focused learning worldwide.
-The collaboration brings together two institutions located at the heart of critical semiconductor ecosystems — Taiwan, home to the world’s most advanced chip manufacturing industry, and the United States, a global leader in semiconductor research, design, and innovation. Developed jointly by NYCU and Purdue, the Semiconductor Academy will offer flexible online courses covering key areas across the semiconductor supply chain, including chip design for AI, semiconductor materials and devices, advanced packaging, reliability, IC design, EDA, and semiconductor industry management.
-The program is designed for working professionals, engineers, and learners seeking to deepen their expertise or enter the rapidly evolving semiconductor field. Courses will be delivered online in a modular, stackable format, allowing learners to tailor their studies to their professional goals and industry needs.
-The Semiconductor Academy is a flexible, industry-aligned portfolio of Purdue University micro-credentials developed in collaboration with faculty from NYCU in Taiwan to help upskill the global semiconductor workforce.
-As one of Taiwan’s leading universities in electrical engineering, computer science, photonics, AI, and semiconductor research, NYCU has long played a central role in nurturing talent for Taiwan’s semiconductor industry and the Hsinchu Science Park ecosystem.
-Through the Semiconductor Academy, NYCU faculty will contribute academic expertise and real-world industry perspectives drawn from Taiwan’s globally influential semiconductor ecosystem, offering international learners a unique window into the technologies and manufacturing practices shaping the future of chips and AI computing.
-“Semiconductor innovation requires a deep understanding of the entire technology stack,” said Mark Lundstrom, Don and Carol Scifres Distinguished Professor of Electrical and Computer Engineering at Purdue University. “By bringing together the strengths of both Purdue and NYCU, the Semiconductor Academy provides learners with a rigorous, globally informed perspective on the technologies shaping the future of the industry.” The collaboration also reflects NYCU’s broader internationalization strategy and its commitment to strengthening global partnerships in semiconductors, AI, and emerging technologies.
-Covering topics from chip design and semiconductor materials to packaging and supply chain management, the Semiconductor Academy’s two-hour modular courses allow learners to build industry-relevant skills at their own pace.
-According to Purdue, the Semiconductor Academy is part of a broader expansion of semiconductor professional education aimed at addressing rising workforce demands across the global chip industry. Each course in the academy will feature approximately 2 hours of focused learning content and be accessible through flexible online formats. The academy will also be featured on SEMI University (SEMI U), a global digital learning platform serving semiconductor professionals and organizations worldwide.
-Topics planned for the initial course offerings include:
-。Chip Design for AI
-。Packaging, Reliability and Characterization
-。IC Design, EDA and Analog
-。Semiconductor Materials and Devices
-。Supply Chain Management and Leadership in the Semiconductor Industry
-Additional semiconductor professional education courses developed by Purdue are expected to launch in summer 2026, including transistor fundamentals, nanolithography, RF design, and data analysis for semiconductor applications. The launch ceremony for the Semiconductor Academy was held via livestream between Purdue and NYCU, underscoring the growing importance of international collaboration in building the future semiconductor workforce.
-For more NYCU News, please visit the official NYCU website.</t>
-        </is>
-      </c>
+          <t>科技產業資訊室</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>18fb0777c7251bbf53690d6e918ab35a43212a286e270a47638a96b4e1d35bf9</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IC semiconductor</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>科技產業資訊室</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Download failed</t>
         </is>

</xml_diff>

<commit_message>
Complete AutoSearchV3 P4 database integration
</commit_message>
<xml_diff>
--- a/output/result.xlsx
+++ b/output/result.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,46 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>error</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ai_summary</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ai_category</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ai_keywords</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ai_importance</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ai_model</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ai_version</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>ai_analyze_time</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ai_confidence</t>
         </is>
       </c>
     </row>
@@ -525,6 +565,14 @@
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -592,6 +640,14 @@
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -632,6 +688,14 @@
           <t>Download failed</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -683,6 +747,14 @@
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -751,6 +823,14 @@
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -760,37 +840,376 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>市場報導： 2026年上半年半導體營收竟然達7千億美元，相當於2024年一整年總營收，AI太可怕了！ - 科技產業資訊室</t>
+          <t>中國 IC 設計市佔已超車台灣！IDC 揭 2026 半導體十大趨勢：地緣政治如何重塑供應鏈？ - TechOrange 科技報橘</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://iknow.stpi.niar.org.tw/Post/Read.aspx?PostID=23258</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Tue, 16 Jun 2026 02:26:21 GMT</t>
-        </is>
+          <t>https://techorange.com/2025/12/05/2026-semiconductor/</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>45996.33333333334</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>科技產業資訊室</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>TechOrange 科技報橘</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>IDC 在今（12/5）發布 2026 年全球半導體市場十大趨勢預測，預期 2026 年全球半導體市場將維持雙位數成長動能，年成長率達 11%。
+「2026 年半導體產業將從爆發性復甦邁向穩健擴張的階段，」IDC 資深研究經理曾冠瑋表示，為了滿足指數級增長的運算需求，從 IC 設計、晶圓製造到先進封裝的整體價值鏈正處於高產能利用率狀態，供應鏈上下游的緊密協作，將是確保 AI 晶片順利量產與效能突破的關鍵。
+針對 2026 年全球半導體市場，IDC 歸納十大趨勢。
+根據 IDC 預測，2028 年全球半導體市場規模將突破 1 兆美元，2030 年更將達到 1.2 兆美元。這股由 AI 驅動的投資週期，將抵銷部分總體經濟的不確定性。
+不過，市場必須留意記憶體價格上漲的趨勢，若價格持續走高，可能影響 2026 下半年的市場動能。
+曾冠瑋分析，運算類別佔據半導體市場營收比重將持續攀升，預計 2025-2026 年市佔達 60%，其中 AI 伺服器核心晶片受惠於雲端訓練與邊緣推論需求的同步爆發，預計成長 32%。
+相對地，車用（Automotive）與消費性（Consumer）市場因庫存調整與成本上升，展望較為保守。
+IDC 預估 2026 年亞太區 IC 設計市場將成長 11%，不過正面臨歷史性的結構轉變，因為中國 IC 設計產值已於 2025 年正式超越台灣，確立其市場領先地位。
+IDC 預測，2026 年中國市佔率將進一步擴大至 45%，台灣則調整至 40%，此消長態勢源自中國在美方制裁下，仍積極發展本土 AI 晶片、高階手機處理器，加上虛擬貨幣與安防晶片需求強勁，因此帶動當地營收呈現倍數級成長。
+先進製程是 2026 年晶圓代工市場成長的核心引擎，預計推動整體產值成長 20%。隨著 AI 晶片算力需求增長，台積電預期市佔率將攀升至 73%，且維持 22-26% 的高成長率。
+在資本支出方面，IDC 預估台積電將達 480 億至 500 億美元，主要用於擴充 3nm、2nm 產能及為 1.6nm 做準備。台積電 2nm 預計於 2025 年底達到月產能 8 萬片。三星與 Intel 則分別在韓國華城、美國德州及俄亥俄州積極布局，試圖在 2027-2028 年的 AI 晶片商機中搶佔一席之地。
+IDC 預估 2026 年平均產能利用率將穩定維持在 80% 以上，特別是中國晶圓廠，受惠於國產替代政策以及驅動 IC、PMIC 等訂單回流，產能利用率預期將保持在 90% 以上的高檔水位。至於台灣、韓國等非中國地區，則受惠於消費性電子復甦，利用率約維持在 80%。
+全球半導體產能版圖正走向區域多元化，美國、中國與日本的晶圓產能年複合成長率（CAGR）預計將分別達到 9.8%、9.8% 與 10% 的新高水位。
+中國面對美方先進製程設備禁令，將資源集中擴充受限較小的成熟製程，並加速扶植國產設備供應鏈，預計最快在 2028 年其「所有製程總產能」將超越台灣居全球之冠，並於 2029 年達到 37% 的全球市佔率。
+在美國方面，台積電亞利桑那州廠進展順利，一廠（P1）已開始量產，二廠（P2A）預計於 2027 年上半年正式量產 3nm 製程，P2B 則鎖定 2027 年底至 2028 年加入 2nm 行列。
+日本亦展現重返半導體強國決心，除台積電熊本廠外，日本政府也全力支持新創晶片製造商 Rapidus。雖然目前日本全球產能佔比僅約 2.5% 至 3%，但在先進製程的戰略地位將顯著提升。
+地緣政治重塑全球封測版圖，預計 2026 年 OSAT 市場將成長 11%。中國在「半導體自主化」政策推動下，要求 IC 設計與晶圓製造盡量採用在地供應鏈，推動中國 OSAT 市佔率預計將從過去的 30% 攀升至 2029 年的 33%。
+然而，高階 AI 晶片封裝仍由台灣與美國大廠掌握優勢。值得注意的是，若以包含晶圓代工廠先進封裝（Foundry-based packaging）的「封裝總市值」重新排名，受惠於 CoWoS 與 InFO 的高價值貢獻，台積電預計將在 2026 年超越傳統封測廠，成為全球封裝市值的實質龍頭。
+先進封裝產能擴張將是 2026 年的主旋律。IDC 預測，台積電 2026 年底 CoWoS 月產能將來到 11 萬片，但面對 NVIDIA、AMD 等巨頭將主力晶片全數投入 3nm 製程且 100% 採用先進封裝，市場供需依然吃緊。
+這股外溢效應將為 OSAT 廠帶來機會：日月光與矽品憑藉與台積電的長期合作，預計在 2025 年中旬開始有明顯的訂單放量；Intel 雖積極推廣封裝代工，但考量玻璃基板與高階封裝的良率需達 90% 以上才具經濟效益，預期要到 2027 年才能在 CSP 自研晶片市場中見到顯著貢獻。
+AI 加速器市場預計迎來爆發性成長。受惠於 Google TPU、AWS Trainium 等 CSP 自研晶片需求，IDC 預估 2026 年 ASIC 市場年增率將高達 173%。
+長期而言，為了優化 TCO，CSP 與模型開發商將持續擴大 ASIC 採用比例，推動 ASIC 在 2024-2029 年的年均複合成長率達到 67%。然而，GPU 並不會因此失勢，因為隨著「影像生成」的需求大增，未來的 AI 電影與即時影像運算需要極具彈性的通用算力，這將是 GPU 長期難以被取代的護城河，也讓 GPU 的年均複合成長率仍維持 56% 的高成長動能。
+針對市場擔憂的「AI 泡沫化」，IDC 認為 2026 年發生機率偏低，主因在於 AI 基礎建設並非無限制擴張，而是受到「電力供應」與「能源網架構」的物理限制。CSP 業者無法在缺乏電力配套下無限採購晶片，這種物理上的「調節閥」反而讓半導體出貨維持在相對健康、理性的成長軌道，避免了過度庫存堆積導致的瞬間崩盤。
+2026 年全球半導體產業將延續雙位數成長，從爆發期邁入「穩健擴張」階段。在這段過程中，地緣政治帶來的供應鏈重組、中國產能的強勢崛起，以及 AI 基礎建設是否會因電力瓶頸而調整節奏，將是決定產業走向的關鍵變數。</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Download failed</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2ff7ce7ea89916c1195ccf726a2cbe400b942f1532cf8c7e112d739602e99d8f</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>半導體通膨趨勢成形，晶圓代工、IC 設計紛漲價 - TechNews 科技新報</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://finance.technews.tw/2026/05/01/semiconductor-inflation-trend-takes-shape-wafer-foundries-ic-design-price-hikes/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Fri, 01 May 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TechNews 科技新報</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>半導體通膨趨勢成形，因應成本高漲，包括晶圓代工及 IC 設計廠紛紛調漲價格，對於智慧手機等消費產品市場影響逐步顯現，智慧手機等今年出貨量恐面臨衰退壓力。
+半導體廠法人說明會陸續登場，成本壓力及產品價格策略成為法人關注的焦點。晶圓代工廠除將持續投入技術開發及擴充產能，中東緊張局勢也造成能源和物流等成本升高。
+晶圓代工廠
+已搶先於今年1月調漲驅動IC及感測器代工價格，3月調漲功率元件代工價格，
+先進跟進於4月調漲代工價格，
+也於4月通知客戶，將於下半年調整價格。
+不僅晶圓代工價格調漲，後段封測價格也傳出漲價消息，IC設計廠紛紛決定調漲產品售價，減緩成本升高的影響，
+3月已通知客戶，
+透露將藉由嚴謹的定價策略，目標將全年毛利率維持在44.5%至47.5%區間。
+觀察目前整體市況依然呈現不同調的態勢，AI相關市場需求持續強勁，消費電子市場需求相對疲弱，IC設計廠不打算全面調漲產品價格。
+雅特力-KY認為，近期微控制器（MCU）市場掀起一波漲價潮，並不是終端市場強勁需求所帶動，而是AI需求強勁占用產能，以及原材料漲價所致，雅特力-KY僅會適度漲價，力求毛利率持穩。
+盛群認為，目前經濟情勢並未變好，需求僅穩定，因應晶圓代工與封測漲價10%至15%，盛群將僅調漲低毛利產品售價，期能讓毛利回歸合理。
+繼記憶體價格飆漲後，晶圓代工和IC設計紛紛調漲價格，半導體通膨趨勢成形，使得智慧手機等消費產品市場，面臨成本升高的壓力進一步加劇。廠商除將資源集中於高階產品因應，需求也開始趨緩，聯發科預估，今年手機出貨量恐減少15%。漲價對市場需求的影響，未來是否進一步擴大，備受市場關注。</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>46237.86427756945</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>c892500cb00e9052a353b06c891bd622ea32067b72b66139cc189e69c86dfbd3</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>全台首家IC設計獲Arm注資 通寶半導體Q4擬申請IPO - 工商時報</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.ctee.com.tw/news/20260304700096-439901</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>工商時報</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>通寶半導體設計公司簡介
+台灣IC設計領域傳出國際策略投資合作捷報，通寶半導體（QBit Semiconductor）公司3日宣布，已完成B輪募資，並獲全球半導體架構大廠安謀公司（Arm Limited）參與投資，成為目前全台唯一獲得Arm投資的IC設計公司。
+安謀現成為通寶十大股東之一，至於安謀持股比例及金額，4月下旬召開法說會可望對外說明，未來通寶擬計畫跨足無人機及機器人市場。
+通寶半導體同時宣布，隨著募資完成營運規模擴大，計畫於今年第四季向臺灣證券交易所申請IPO上市，進一步邁向資本市場新里程碑，實際時程仍須視主管機關核准及市場狀況而定。
+通寶半導體為專攻多功能列印機及事務機系統晶片的IC設計公司，其客戶主要市場遍及美國、日本、中國跟台灣。除Arm參與投資外，據悉，通寶半導體在A輪募資時，台灣政府法人機構持有通寶半導體約6％股權，包括國發基金持股2.7％，以及台肥、工研院等公股事業合計持股比例約6％，還有智原科技等半導體產業加入，整體A輪投資人持股比例約為通寶已發行股權10％。
+對於這項注資，Arm全球執行副總裁暨商務長Will Abbey表示，透過與通寶的合作，可以結合先進影像處理、控制與安全能力，以支持列印及影像市場的創新。此類合作展現Arm更廣泛的策略，亦即推動具差異化的解決方案，從高效能系統延伸至更具成本效益的裝置，同時為各類產品建立成長基礎。
+通寶半導體創辦人暨執行長沈軾榮也表示，很榮幸成為獲得Arm唯一投資的台灣半導體設計公司，未來通寶將持續深化在印表機影像市場的布局，並拓展至更廣泛的影像相關應用領域。
+將工商時報加入Google偏好來源</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>46237.8643865162</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ab0ba52b718011d084d7791b678dec6ea2fcabe421fbf2d21d47ffbe4c3e8366</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ICTGC競賽首登矽谷 進軍CES廣邀全球IC新創鏈結臺灣半導體生態鏈 - tca.org.tw</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.tca.org.tw/news_detail.php?n=2454&amp;t=h</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fri, 02 Jan 2026 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tca.org.tw</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ICTGC競賽首登矽谷 進軍CES廣邀全球IC新創鏈結臺灣半導體生態鏈
+IC Taiwan Grand Challenge團隊於CES 2025展中之TTA國家館介紹競賽
+國家科學及技術委員會（NSTC）指導的國際創新競賽IC Taiwan Grand Challenge（ICTGC）將與全球新創展會 InnoVEX 主辦單位—台北市電腦公會（TCA）於 CES 2026 期間共同啟動一系列國際交流活動。
+面對 AI 硬體、機器人、先進晶片與高科技創新快速演進的全球浪潮，InnoVEX 持續作為國際新創對接亞洲最先進科技產業的關鍵入口，此次 ICTGC x InnoVEX 國際推廣行動除了在CES展會亮相，之後將於 1 月 13 日在矽谷舉辦專場活動，協助更多矽谷團隊深入了解如何串連台灣在半導體與 AI 領域的世界級資源，展現台灣推動跨國合作與支持下一代關鍵技術的決心與承諾。
+ICTGC、InnoVEX將於CES 2026領銜登場 廣邀全球新創蒞臨TTA國家館
+在 CES 2026展會期間， IC Taiwan Grand Challenge（ICTGC）將攜手全球創新展會InnoVEX 將亮相於CES Eureka Park 的 Taiwan Tech Arena（TTA）國家館（Booth Venetian Expo, Hall G — 62201）。TTA 為國科會於 CES 設立的官方展區，鎖定具備研究導向與未來深科技潛力的新創團隊，每年吸引全球投資人、國際媒體與科技領袖參訪。
+ICTGC 團隊也將於 TTA Stage 深入介紹臺灣唯一具有完整輔導機制、可深入對接產業鏈之半導體新創競賽，及以獲獎新創案例分享ICTGC如何為新創提供從設計到量產的完整加速支持。
+國際觀展者亦歡迎蒞臨現場與 InnoVEX 及ICTGC 團隊交流，瞭解資源鏈結與競賽的徵件參與方式。
+ICTGC 2026 全球徵件開跑！助攻國際新創鍵結矽島
+ICTGC 現正開放全球報名，申請截止日為 2026 年 2 月 28 日。歡迎來自 AI、機器人、半導體技術、感測系統、次世代運算、深科技等領域的早期新創、學研團隊與技術開發者提交具潛力的創新應用提案。
+為協助國際新創擴大影響力、加速技術落地，入選團隊將於 2026 年 6 月 2 至 5 日在台北舉行的 COMPUTEX TAIPEI 與 InnoVEX 新創展中，獲得免費參展機會。
+作為亞洲指標性的 B2B 科技展，COMPUTEX 結合 InnoVEX 一站式的創投對接與國際媒合舞台，讓團隊有機會直接鏈結製造夥伴、半導體供應鏈、創投資源與國際買主，為布局半導體產業鏈之關鍵跳板。透過ICTGC計畫，獲獎團隊可望攜手台灣半導體生態系，共同開發具國際競爭力創新解決方案。
+報名網址：ictaiwanchallenge.org
+ICTGC首度矽谷登場　1 月 13 日攜手InnoVEX舉辦論壇深化台矽半導體與AI合作
+延續CES國際推廣動能，ICTGC將於2026年1月13日首度在矽谷Palo Alto的Startup Island TAIWAN – Silicon Valley Hub舉辦「Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies」論壇。論壇匯聚矽谷創業者、投資人與技術專家，探討如何善用台灣半導體與AI供應鏈資源，強化創新落地與國際合作，更於現場為有興趣參與深度介紹將介紹競賽徵件內容與評選重點，及成功案例分享。
+國際團隊亦可藉由參加此論壇，了解更多於台灣 COMPUTEX/InnoVEX 展出資訊，協助其掌握成功進入市場的路徑並與臺灣ICT產業生態系建立實質連結。
+此次活動論壇除了邀請四位講者Laura Swan-Silicon Catalyst Ventures 共同合夥人，Andy Lombard-Tesoro Venture Capital 管理合夥人, Janis Skriveris-Plug and Play Ventures 投資總監暨高科技負責人以及Sam Fok-femtoAI 共同創辦人暨執行長，台北市電腦公會楊櫻姿副總幹事將帶領團隊提供矽谷新創人士更多鍵結台灣的資源，共同茁壯成長。
+現場將同時進行全球直播，預計將吸引全球相關新創人士觀看。直播連結為：
+Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies
+2026 年 1 月 13 日（星期二）｜下午 5:00（PST）
+Startup Island TAIWAN – Silicon Valley Hub
+299 California Ave STE 300, Palo Alto, CA 94306 U.S.A.
+參考網址：
+「Bridging Silicon Valley and Taiwan: Semiconductor &amp; AI Synergies」論壇
+（發佈時間：2026-01-02）</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>46237.864415625</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>e4ac11cb4fcbfe85b0cee5b80deaf1b76ee2e40c21af99a317cd4a3a94cab310</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>中國 IC 設計市佔已超車台灣！IDC 揭 2026 半導體十大趨勢：地緣政治如何重塑供應鏈？ - TechOrange 科技報橘</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://techorange.com/2025/12/05/2026-semiconductor/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Fri, 05 Dec 2025 08:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TechOrange 科技報橘</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>IDC 在今（12/5）發布 2026 年全球半導體市場十大趨勢預測，預期 2026 年全球半導體市場將維持雙位數成長動能，年成長率達 11%。
+「2026 年半導體產業將從爆發性復甦邁向穩健擴張的階段，」IDC 資深研究經理曾冠瑋表示，為了滿足指數級增長的運算需求，從 IC 設計、晶圓製造到先進封裝的整體價值鏈正處於高產能利用率狀態，供應鏈上下游的緊密協作，將是確保 AI 晶片順利量產與效能突破的關鍵。
+針對 2026 年全球半導體市場，IDC 歸納十大趨勢。
+根據 IDC 預測，2028 年全球半導體市場規模將突破 1 兆美元，2030 年更將達到 1.2 兆美元。這股由 AI 驅動的投資週期，將抵銷部分總體經濟的不確定性。
+不過，市場必須留意記憶體價格上漲的趨勢，若價格持續走高，可能影響 2026 下半年的市場動能。
+曾冠瑋分析，運算類別佔據半導體市場營收比重將持續攀升，預計 2025-2026 年市佔達 60%，其中 AI 伺服器核心晶片受惠於雲端訓練與邊緣推論需求的同步爆發，預計成長 32%。
+相對地，車用（Automotive）與消費性（Consumer）市場因庫存調整與成本上升，展望較為保守。
+IDC 預估 2026 年亞太區 IC 設計市場將成長 11%，不過正面臨歷史性的結構轉變，因為中國 IC 設計產值已於 2025 年正式超越台灣，確立其市場領先地位。
+IDC 預測，2026 年中國市佔率將進一步擴大至 45%，台灣則調整至 40%，此消長態勢源自中國在美方制裁下，仍積極發展本土 AI 晶片、高階手機處理器，加上虛擬貨幣與安防晶片需求強勁，因此帶動當地營收呈現倍數級成長。
+先進製程是 2026 年晶圓代工市場成長的核心引擎，預計推動整體產值成長 20%。隨著 AI 晶片算力需求增長，台積電預期市佔率將攀升至 73%，且維持 22-26% 的高成長率。
+在資本支出方面，IDC 預估台積電將達 480 億至 500 億美元，主要用於擴充 3nm、2nm 產能及為 1.6nm 做準備。台積電 2nm 預計於 2025 年底達到月產能 8 萬片。三星與 Intel 則分別在韓國華城、美國德州及俄亥俄州積極布局，試圖在 2027-2028 年的 AI 晶片商機中搶佔一席之地。
+IDC 預估 2026 年平均產能利用率將穩定維持在 80% 以上，特別是中國晶圓廠，受惠於國產替代政策以及驅動 IC、PMIC 等訂單回流，產能利用率預期將保持在 90% 以上的高檔水位。至於台灣、韓國等非中國地區，則受惠於消費性電子復甦，利用率約維持在 80%。
+全球半導體產能版圖正走向區域多元化，美國、中國與日本的晶圓產能年複合成長率（CAGR）預計將分別達到 9.8%、9.8% 與 10% 的新高水位。
+中國面對美方先進製程設備禁令，將資源集中擴充受限較小的成熟製程，並加速扶植國產設備供應鏈，預計最快在 2028 年其「所有製程總產能」將超越台灣居全球之冠，並於 2029 年達到 37% 的全球市佔率。
+在美國方面，台積電亞利桑那州廠進展順利，一廠（P1）已開始量產，二廠（P2A）預計於 2027 年上半年正式量產 3nm 製程，P2B 則鎖定 2027 年底至 2028 年加入 2nm 行列。
+日本亦展現重返半導體強國決心，除台積電熊本廠外，日本政府也全力支持新創晶片製造商 Rapidus。雖然目前日本全球產能佔比僅約 2.5% 至 3%，但在先進製程的戰略地位將顯著提升。
+地緣政治重塑全球封測版圖，預計 2026 年 OSAT 市場將成長 11%。中國在「半導體自主化」政策推動下，要求 IC 設計與晶圓製造盡量採用在地供應鏈，推動中國 OSAT 市佔率預計將從過去的 30% 攀升至 2029 年的 33%。
+然而，高階 AI 晶片封裝仍由台灣與美國大廠掌握優勢。值得注意的是，若以包含晶圓代工廠先進封裝（Foundry-based packaging）的「封裝總市值」重新排名，受惠於 CoWoS 與 InFO 的高價值貢獻，台積電預計將在 2026 年超越傳統封測廠，成為全球封裝市值的實質龍頭。
+先進封裝產能擴張將是 2026 年的主旋律。IDC 預測，台積電 2026 年底 CoWoS 月產能將來到 11 萬片，但面對 NVIDIA、AMD 等巨頭將主力晶片全數投入 3nm 製程且 100% 採用先進封裝，市場供需依然吃緊。
+這股外溢效應將為 OSAT 廠帶來機會：日月光與矽品憑藉與台積電的長期合作，預計在 2025 年中旬開始有明顯的訂單放量；Intel 雖積極推廣封裝代工，但考量玻璃基板與高階封裝的良率需達 90% 以上才具經濟效益，預期要到 2027 年才能在 CSP 自研晶片市場中見到顯著貢獻。
+AI 加速器市場預計迎來爆發性成長。受惠於 Google TPU、AWS Trainium 等 CSP 自研晶片需求，IDC 預估 2026 年 ASIC 市場年增率將高達 173%。
+長期而言，為了優化 TCO，CSP 與模型開發商將持續擴大 ASIC 採用比例，推動 ASIC 在 2024-2029 年的年均複合成長率達到 67%。然而，GPU 並不會因此失勢，因為隨著「影像生成」的需求大增，未來的 AI 電影與即時影像運算需要極具彈性的通用算力，這將是 GPU 長期難以被取代的護城河，也讓 GPU 的年均複合成長率仍維持 56% 的高成長動能。
+針對市場擔憂的「AI 泡沫化」，IDC 認為 2026 年發生機率偏低，主因在於 AI 基礎建設並非無限制擴張，而是受到「電力供應」與「能源網架構」的物理限制。CSP 業者無法在缺乏電力配套下無限採購晶片，這種物理上的「調節閥」反而讓半導體出貨維持在相對健康、理性的成長軌道，避免了過度庫存堆積導致的瞬間崩盤。
+2026 年全球半導體產業將延續雙位數成長，從爆發期邁入「穩健擴張」階段。在這段過程中，地緣政治帶來的供應鏈重組、中國產能的強勢崛起，以及 AI 基礎建設是否會因電力瓶頸而調整節奏，將是決定產業走向的關鍵變數。</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>46237.86443957176</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>c2c888cdc2d8914d55b2a9bb7e967671464e5d36db98adfd86fd9fe4d8cf4879</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: complete AutoSearch V4 P4 data sources
</commit_message>
<xml_diff>
--- a/output/result.xlsx
+++ b/output/result.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U57"/>
+  <dimension ref="A1:U62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5795,6 +5795,434 @@
       <c r="T57" t="inlineStr"/>
       <c r="U57" t="inlineStr"/>
     </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>66</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>df3f5e636daa45107d35475009ed5e4fbffe1503d52eb91981ee34c59ca4a6a4</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>【2026最新】半導體業平均薪資出爐！日月光投控628萬奪冠、台積電破400萬 - 104職場力</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://blog.104.com.tw/top-10-semiconductor-industry-salary-2025/</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>104職場力</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Wed, 03 Jun 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" s="1" t="n">
+        <v>46252.80205401662</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O58" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>67</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>a0e5c4996be3fa353c6c653650971b467627207c9509a31d4e70eb5429f914ec</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2026/08/11 Sony Semiconductor Solutions and TSMC Agreed to Establish Joint Venture for Next-Generation Image Sensors</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://pr.tsmc.com/english/news/3333</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Sony Semiconductor Solutions and TSMC Agreed to Establish Joint Venture for Next-Generation Image Sensors
+Issued by: TSMC
+Issued on:
+2026/08/11
+HSINCHU, Taiwan, R.O.C. and ATSUGI, Japan, August 11, 2026 -
+Sony Semiconductor Solutions Corporation (“Sony”) and Taiwan Semiconductor Manufacturing Company Limited (“TSMC”) (TWSE: 2330, NYSE: TSM) today announced the execution of a legally binding definitive agreement for the establishment of Advanced Vision Semiconductor Manufacturing Corporation as a joint venture (“JV”) in Koshi City, Kumamoto Prefecture, Japan. The JV will serve as a core hub for the development and manufacturing activities required for the volume production of image sensors for smartphones utilizing advanced manufacturing process technology. The JV is expected to commence volume production in 2029.
+Sony will be the sole controlling shareholder and the JV is planned to operate as a consolidated subsidiary of Sony Group Corporation. The Representative Director of the JV is planned to be appointed by Sony.
+Pursuant to the definitive agreement, Sony plans to contribute approximately 465 billion yen to the JV through a combination of cash contributions and the transfer of its assets* through a company split. TSMC plans to make cash contributions of approximately 282 billion yen. These capital contributions are expected to be made in phases based on market demand and other relevant business conditions. In addition to these capital contributions by Sony and TSMC, investments required to realize the production capacity planned by the JV are being considered on the premise that they would receive support from the Japanese government.
+Under the strategic partnership, Sony intends to take a leading role in the development of core image sensor technologies, as well as product planning and product design. The JV plans to leverage TSMC’s advanced process technology and manufacturing expertise to drive development and manufacturing activities required for the volume production. Through this collaboration, the companies intend to accelerate the commercialization of image sensor products driven by customer needs while advancing technological innovation and strengthening manufacturing capacity.
+The establishment of the JV and completion of the transaction are subject to the receipt of required regulatory approvals and the satisfaction of other customary closing conditions.
+All other aspects of the partnership remain unchanged from the announcement by Sony and TSMC titled “Sony Semiconductor Solutions and TSMC Enter Preliminary Agreement for Next-Generation Image Sensor Strategic Partnership” issued on May 8, 2026.
+* Sony’s newly constructed fab in Koshi City, Kumamoto Prefecture, Japan, in which Sony has already invested.
+TSMC Spokesperson
+Wendell Huang
+Senior Vice President &amp; Chief Financial Officer
+TSMC Deputy Spokesperson
+Nina Kao
+Public Relations Division
+TSMC Media Contact</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="n">
+        <v>46252.80282093724</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="n">
+        <v>0</v>
+      </c>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>68</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>33a6723168a7b53184d89698b6359e00ea6cdcda94022f36fa13b7fd632bee65</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2026/05/15 TSMC to Sell 8.1% of Vanguard International Semiconductor</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://pr.tsmc.com/english/news/3314</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TSMC to Sell 8.1% of Vanguard International Semiconductor
+Issued by: TSMC
+Issued on:
+2026/05/15
+HSINCHU, Taiwan, R.O.C., May 15, 2026 –
+TSMC (TWSE: 2330, NYSE: TSM) plans to execute the sale of up to 152.0 million common shares of Vanguard International Semiconductor Corporation (“VIS”), or approximately 8.1% of VIS’ fully-diluted paid-in-capital through a block trade to financial institutional investors.
+The proposed share sale will not affect TSMC’s strategic relations with VIS, including outsourcing of interposer production and licensing of GaN technology to VIS. The proposed share sale is part of TSMC’s plan to focus its resources on core business activities. In June 2024, TSMC ceased to have representation on VIS’ board of directors.
+TSMC currently holds approximately 27.1% of VIS shares on a fully diluted basis. Upon the completion of this share sale, TSMC expects to reduce its shareholding in VIS to approximately 19%. TSMC has no plan to sell more VIS shares in the foreseeable future.
+TSMC Spokesperson
+Wendell Huang
+Senior Vice President &amp; Chief Financial Officer
+TSMC Deputy Spokesperson
+Nina Kao
+Public Relations Division
+TSMC Media Contact</t>
+        </is>
+      </c>
+      <c r="I60" s="1" t="n">
+        <v>46252.80286494823</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="n">
+        <v>0</v>
+      </c>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>69</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>80bb08a00be68949140e3b543787a768fc20fed0be49f04b3b3a8eb00e31c914</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2026/05/08 Sony Semiconductor Solutions and TSMC Enter Preliminary Agreement for Next-Generation Image Sensor Strategic Partnership</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://pr.tsmc.com/english/news/3308</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Sony Semiconductor Solutions and TSMC Enter Preliminary Agreement for Next-Generation Image Sensor Strategic Partnership
+Issued by: Sony Semiconductor Solutions Corporation and TSMC
+Issued on:
+2026/05/08
+Hsinchu, Taiwan, R.O.C., May 8, 2026 -
+Sony Semiconductor Solutions Corporation (“Sony”) and TSMC (TWSE: 2330, NYSE: TSM) today announced the signing of a non-binding memorandum of understanding (“MOU”) to form a strategic partnership for the development and manufacturing of next-generation image sensors.
+Under the proposed partnership, Sony and TSMC intend to establish a joint venture (“JV”), with Sony being the majority and controlling shareholder, to set up development and production lines in Sony’s newly constructed fab in Koshi City, Kumamoto Prefecture. Through the JV, both companies expect to leverage Sony's expertise in sensor design alongside TSMC’s strengths in process technology and manufacturing excellence as part of a broader collaboration aimed at enhancing image sensor performance.
+With the MOU signed, Sony and TSMC are discussing potential investments by the JV. These investments, along with new capital investment by Sony in its existing plant in Nagasaki, are being considered on the premise that they would be implemented in phases based on market demand, and that they would receive support from the Japanese government.
+This partnership also seeks to explore and address emerging opportunities in physical AI applications, such as automotive and robotics, paving the way for future innovations and expanded technological advancements. The establishment of the JV remains subject to the execution of a definitive legally binding agreement regarding the partnership and the satisfaction of customary closing conditions.
+“Building on the trust cultivated through our long-standing collaboration with TSMC, I am delighted that we have reached an agreement to advance our partnership to a new stage,” said Shinji Sashida, President and CEO of Sony Semiconductor Solutions Corporation. “This JV is a significant initiative that brings together the strengths of both companies and aims to drive further advancement in technology and business within the next-generation image sensor field. Building on this JV, Sony intends to further strengthen its business operations with a focus on creating high added value. Rooted in the Sony Spirit that has guided us since our founding, we intend to continue to take on the challenge of creating new markets through unprecedented ideas and distinctive technologies.”
+“Sony has been our long-time partner in the CMOS image sensor business. We are excited to elevate our collaboration to the next level, which represents a key step forward in driving future sensing technology in the AI era,” said TSMC Senior Vice President and Deputy Co-COO, Dr. Kevin Zhang. “This partnership underscores our shared commitment and mutual vision of leveraging cutting-edge technologies and innovative solutions to deliver leading sensing technology and products. We look forward to working closely together to achieve impactful results and create lasting value for all stakeholders.”
+TSMC Spokesperson
+Wendell Huang
+Senior Vice President &amp; Chief Financial Officer
+TSMC Deputy Spokesperson
+Nina Kao
+Public Relations Division
+TSMC Media Contact</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="n">
+        <v>46252.80290519664</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="n">
+        <v>0</v>
+      </c>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>70</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>fc0c6a277e289c6215faee30099dbc75fc8b6fc7aafc2efee48020b4189e8c37</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>IC semiconductor</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2026/04/23 TSMC Debuts A13 Technology at 2026 North America Technology Symposium</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://pr.tsmc.com/english/news/3302</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TSMC Debuts A13 Technology at 2026 North America Technology Symposium
+Newest Node Pushes Density Scaling and Energy Efficiency to New Heights to Address Industry’s Most Demanding Applications
+Issued by: TSMC
+Issued on:
+2026/04/23
+SANTA CLARA, CA, Apr. 22, 2026 --
+TSMC (TWSE: 2330, NYSE: TSM) today debuted its latest innovation in its most advanced process technology at the Company’s 2026 North America Technology Symposium. TSMC’s new A13 process is a direct shrink of its industry-leading A14 node announced in 2025, enabling even more compact and efficient designs to address insatiable customer demand in computational requirements for next-generation artificial intelligence, high performance computing (HPC), and mobile applications.
+Representing TSMC’s commitment to continuous improvement, A13 provides 6% area savings from A14. Design rules are fully backward compatible with A14, enabling customers to quickly migrate their designs to TSMC’s latest nanosheet transistor technology. In addition, A13 delivers increased power efficiency and performance gains through design-technology co-optimization, and is scheduled to enter production in 2029, one year after A14.
+A13 was one of many technology innovations highlighted at TSMC’s North America Technology Symposium in Santa Clara, California, which kicks off the event series around the world in the coming months. With the theme of “Expanding AI with Leadership Silicon,” the technology symposiums are TSMC’s largest annual customer events, showcasing the Company’s breakthroughs in technology development and manufacturing service.
+“At TSMC, we understand our customers are always looking ahead to their next innovation and they come to us for a reliable stream of new silicon technologies, like A13, meticulously engineered to be ready for high-volume production right when their visionary new designs demand them,” said TSMC Chairman and CEO Dr. C.C. Wei. “TSMC’s advanced process technologies lead the industry in density, performance and power efficiency, and we continually strive to make them even better for our customers’ future products, ensuring customers’ success as their most reliable technological partner."
+Other new technologies unveiled at the North America Technology Symposium include:
+Advanced Logic
+At the event, TSMC is also previewing its A14 platform enhancement
+, which features Super Power Rail technology to provide backside power delivery for AI and HPC applications. A12 is also scheduled to enter production in 2029.
+TSMC continues to advance its 2nm platform with the introduction of
+, which employs design-technology co-optimization to reach speed gains of 3-4% or power reduction of 8-10% and a 1.02-1.03X logic density improvement from N2P. A balanced option for AI, HPC, and mobile applications leveraging the process maturity and strong yield performance of the 2nm technology platform, N2U is scheduled for production in 2028.
+TSMC 3DFabric
+Advanced Packaging and 3D Silicon Stacking
+To support AI demand for more computing power and memory in a single package, TSMC continues to expand its Chip on Wafer on Substrate (CoWoS
+) technology to integrate more silicon. The Company is now producing 5.5-reticle size CoWoS and planning for even larger versions. A
+14-reticle size CoWoS
+, capable of integrating approximately 10 large compute dies and 20 HBM stacks, is slated for production in 2028. This will be followed by an expansion to beyond 14 reticles in 2029. These new offerings provide customers with more options for AI compute scaling and complement TSMC’s 40-reticle size SoW-X System-on-Wafer technology also expected in 2029.
+TSMC is also offering its TSMC-SoIC
+3D chip stacking technology on its most advanced technology platform, with
+A14-to-A14 SoIC
+set to be available for production in 2029. It will provide 1.8X higher die-to-die I/O density compared with N2-on-N2 SoIC, supporting higher bandwidth of data transfer between stacked chips.
+TSMC’s Compact Universal Photonic Engine (TSMC-COUPE™) is set to reach a key milestone with a true co-packaged optics solution using
+COUPE on substrate
+beginning production in 2026. By integrating the COUPE optical engine directly inside the package, TSMC achieves 2X power efficiency and 10X latency reduction versus a pluggable version on the circuit board. The technology is featured in a 200Gbps micro-ring modulator, a highly compact and energy-efficient solution to move data between racks in data centers.
+Automotive and Robotics
+Advanced Driver Assistance Systems (ADAS) and autonomous vehicles require leading-edge technologies along with stringent quality and reliability standards. Physical AI applications, such as humanoid robots, are adopting similarly demanding requirements. To address these needs, TSMC announced
+, the first automotive-grade process technology with nanosheet transistors. N2A provides 15-20% speed gain at the same power compared with N3A and is scheduled to complete AEC-Q100 qualification in 2028. Furthermore, TSMC is making “Auto-Use” design kits available within its N2P process design kit (PDK), enabling customers to factor in automotive usage conditions in the design. This allows customers an earlier design start before N2A process is fully qualified.
+TSMC’s efforts to speed up automotive product cycles are already paying off for customers as
+enters production in 2026. With the N3 “Auto Early” program, customers were able to start designs in 2023, and today more than 10 products are planned on N3A technology to make automobiles smarter, greener, and safer for consumers.
+Specialty Technology
+TSMC is the first to bring high voltage technology into the FinFET era in 2026 with its
+N16HV
+process aimed at display driver applications. For smartphone display drivers, N16HV will increase gate density by 41% and reduce power by 35% compared to TSMC’s N28HV process. For near-eye displays, N16HV can shrink die area by 40% and reduce power by over 20%, enhancing the usability of applications such as smart glasses.
+TSMC Spokesperson
+Wendell Huang
+Senior Vice President &amp; Chief Financial Officer
+TSMC Deputy Spokesperson
+Nina Kao
+Public Relations Division
+TSMC Media Contact</t>
+        </is>
+      </c>
+      <c r="I62" s="1" t="n">
+        <v>46252.80295300022</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="n">
+        <v>0</v>
+      </c>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>